<commit_message>
final update: all titles 180-195 chars with max SEO keywords
</commit_message>
<xml_diff>
--- a/KEIKI_Boneless_新标题.xlsx
+++ b/KEIKI_Boneless_新标题.xlsx
@@ -486,7 +486,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Light Camel</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Light...</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Green</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Green</t>
         </is>
       </c>
     </row>
@@ -554,7 +554,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating White</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Black</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Black</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Pink</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Pink</t>
         </is>
       </c>
     </row>
@@ -656,7 +656,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Black Green</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Black Green</t>
         </is>
       </c>
     </row>
@@ -690,7 +690,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Green Pink</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Green Pink</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating White Green</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White Green</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Black Green</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Black Green</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Pink Black</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Pink Black</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating White Black</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White Black</t>
         </is>
       </c>
     </row>
@@ -860,7 +860,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Pink Green</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Pink Green</t>
         </is>
       </c>
     </row>
@@ -894,7 +894,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Pink Black</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Pink Black</t>
         </is>
       </c>
     </row>
@@ -928,7 +928,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Pink White</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Pink White</t>
         </is>
       </c>
     </row>
@@ -962,7 +962,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating White Green</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White Green</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Black White</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Black White</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Pink White</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Pink White</t>
         </is>
       </c>
     </row>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Brown</t>
+          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1104,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Brown</t>
+          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Brown</t>
+          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Brown</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Brown</t>
         </is>
       </c>
     </row>
@@ -1215,7 +1215,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Brown</t>
+          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1252,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Brown</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Brown</t>
         </is>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Brown</t>
+          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Brown</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Brown</t>
         </is>
       </c>
     </row>
@@ -1363,7 +1363,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Light Camel</t>
+          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
         </is>
       </c>
     </row>
@@ -1400,7 +1400,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Light Camel</t>
+          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Light Camel</t>
+          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
         </is>
       </c>
     </row>
@@ -1474,7 +1474,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Light Camel</t>
+          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Light Camel</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Light...</t>
         </is>
       </c>
     </row>
@@ -1548,7 +1548,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Light Camel</t>
+          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Light Camel</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Light...</t>
         </is>
       </c>
     </row>
@@ -1622,7 +1622,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Green</t>
+          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
         </is>
       </c>
     </row>
@@ -1659,7 +1659,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Green</t>
+          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
         </is>
       </c>
     </row>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Green</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Green</t>
         </is>
       </c>
     </row>
@@ -1733,7 +1733,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Green</t>
+          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
         </is>
       </c>
     </row>
@@ -1770,7 +1770,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Green</t>
+          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1807,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Green</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Green</t>
         </is>
       </c>
     </row>
@@ -1844,7 +1844,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Green</t>
+          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Green</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Green</t>
         </is>
       </c>
     </row>
@@ -1918,7 +1918,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Red</t>
+          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Red</t>
         </is>
       </c>
     </row>
@@ -1955,7 +1955,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Red</t>
+          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Red</t>
         </is>
       </c>
     </row>
@@ -1992,7 +1992,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Red</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Red</t>
         </is>
       </c>
     </row>
@@ -2029,7 +2029,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Red</t>
+          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Red</t>
         </is>
       </c>
     </row>
@@ -2066,7 +2066,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Red</t>
+          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Red</t>
         </is>
       </c>
     </row>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Red</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Red</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Red</t>
+          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Red</t>
         </is>
       </c>
     </row>
@@ -2177,7 +2177,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Red</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Red</t>
         </is>
       </c>
     </row>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Green</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supporti...</t>
         </is>
       </c>
     </row>
@@ -2257,7 +2257,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Light Camel</t>
+          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Light Camel</t>
         </is>
       </c>
     </row>
@@ -2297,7 +2297,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Black</t>
+          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
         </is>
       </c>
     </row>
@@ -2337,7 +2337,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Black</t>
+          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
         </is>
       </c>
     </row>
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Black</t>
+          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
         </is>
       </c>
     </row>
@@ -2417,7 +2417,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Black</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supporti...</t>
         </is>
       </c>
     </row>
@@ -2457,7 +2457,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Black</t>
+          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
         </is>
       </c>
     </row>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Black</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supporti...</t>
         </is>
       </c>
     </row>
@@ -2537,7 +2537,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Black</t>
+          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
         </is>
       </c>
     </row>
@@ -2577,7 +2577,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Black</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supporti...</t>
         </is>
       </c>
     </row>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Green</t>
+          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
         </is>
       </c>
     </row>
@@ -2657,7 +2657,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Green</t>
+          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
         </is>
       </c>
     </row>
@@ -2697,7 +2697,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Green</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supporti...</t>
         </is>
       </c>
     </row>
@@ -2737,7 +2737,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Green</t>
+          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
         </is>
       </c>
     </row>
@@ -2777,7 +2777,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Green</t>
+          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
         </is>
       </c>
     </row>
@@ -2817,7 +2817,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Green</t>
+          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
         </is>
       </c>
     </row>
@@ -2857,7 +2857,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Green</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supporti...</t>
         </is>
       </c>
     </row>
@@ -2897,7 +2897,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Cream</t>
+          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
         </is>
       </c>
     </row>
@@ -2937,7 +2937,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Cream</t>
+          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
         </is>
       </c>
     </row>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Cream</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supporti...</t>
         </is>
       </c>
     </row>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Cream</t>
+          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
         </is>
       </c>
     </row>
@@ -3057,7 +3057,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Cream</t>
+          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
         </is>
       </c>
     </row>
@@ -3097,7 +3097,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Cream</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supporti...</t>
         </is>
       </c>
     </row>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Cream</t>
+          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
         </is>
       </c>
     </row>
@@ -3177,7 +3177,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Cream</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supporti...</t>
         </is>
       </c>
     </row>
@@ -3217,7 +3217,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Light Camel</t>
+          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Light Camel</t>
         </is>
       </c>
     </row>
@@ -3257,7 +3257,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Light Camel</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supporti...</t>
         </is>
       </c>
     </row>
@@ -3297,7 +3297,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Light Camel</t>
+          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Light Camel</t>
         </is>
       </c>
     </row>
@@ -3337,7 +3337,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Light Camel</t>
+          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Light Camel</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Light Camel</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supporti...</t>
         </is>
       </c>
     </row>
@@ -3417,7 +3417,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Light Camel</t>
+          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Light Camel</t>
         </is>
       </c>
     </row>
@@ -3457,7 +3457,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Light Camel</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supporti...</t>
         </is>
       </c>
     </row>
@@ -3495,7 +3495,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 77.2" Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Black</t>
+          <t>KEIKI Full Chaise 77.2" Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive B...</t>
         </is>
       </c>
     </row>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 135" Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Black</t>
+          <t>KEIKI Full Chaise 135" Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Black</t>
         </is>
       </c>
     </row>
@@ -3571,7 +3571,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise 106" Modular Boneless Velvet Sofa Couch for Living Room Comfy Lounge Seating Black</t>
+          <t>KEIKI Left Chaise 106" Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Black</t>
         </is>
       </c>
     </row>
@@ -3609,7 +3609,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise 106" Modular Boneless Velvet Sofa Couch for Living Room Comfy Lounge Seating Black</t>
+          <t>KEIKI Right Chaise 106" Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive B...</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3647,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 77.2" Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Green</t>
+          <t>KEIKI Full Chaise 77.2" Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive G...</t>
         </is>
       </c>
     </row>
@@ -3685,7 +3685,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 135" Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Green</t>
+          <t>KEIKI Full Chaise 135" Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Green</t>
         </is>
       </c>
     </row>
@@ -3723,7 +3723,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise 106" Modular Boneless Velvet Sofa Couch for Living Room Comfy Lounge Seating Green</t>
+          <t>KEIKI Left Chaise 106" Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Green</t>
         </is>
       </c>
     </row>
@@ -3761,7 +3761,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise 106" Modular Boneless Velvet Sofa Couch for Living Room Comfy Lounge Seating Green</t>
+          <t>KEIKI Right Chaise 106" Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive G...</t>
         </is>
       </c>
     </row>
@@ -3799,7 +3799,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 77.2" Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Camel</t>
+          <t>KEIKI Full Chaise 77.2" Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive C...</t>
         </is>
       </c>
     </row>
@@ -3837,7 +3837,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 135" Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Camel</t>
+          <t>KEIKI Full Chaise 135" Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Camel</t>
         </is>
       </c>
     </row>
@@ -3875,7 +3875,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise 106" Modular Boneless Velvet Sofa Couch for Living Room Comfy Lounge Seating Camel</t>
+          <t>KEIKI Left Chaise 106" Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Camel</t>
         </is>
       </c>
     </row>
@@ -3913,7 +3913,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise 106" Modular Boneless Velvet Sofa Couch for Living Room Comfy Lounge Seating Camel</t>
+          <t>KEIKI Right Chaise 106" Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive C...</t>
         </is>
       </c>
     </row>
@@ -3951,7 +3951,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 77.2" Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating White</t>
+          <t>KEIKI Full Chaise 77.2" Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive W...</t>
         </is>
       </c>
     </row>
@@ -3989,7 +3989,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 135" Modular Boneless Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating White</t>
+          <t>KEIKI Full Chaise 135" Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White</t>
         </is>
       </c>
     </row>
@@ -4027,7 +4027,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise 106" Modular Boneless Velvet Sofa Couch for Living Room Comfy Lounge Seating White</t>
+          <t>KEIKI Left Chaise 106" Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White</t>
         </is>
       </c>
     </row>
@@ -4065,7 +4065,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise 106" Modular Boneless Velvet Sofa Couch for Living Room Comfy Lounge Seating White</t>
+          <t>KEIKI Right Chaise 106" Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive W...</t>
         </is>
       </c>
     </row>
@@ -4099,7 +4099,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>KEIKI Velvet Sofa Couch for Living Room Comfy Lounge Seating Black</t>
+          <t>KEIKI Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spacious Inviting Warm Spaciou...</t>
         </is>
       </c>
     </row>
@@ -4133,7 +4133,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>KEIKI Velvet Sofa Couch for Living Room Comfy Lounge Seating Gray</t>
+          <t>KEIKI Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spacious Inviting Warm Spaciou...</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>KEIKI Velvet Sofa Couch for Living Room Comfy Lounge Seating Beige</t>
+          <t>KEIKI Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spacious Inviting Warm Spaciou...</t>
         </is>
       </c>
     </row>
@@ -4204,7 +4204,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Camel</t>
+          <t>KEIKI Left Chaise Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Camel</t>
         </is>
       </c>
     </row>
@@ -4241,7 +4241,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Green</t>
+          <t>KEIKI Left Chaise Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Green</t>
         </is>
       </c>
     </row>
@@ -4278,7 +4278,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating White</t>
+          <t>KEIKI Left Chaise Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White</t>
         </is>
       </c>
     </row>
@@ -4315,7 +4315,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Black</t>
+          <t>KEIKI Left Chaise Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Black</t>
         </is>
       </c>
     </row>
@@ -4352,7 +4352,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Camel</t>
+          <t>KEIKI Right Chaise Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Camel</t>
         </is>
       </c>
     </row>
@@ -4389,7 +4389,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Green</t>
+          <t>KEIKI Right Chaise Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Green</t>
         </is>
       </c>
     </row>
@@ -4426,7 +4426,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating White</t>
+          <t>KEIKI Right Chaise Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White</t>
         </is>
       </c>
     </row>
@@ -4463,7 +4463,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Black</t>
+          <t>KEIKI Right Chaise Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Black</t>
         </is>
       </c>
     </row>
@@ -4500,7 +4500,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Turtle Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Green</t>
+          <t>KEIKI Left Chaise Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Green</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4537,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Turtle Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Green</t>
+          <t>KEIKI Right Chaise Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Green</t>
         </is>
       </c>
     </row>
@@ -4574,7 +4574,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Turtle Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating White</t>
+          <t>KEIKI Left Chaise Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White</t>
         </is>
       </c>
     </row>
@@ -4611,7 +4611,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Turtle Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating White</t>
+          <t>KEIKI Right Chaise Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White</t>
         </is>
       </c>
     </row>
@@ -4648,7 +4648,7 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Turtle Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Black</t>
+          <t>KEIKI Left Chaise Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Black</t>
         </is>
       </c>
     </row>
@@ -4685,7 +4685,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Turtle Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Black</t>
+          <t>KEIKI Right Chaise Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Black</t>
         </is>
       </c>
     </row>
@@ -4722,7 +4722,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Turtle Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Pink</t>
+          <t>KEIKI Left Chaise Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Pink</t>
         </is>
       </c>
     </row>
@@ -4759,7 +4759,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Turtle Velvet Sofa Couch for Living Room Flexible Layout Comfy Lounge Seating Pink</t>
+          <t>KEIKI Right Chaise Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Pink</t>
         </is>
       </c>
     </row>
@@ -4815,7 +4815,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat Modular Boneless Velvet Sofa Couch for Living Room Comfy Lounge Seating Light Grey</t>
+          <t>KEIKI Loveseat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Light Grey</t>
         </is>
       </c>
     </row>
@@ -4871,7 +4871,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat Modular Boneless Velvet Sofa Couch for Living Room Comfy Lounge Seating Dark Grey</t>
+          <t>KEIKI Loveseat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Dark Grey</t>
         </is>
       </c>
     </row>
@@ -4927,7 +4927,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat Modular Boneless Velvet Sofa Couch for Living Room Comfy Lounge Seating Orange</t>
+          <t>KEIKI Loveseat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Orange</t>
         </is>
       </c>
     </row>
@@ -4983,7 +4983,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat Modular Boneless Velvet Sofa Couch for Living Room Comfy Lounge Seating White</t>
+          <t>KEIKI Loveseat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White</t>
         </is>
       </c>
     </row>
@@ -5027,7 +5027,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>KEIKI 2 seat Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Dark Grey</t>
+          <t>KEIKI 2 seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Dark Grey</t>
         </is>
       </c>
     </row>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>KEIKI 2 seat Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Light Grey</t>
+          <t>KEIKI 2 seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Light Grey</t>
         </is>
       </c>
     </row>
@@ -5115,7 +5115,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>KEIKI 2 seat Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating White</t>
+          <t>KEIKI 2 seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
         </is>
       </c>
     </row>
@@ -5159,7 +5159,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>KEIKI 2 seat Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Orange</t>
+          <t>KEIKI 2 seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
         </is>
       </c>
     </row>
@@ -5203,7 +5203,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>KEIKI 1 seater and 1 Ottoman Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Dark Grey</t>
+          <t>KEIKI 1 seater and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Dark ...</t>
         </is>
       </c>
     </row>
@@ -5247,7 +5247,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>KEIKI 1 seater and 1 Ottoman Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Light Grey</t>
+          <t>KEIKI 1 seater and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Light...</t>
         </is>
       </c>
     </row>
@@ -5291,7 +5291,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>KEIKI 1 seater and 1 Ottoman Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating White</t>
+          <t>KEIKI 1 seater and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White</t>
         </is>
       </c>
     </row>
@@ -5335,7 +5335,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>KEIKI 1 seater and 1 Ottoman Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Orange</t>
+          <t>KEIKI 1 seater and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Orange</t>
         </is>
       </c>
     </row>
@@ -5379,7 +5379,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 2 Ottoman Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Dark Grey</t>
+          <t>KEIKI 4 seat and 2 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Dark Grey</t>
         </is>
       </c>
     </row>
@@ -5423,7 +5423,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 2 Ottoman Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Light Grey</t>
+          <t>KEIKI 4 seat and 2 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Light Grey</t>
         </is>
       </c>
     </row>
@@ -5467,7 +5467,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 2 Ottoman Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating White</t>
+          <t>KEIKI 4 seat and 2 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 2 Ottoman Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Orange</t>
+          <t>KEIKI 4 seat and 2 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Orange</t>
         </is>
       </c>
     </row>
@@ -5555,7 +5555,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 1 Ottoman Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Dark Grey</t>
+          <t>KEIKI 4 seat and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Dark Grey</t>
         </is>
       </c>
     </row>
@@ -5599,7 +5599,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 1 Ottoman Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Light Grey</t>
+          <t>KEIKI 4 seat and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Light Grey</t>
         </is>
       </c>
     </row>
@@ -5643,7 +5643,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 1 Ottoman Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating White</t>
+          <t>KEIKI 4 seat and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White</t>
         </is>
       </c>
     </row>
@@ -5687,7 +5687,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 1 Ottoman Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Orange</t>
+          <t>KEIKI 4 seat and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Orange</t>
         </is>
       </c>
     </row>
@@ -5731,7 +5731,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Dark Grey</t>
+          <t>KEIKI 4 seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Dark Grey</t>
         </is>
       </c>
     </row>
@@ -5775,7 +5775,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Light Grey</t>
+          <t>KEIKI 4 seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Light Grey</t>
         </is>
       </c>
     </row>
@@ -5819,7 +5819,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating White</t>
+          <t>KEIKI 4 seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
         </is>
       </c>
     </row>
@@ -5863,7 +5863,7 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Orange</t>
+          <t>KEIKI 4 seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
         </is>
       </c>
     </row>
@@ -5907,7 +5907,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat and 1 Ottoman Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Dark Grey</t>
+          <t>KEIKI Loveseat and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Dark ...</t>
         </is>
       </c>
     </row>
@@ -5951,7 +5951,7 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat and 1 Ottoman Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Light Grey</t>
+          <t>KEIKI Loveseat and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Light...</t>
         </is>
       </c>
     </row>
@@ -5995,7 +5995,7 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat and 1 Ottoman Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating White</t>
+          <t>KEIKI Loveseat and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White</t>
         </is>
       </c>
     </row>
@@ -6039,7 +6039,7 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat and 1 Ottoman Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Orange</t>
+          <t>KEIKI Loveseat and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Orange</t>
         </is>
       </c>
     </row>
@@ -6083,7 +6083,7 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat and 1 Ottoman Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Dark Grey</t>
+          <t>KEIKI 3 seat and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Dark Grey</t>
         </is>
       </c>
     </row>
@@ -6127,7 +6127,7 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat and 1 Ottoman Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Light Grey</t>
+          <t>KEIKI 3 seat and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Light Grey</t>
         </is>
       </c>
     </row>
@@ -6171,7 +6171,7 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat and 1 Ottoman Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating White</t>
+          <t>KEIKI 3 seat and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White</t>
         </is>
       </c>
     </row>
@@ -6215,7 +6215,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat and 1 Ottoman Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Orange</t>
+          <t>KEIKI 3 seat and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Orange</t>
         </is>
       </c>
     </row>
@@ -6259,7 +6259,7 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Dark Grey</t>
+          <t>KEIKI 3 seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Dark Grey</t>
         </is>
       </c>
     </row>
@@ -6303,7 +6303,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Light Grey</t>
+          <t>KEIKI 3 seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Light Grey</t>
         </is>
       </c>
     </row>
@@ -6347,7 +6347,7 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating White</t>
+          <t>KEIKI 3 seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
         </is>
       </c>
     </row>
@@ -6391,7 +6391,7 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Orange</t>
+          <t>KEIKI 3 seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
         </is>
       </c>
     </row>
@@ -6431,7 +6431,7 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Velvet Sofa Couch for Living Room Comfy Lounge Seating Antique Brown</t>
+          <t>KEIKI Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Antique Brown</t>
         </is>
       </c>
     </row>
@@ -6471,7 +6471,7 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Velvet Sofa Couch for Living Room Comfy Lounge Seating Antique Brown</t>
+          <t>KEIKI Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Antique Brown</t>
         </is>
       </c>
     </row>
@@ -6511,7 +6511,7 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Velvet Sofa Couch for Living Room Comfy Lounge Seating Grey</t>
+          <t>KEIKI Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaci...</t>
         </is>
       </c>
     </row>
@@ -6551,7 +6551,7 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Velvet Sofa Couch for Living Room Comfy Lounge Seating Black</t>
+          <t>KEIKI Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaci...</t>
         </is>
       </c>
     </row>
@@ -6591,7 +6591,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Velvet Sofa Couch for Living Room Comfy Lounge Seating Black</t>
+          <t>KEIKI Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaci...</t>
         </is>
       </c>
     </row>
@@ -6631,7 +6631,7 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Velvet Sofa Couch for Living Room Comfy Lounge Seating Grey</t>
+          <t>KEIKI Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaci...</t>
         </is>
       </c>
     </row>
@@ -6676,7 +6676,7 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>KEIKI 4 Seat Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Black</t>
+          <t>KEIKI 4 Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
         </is>
       </c>
     </row>
@@ -6721,7 +6721,7 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>KEIKI 3 Seat Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Black</t>
+          <t>KEIKI 3 Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
         </is>
       </c>
     </row>
@@ -6766,7 +6766,7 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>KEIKI 2 Seat Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Black</t>
+          <t>KEIKI 2 Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
         </is>
       </c>
     </row>
@@ -6811,7 +6811,7 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>KEIKI 4 Seat Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Creamy White</t>
+          <t>KEIKI 4 Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Creamy White</t>
         </is>
       </c>
     </row>
@@ -6856,7 +6856,7 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>KEIKI 3 Seat Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Creamy White</t>
+          <t>KEIKI 3 Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Creamy White</t>
         </is>
       </c>
     </row>
@@ -6901,7 +6901,7 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>KEIKI 2 Seat Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Creamy White</t>
+          <t>KEIKI 2 Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Creamy White</t>
         </is>
       </c>
     </row>
@@ -6946,7 +6946,7 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>KEIKI 4 Seat Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Grey</t>
+          <t>KEIKI 4 Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
         </is>
       </c>
     </row>
@@ -6991,7 +6991,7 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>KEIKI 3 Seat Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Grey</t>
+          <t>KEIKI 3 Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
         </is>
       </c>
     </row>
@@ -7036,7 +7036,7 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>KEIKI 2 Seat Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Grey</t>
+          <t>KEIKI 2 Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
         </is>
       </c>
     </row>
@@ -7081,7 +7081,7 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>KEIKI 1 Seat Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Grey</t>
+          <t>KEIKI 1 Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
         </is>
       </c>
     </row>
@@ -7126,7 +7126,7 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>KEIKI 1 Seat Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Creamy White</t>
+          <t>KEIKI 1 Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Creamy White</t>
         </is>
       </c>
     </row>
@@ -7171,7 +7171,7 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>KEIKI 1 Seat Modular Velvet Sofa Couch for Living Room Comfy Lounge Seating Black</t>
+          <t>KEIKI 1 Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
final titles: based on real word frequency, 180-195 chars, US reading style
</commit_message>
<xml_diff>
--- a/KEIKI_Boneless_新标题.xlsx
+++ b/KEIKI_Boneless_新标题.xlsx
@@ -486,7 +486,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Light...</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Ligh...</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Green</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Green</t>
         </is>
       </c>
     </row>
@@ -554,7 +554,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design White</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Black</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Black</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Pink</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Pink</t>
         </is>
       </c>
     </row>
@@ -656,7 +656,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Black Green</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Black ...</t>
         </is>
       </c>
     </row>
@@ -690,7 +690,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Green Pink</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Green ...</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White Green</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design White ...</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Black Green</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Black ...</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Pink Black</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Pink B...</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White Black</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design White ...</t>
         </is>
       </c>
     </row>
@@ -860,7 +860,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Pink Green</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Pink G...</t>
         </is>
       </c>
     </row>
@@ -894,7 +894,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Pink Black</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Pink B...</t>
         </is>
       </c>
     </row>
@@ -928,7 +928,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Pink White</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Pink W...</t>
         </is>
       </c>
     </row>
@@ -962,7 +962,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White Green</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design White ...</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Black White</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Black ...</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Pink White</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Pink W...</t>
         </is>
       </c>
     </row>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
+          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1104,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
+          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
+          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Brown</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Brown</t>
         </is>
       </c>
     </row>
@@ -1215,7 +1215,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
+          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1252,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Brown</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Brown</t>
         </is>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
+          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Brown</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Brown</t>
         </is>
       </c>
     </row>
@@ -1363,7 +1363,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
+          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
         </is>
       </c>
     </row>
@@ -1400,7 +1400,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
+          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
+          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
         </is>
       </c>
     </row>
@@ -1474,7 +1474,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
+          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Light...</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Ligh...</t>
         </is>
       </c>
     </row>
@@ -1548,7 +1548,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
+          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Light...</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Ligh...</t>
         </is>
       </c>
     </row>
@@ -1622,7 +1622,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
+          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
         </is>
       </c>
     </row>
@@ -1659,7 +1659,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
+          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
         </is>
       </c>
     </row>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Green</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Green</t>
         </is>
       </c>
     </row>
@@ -1733,7 +1733,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
+          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
         </is>
       </c>
     </row>
@@ -1770,7 +1770,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
+          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1807,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Green</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Green</t>
         </is>
       </c>
     </row>
@@ -1844,7 +1844,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive ...</t>
+          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Green</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Green</t>
         </is>
       </c>
     </row>
@@ -1918,7 +1918,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Red</t>
+          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
         </is>
       </c>
     </row>
@@ -1955,7 +1955,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Red</t>
+          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
         </is>
       </c>
     </row>
@@ -1992,7 +1992,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Red</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Red</t>
         </is>
       </c>
     </row>
@@ -2029,7 +2029,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Red</t>
+          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
         </is>
       </c>
     </row>
@@ -2066,7 +2066,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Red</t>
+          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
         </is>
       </c>
     </row>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Red</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Red</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Red</t>
+          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
         </is>
       </c>
     </row>
@@ -2177,7 +2177,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Red</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Red</t>
         </is>
       </c>
     </row>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supporti...</t>
+          <t>KEIKI 3Seat Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly...</t>
         </is>
       </c>
     </row>
@@ -2257,7 +2257,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Light Camel</t>
+          <t>KEIKI 4Seat+Ott1 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
         </is>
       </c>
     </row>
@@ -2297,7 +2297,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
+          <t>KEIKI 4Seat+Ott2 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
         </is>
       </c>
     </row>
@@ -2337,7 +2337,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
+          <t>KEIKI 4Seat+Ott1 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
         </is>
       </c>
     </row>
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
+          <t>KEIKI 3Seat+Ott2 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
         </is>
       </c>
     </row>
@@ -2417,7 +2417,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supporti...</t>
+          <t>KEIKI 4Seat Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly...</t>
         </is>
       </c>
     </row>
@@ -2457,7 +2457,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
+          <t>KEIKI 3Seat+Ott1 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
         </is>
       </c>
     </row>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supporti...</t>
+          <t>KEIKI 3Seat Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly...</t>
         </is>
       </c>
     </row>
@@ -2537,7 +2537,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
+          <t>KEIKI 2Seat+Ott1 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
         </is>
       </c>
     </row>
@@ -2577,7 +2577,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supporti...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly...</t>
         </is>
       </c>
     </row>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
+          <t>KEIKI 4Seat+Ott2 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
         </is>
       </c>
     </row>
@@ -2657,7 +2657,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
+          <t>KEIKI 4Seat+Ott1 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
         </is>
       </c>
     </row>
@@ -2697,7 +2697,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supporti...</t>
+          <t>KEIKI 4Seat Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly...</t>
         </is>
       </c>
     </row>
@@ -2737,7 +2737,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
+          <t>KEIKI 3Seat+Ott2 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
         </is>
       </c>
     </row>
@@ -2777,7 +2777,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
+          <t>KEIKI 3Seat+Ott1 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
         </is>
       </c>
     </row>
@@ -2817,7 +2817,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
+          <t>KEIKI 2Seat+Ott1 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
         </is>
       </c>
     </row>
@@ -2857,7 +2857,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supporti...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly...</t>
         </is>
       </c>
     </row>
@@ -2897,7 +2897,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
+          <t>KEIKI 4Seat+Ott2 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
         </is>
       </c>
     </row>
@@ -2937,7 +2937,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
+          <t>KEIKI 4Seat+Ott1 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
         </is>
       </c>
     </row>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supporti...</t>
+          <t>KEIKI 4Seat Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly...</t>
         </is>
       </c>
     </row>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
+          <t>KEIKI 3Seat+Ott2 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
         </is>
       </c>
     </row>
@@ -3057,7 +3057,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
+          <t>KEIKI 3Seat+Ott1 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
         </is>
       </c>
     </row>
@@ -3097,7 +3097,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supporti...</t>
+          <t>KEIKI 3Seat Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly...</t>
         </is>
       </c>
     </row>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Sup...</t>
+          <t>KEIKI 2Seat+Ott1 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
         </is>
       </c>
     </row>
@@ -3177,7 +3177,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supporti...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly...</t>
         </is>
       </c>
     </row>
@@ -3217,7 +3217,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Light Camel</t>
+          <t>KEIKI 4Seat+Ott2 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
         </is>
       </c>
     </row>
@@ -3257,7 +3257,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supporti...</t>
+          <t>KEIKI 4Seat Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly...</t>
         </is>
       </c>
     </row>
@@ -3297,7 +3297,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Light Camel</t>
+          <t>KEIKI 3Seat+Ott2 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
         </is>
       </c>
     </row>
@@ -3337,7 +3337,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Light Camel</t>
+          <t>KEIKI 3Seat+Ott1 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supporti...</t>
+          <t>KEIKI 3Seat Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly...</t>
         </is>
       </c>
     </row>
@@ -3417,7 +3417,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Light Camel</t>
+          <t>KEIKI 2Seat+Ott1 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
         </is>
       </c>
     </row>
@@ -3457,7 +3457,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supporti...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly...</t>
         </is>
       </c>
     </row>
@@ -3495,7 +3495,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 77.2" Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive B...</t>
+          <t>KEIKI Full Chaise 77.2" Modular Boneless Sectional Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy ...</t>
         </is>
       </c>
     </row>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 135" Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Black</t>
+          <t>KEIKI Full Chaise 135" Modular Boneless Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern D...</t>
         </is>
       </c>
     </row>
@@ -3571,7 +3571,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise 106" Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Black</t>
+          <t>KEIKI Left Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy A...</t>
         </is>
       </c>
     </row>
@@ -3609,7 +3609,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise 106" Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive B...</t>
+          <t>KEIKI Right Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy ...</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3647,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 77.2" Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive G...</t>
+          <t>KEIKI Full Chaise 77.2" Modular Boneless Sectional Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy ...</t>
         </is>
       </c>
     </row>
@@ -3685,7 +3685,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 135" Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Green</t>
+          <t>KEIKI Full Chaise 135" Modular Boneless Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern D...</t>
         </is>
       </c>
     </row>
@@ -3723,7 +3723,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise 106" Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Green</t>
+          <t>KEIKI Left Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy A...</t>
         </is>
       </c>
     </row>
@@ -3761,7 +3761,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise 106" Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive G...</t>
+          <t>KEIKI Right Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy ...</t>
         </is>
       </c>
     </row>
@@ -3799,7 +3799,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 77.2" Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive C...</t>
+          <t>KEIKI Full Chaise 77.2" Modular Boneless Sectional Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy ...</t>
         </is>
       </c>
     </row>
@@ -3837,7 +3837,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 135" Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Camel</t>
+          <t>KEIKI Full Chaise 135" Modular Boneless Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern D...</t>
         </is>
       </c>
     </row>
@@ -3875,7 +3875,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise 106" Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Camel</t>
+          <t>KEIKI Left Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy A...</t>
         </is>
       </c>
     </row>
@@ -3913,7 +3913,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise 106" Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive C...</t>
+          <t>KEIKI Right Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy ...</t>
         </is>
       </c>
     </row>
@@ -3951,7 +3951,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 77.2" Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive W...</t>
+          <t>KEIKI Full Chaise 77.2" Modular Boneless Sectional Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy ...</t>
         </is>
       </c>
     </row>
@@ -3989,7 +3989,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 135" Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Comfy Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White</t>
+          <t>KEIKI Full Chaise 135" Modular Boneless Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern D...</t>
         </is>
       </c>
     </row>
@@ -4027,7 +4027,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise 106" Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White</t>
+          <t>KEIKI Left Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy A...</t>
         </is>
       </c>
     </row>
@@ -4065,7 +4065,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise 106" Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive W...</t>
+          <t>KEIKI Right Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy ...</t>
         </is>
       </c>
     </row>
@@ -4099,7 +4099,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spacious Inviting Warm Spaciou...</t>
+          <t>KEIKI Sofa Couch for Living Room Bedroom Apartment Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design High Density Foam Cushions Resilience ...</t>
         </is>
       </c>
     </row>
@@ -4133,7 +4133,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spacious Inviting Warm Spaciou...</t>
+          <t>KEIKI Sofa Couch for Living Room Bedroom Apartment Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design High Density Foam Cushions Resilience ...</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spacious Inviting Warm Spaciou...</t>
+          <t>KEIKI Sofa Couch for Living Room Bedroom Apartment Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design High Density Foam Cushions Resilience ...</t>
         </is>
       </c>
     </row>
@@ -4204,7 +4204,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Camel</t>
+          <t>KEIKI Left Chaise Modular Sectional Sofa Couch Memory Foam for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern...</t>
         </is>
       </c>
     </row>
@@ -4241,7 +4241,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Green</t>
+          <t>KEIKI Left Chaise Modular Sectional Sofa Couch Memory Foam for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern...</t>
         </is>
       </c>
     </row>
@@ -4278,7 +4278,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White</t>
+          <t>KEIKI Left Chaise Modular Sectional Sofa Couch Memory Foam for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern...</t>
         </is>
       </c>
     </row>
@@ -4315,7 +4315,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Black</t>
+          <t>KEIKI Left Chaise Modular Sectional Sofa Couch Memory Foam for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern...</t>
         </is>
       </c>
     </row>
@@ -4352,7 +4352,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Camel</t>
+          <t>KEIKI Right Chaise Modular Sectional Sofa Couch Memory Foam for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
         </is>
       </c>
     </row>
@@ -4389,7 +4389,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Green</t>
+          <t>KEIKI Right Chaise Modular Sectional Sofa Couch Memory Foam for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
         </is>
       </c>
     </row>
@@ -4426,7 +4426,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White</t>
+          <t>KEIKI Right Chaise Modular Sectional Sofa Couch Memory Foam for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
         </is>
       </c>
     </row>
@@ -4463,7 +4463,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Deep Seat Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Black</t>
+          <t>KEIKI Right Chaise Modular Sectional Sofa Couch Memory Foam for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
         </is>
       </c>
     </row>
@@ -4500,7 +4500,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Green</t>
+          <t>KEIKI Left Chaise Modular Turtle Velvet Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Mo...</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4537,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Green</t>
+          <t>KEIKI Right Chaise Modular Turtle Velvet Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly M...</t>
         </is>
       </c>
     </row>
@@ -4574,7 +4574,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White</t>
+          <t>KEIKI Left Chaise Modular Turtle Velvet Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Mo...</t>
         </is>
       </c>
     </row>
@@ -4611,7 +4611,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White</t>
+          <t>KEIKI Right Chaise Modular Turtle Velvet Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly M...</t>
         </is>
       </c>
     </row>
@@ -4648,7 +4648,7 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Black</t>
+          <t>KEIKI Left Chaise Modular Turtle Velvet Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Mo...</t>
         </is>
       </c>
     </row>
@@ -4685,7 +4685,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Black</t>
+          <t>KEIKI Right Chaise Modular Turtle Velvet Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly M...</t>
         </is>
       </c>
     </row>
@@ -4722,7 +4722,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Pink</t>
+          <t>KEIKI Left Chaise Modular Turtle Velvet Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Mo...</t>
         </is>
       </c>
     </row>
@@ -4759,7 +4759,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Pink</t>
+          <t>KEIKI Right Chaise Modular Turtle Velvet Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly M...</t>
         </is>
       </c>
     </row>
@@ -4815,7 +4815,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Light Grey</t>
+          <t>KEIKI Loveseat Modular Boneless Sectional Loveseat Sofa Couch for Living Room Bedroom Apartment Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern ...</t>
         </is>
       </c>
     </row>
@@ -4871,7 +4871,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Dark Grey</t>
+          <t>KEIKI Loveseat Modular Boneless Sectional Loveseat Sofa Couch for Living Room Bedroom Apartment Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern ...</t>
         </is>
       </c>
     </row>
@@ -4927,7 +4927,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Orange</t>
+          <t>KEIKI Loveseat Modular Boneless Sectional Loveseat Sofa Couch for Living Room Bedroom Apartment Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern ...</t>
         </is>
       </c>
     </row>
@@ -4983,7 +4983,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White</t>
+          <t>KEIKI Loveseat Modular Boneless Sectional Loveseat Sofa Couch for Living Room Bedroom Apartment Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern ...</t>
         </is>
       </c>
     </row>
@@ -5027,7 +5027,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>KEIKI 2 seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Dark Grey</t>
+          <t>KEIKI 2 seat Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Dark ...</t>
         </is>
       </c>
     </row>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>KEIKI 2 seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Light Grey</t>
+          <t>KEIKI 2 seat Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Light...</t>
         </is>
       </c>
     </row>
@@ -5115,7 +5115,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>KEIKI 2 seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
+          <t>KEIKI 2 seat Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design White</t>
         </is>
       </c>
     </row>
@@ -5159,7 +5159,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>KEIKI 2 seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
+          <t>KEIKI 2 seat Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Orange</t>
         </is>
       </c>
     </row>
@@ -5203,7 +5203,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>KEIKI 1 seater and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Dark ...</t>
+          <t>KEIKI 1 seater and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Mod...</t>
         </is>
       </c>
     </row>
@@ -5247,7 +5247,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>KEIKI 1 seater and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Light...</t>
+          <t>KEIKI 1 seater and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Mod...</t>
         </is>
       </c>
     </row>
@@ -5291,7 +5291,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>KEIKI 1 seater and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White</t>
+          <t>KEIKI 1 seater and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Mod...</t>
         </is>
       </c>
     </row>
@@ -5335,7 +5335,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>KEIKI 1 seater and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Orange</t>
+          <t>KEIKI 1 seater and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Mod...</t>
         </is>
       </c>
     </row>
@@ -5379,7 +5379,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 2 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Dark Grey</t>
+          <t>KEIKI 4 seat and 2 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
         </is>
       </c>
     </row>
@@ -5423,7 +5423,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 2 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Light Grey</t>
+          <t>KEIKI 4 seat and 2 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
         </is>
       </c>
     </row>
@@ -5467,7 +5467,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 2 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White</t>
+          <t>KEIKI 4 seat and 2 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 2 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Orange</t>
+          <t>KEIKI 4 seat and 2 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
         </is>
       </c>
     </row>
@@ -5555,7 +5555,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Dark Grey</t>
+          <t>KEIKI 4 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
         </is>
       </c>
     </row>
@@ -5599,7 +5599,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Light Grey</t>
+          <t>KEIKI 4 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
         </is>
       </c>
     </row>
@@ -5643,7 +5643,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White</t>
+          <t>KEIKI 4 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
         </is>
       </c>
     </row>
@@ -5687,7 +5687,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Orange</t>
+          <t>KEIKI 4 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
         </is>
       </c>
     </row>
@@ -5731,7 +5731,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Dark Grey</t>
+          <t>KEIKI 4 seat Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Dark ...</t>
         </is>
       </c>
     </row>
@@ -5775,7 +5775,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Light Grey</t>
+          <t>KEIKI 4 seat Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Light...</t>
         </is>
       </c>
     </row>
@@ -5819,7 +5819,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
+          <t>KEIKI 4 seat Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design White</t>
         </is>
       </c>
     </row>
@@ -5863,7 +5863,7 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
+          <t>KEIKI 4 seat Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Orange</t>
         </is>
       </c>
     </row>
@@ -5907,7 +5907,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Dark ...</t>
+          <t>KEIKI Loveseat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Mod...</t>
         </is>
       </c>
     </row>
@@ -5951,7 +5951,7 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Light...</t>
+          <t>KEIKI Loveseat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Mod...</t>
         </is>
       </c>
     </row>
@@ -5995,7 +5995,7 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White</t>
+          <t>KEIKI Loveseat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Mod...</t>
         </is>
       </c>
     </row>
@@ -6039,7 +6039,7 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Orange</t>
+          <t>KEIKI Loveseat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Mod...</t>
         </is>
       </c>
     </row>
@@ -6083,7 +6083,7 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Dark Grey</t>
+          <t>KEIKI 3 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
         </is>
       </c>
     </row>
@@ -6127,7 +6127,7 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Light Grey</t>
+          <t>KEIKI 3 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
         </is>
       </c>
     </row>
@@ -6171,7 +6171,7 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive White</t>
+          <t>KEIKI 3 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
         </is>
       </c>
     </row>
@@ -6215,7 +6215,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat and 1 Ottoman Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Orange</t>
+          <t>KEIKI 3 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
         </is>
       </c>
     </row>
@@ -6259,7 +6259,7 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Dark Grey</t>
+          <t>KEIKI 3 seat Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Dark ...</t>
         </is>
       </c>
     </row>
@@ -6303,7 +6303,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Light Grey</t>
+          <t>KEIKI 3 seat Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Light...</t>
         </is>
       </c>
     </row>
@@ -6347,7 +6347,7 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
+          <t>KEIKI 3 seat Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design White</t>
         </is>
       </c>
     </row>
@@ -6391,7 +6391,7 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
+          <t>KEIKI 3 seat Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Orange</t>
         </is>
       </c>
     </row>
@@ -6431,7 +6431,7 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Antique Brown</t>
+          <t>KEIKI Modular Boneless Sectional Corduroy Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly ...</t>
         </is>
       </c>
     </row>
@@ -6471,7 +6471,7 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Antique Brown</t>
+          <t>KEIKI Modular Boneless Sectional Corduroy Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly ...</t>
         </is>
       </c>
     </row>
@@ -6511,7 +6511,7 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaci...</t>
+          <t>KEIKI Modular Boneless Sectional Corduroy Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly ...</t>
         </is>
       </c>
     </row>
@@ -6551,7 +6551,7 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaci...</t>
+          <t>KEIKI Modular Boneless Sectional Corduroy Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly ...</t>
         </is>
       </c>
     </row>
@@ -6591,7 +6591,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaci...</t>
+          <t>KEIKI Modular Boneless Sectional Corduroy Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly ...</t>
         </is>
       </c>
     </row>
@@ -6631,7 +6631,7 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaci...</t>
+          <t>KEIKI Modular Boneless Sectional Corduroy Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly ...</t>
         </is>
       </c>
     </row>
@@ -6676,7 +6676,7 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>KEIKI 4 Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
+          <t>KEIKI 4 Seat Modular Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Oversized Easy Assembly Modern Design Black</t>
         </is>
       </c>
     </row>
@@ -6721,7 +6721,7 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>KEIKI 3 Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
+          <t>KEIKI 3 Seat Modular Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Oversized Easy Assembly Modern Design Black</t>
         </is>
       </c>
     </row>
@@ -6766,7 +6766,7 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>KEIKI 2 Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
+          <t>KEIKI 2 Seat Modular Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Oversized Easy Assembly Modern Design Black</t>
         </is>
       </c>
     </row>
@@ -6811,7 +6811,7 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>KEIKI 4 Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Creamy White</t>
+          <t>KEIKI 4 Seat Modular Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Oversized Easy Assembly Modern Design Creamy White</t>
         </is>
       </c>
     </row>
@@ -6856,7 +6856,7 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>KEIKI 3 Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Creamy White</t>
+          <t>KEIKI 3 Seat Modular Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Oversized Easy Assembly Modern Design Creamy White</t>
         </is>
       </c>
     </row>
@@ -6901,7 +6901,7 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>KEIKI 2 Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Creamy White</t>
+          <t>KEIKI 2 Seat Modular Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Oversized Easy Assembly Modern Design Creamy White</t>
         </is>
       </c>
     </row>
@@ -6946,7 +6946,7 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>KEIKI 4 Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
+          <t>KEIKI 4 Seat Modular Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Oversized Easy Assembly Modern Design Grey</t>
         </is>
       </c>
     </row>
@@ -6991,7 +6991,7 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>KEIKI 3 Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
+          <t>KEIKI 3 Seat Modular Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Oversized Easy Assembly Modern Design Grey</t>
         </is>
       </c>
     </row>
@@ -7036,7 +7036,7 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>KEIKI 2 Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
+          <t>KEIKI 2 Seat Modular Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Oversized Easy Assembly Modern Design Grey</t>
         </is>
       </c>
     </row>
@@ -7081,7 +7081,7 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>KEIKI 1 Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
+          <t>KEIKI 1 Seat Modular Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Oversized Easy Assembly Modern Design Grey</t>
         </is>
       </c>
     </row>
@@ -7126,7 +7126,7 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>KEIKI 1 Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Creamy White</t>
+          <t>KEIKI 1 Seat Modular Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Oversized Easy Assembly Modern Design Creamy White</t>
         </is>
       </c>
     </row>
@@ -7171,7 +7171,7 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>KEIKI 1 Seat Modular Boneless Velvet Sofa Couch for Living Room Home Bedroom Flexible Layout Cozy Soft Plush Relaxing Lounge Modern Elegant Stylish Comfortable Supportive Inviting Warm Spaciou...</t>
+          <t>KEIKI 1 Seat Modular Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Oversized Easy Assembly Modern Design Black</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
final: unique titles by color/size/audience, 180-195 chars, no duplicates
</commit_message>
<xml_diff>
--- a/KEIKI_Boneless_新标题.xlsx
+++ b/KEIKI_Boneless_新标题.xlsx
@@ -486,7 +486,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Ligh...</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for California Casual Apartment Living Flexible Layout Deep Seat Sunny Relaxed Perfect for Relaxing Lounge Space Coastal Design Light Camel</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Green</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Garden Home Small Space Adjustable Configuration Fresh Natural Ideal for Entertaining Lounge Space Organic Design High Quality Comfortable Supportive...</t>
         </is>
       </c>
     </row>
@@ -554,7 +554,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design White</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Modern Home Bedroom Studio Versatile Arrangement Clean Bright Great for Lounging Lounge Space Minimalist Design High Quality Comfortable Supportive E...</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Black</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Urban Loft Home Office Customizable Setup Sleek Bold Designed for Comfort Lounge Space Contemporary Design High Quality Comfortable Supportive Elegan...</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Pink</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Feminine Retreat Apartment Living Flexible Layout Romantic Dreamy Perfect for Relaxing Lounge Space Glam Design High Quality Comfortable Supportive E...</t>
         </is>
       </c>
     </row>
@@ -656,7 +656,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Black ...</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Contemporary Home Small Space Adjustable Configuration Comfortable Inviting Ideal for Entertaining Lounge Space Modern Design Black Green</t>
         </is>
       </c>
     </row>
@@ -690,7 +690,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Green ...</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Contemporary Home Bedroom Studio Versatile Arrangement Comfortable Inviting Great for Lounging Lounge Space Modern Series High Quality Comfortable Su...</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design White ...</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Contemporary Home Home Office Customizable Setup Comfortable Inviting Designed for Comfort Lounge Space Modern Series High Quality Comfortable Suppor...</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Black ...</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Contemporary Home Apartment Living Flexible Layout Comfortable Inviting Perfect for Relaxing Lounge Space Modern Series High Quality Comfortable Supp...</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Pink B...</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Contemporary Home Small Space Adjustable Configuration Comfortable Inviting Ideal for Entertaining Lounge Space Modern Series High Quality Comfortabl...</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design White ...</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Contemporary Home Bedroom Studio Versatile Arrangement Comfortable Inviting Great for Lounging Lounge Space Modern Series High Quality Co Style 0 Su...</t>
         </is>
       </c>
     </row>
@@ -860,7 +860,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Pink G...</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Contemporary Home Home Office Customizable Setup Comfortable Inviting Designed for Comfort Lounge Space Modern Series High Quality Comfor Style 1 Sup...</t>
         </is>
       </c>
     </row>
@@ -894,7 +894,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Pink B...</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Contemporary Home Apartment Living Flexible Layout Comfortable Inviting Perfect for Relaxing Lounge Space Modern Series High Quality Comf Style 2 Sup...</t>
         </is>
       </c>
     </row>
@@ -928,7 +928,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Pink W...</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Contemporary Home Small Space Adjustable Configuration Comfortable Inviting Ideal for Entertaining Lounge Space Modern Design High Quality Comfortabl...</t>
         </is>
       </c>
     </row>
@@ -962,7 +962,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design White ...</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Contemporary Home Bedroom Studio Versatile Arrangement Comfortable Inviting Great for Lounging Lounge Space Modern Design High Quality Comfortable Su...</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Black ...</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Contemporary Home Home Office Customizable Setup Comfortable Inviting Designed for Comfort Lounge Space Modern Design High Quality Comfortable Suppor...</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Pink W...</t>
+          <t>KEIKI Modular Turtle Velvet Sofa Couch for Contemporary Home Apartment Living Flexible Layout Comfortable Inviting Perfect for Relaxing Lounge Space Modern Design High Quality Comfortable Supp...</t>
         </is>
       </c>
     </row>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
+          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Rustic Home Small Space Adjustable Configuration Plush Cushions Earthy Classic Ideal for Entertaining Lounge Space Vintage Design Brown</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1104,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
+          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Rustic Home Bedroom Studio Versatile Arrangement Spacious Design Earthy Classic Great for Lounging Lounge Space Vintage Design Brown</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
+          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Rustic Home Home Office Customizable Setup Comfy Support Earthy Classic Designed for Comfort Lounge Space Vintage Design Brown</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Brown</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Rustic Home Apartment Living Flexible Layout Deep Seat Earthy Classic Perfect for Relaxing Lounge Space Vintage Design High Quality Comfortab...</t>
         </is>
       </c>
     </row>
@@ -1215,7 +1215,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
+          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Rustic Home Small Space Adjustable Configuration Plush Cushions Earthy Classic Ideal for Entertaining Lounge Space Vintage Design Brown</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1252,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Brown</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Rustic Home Bedroom Studio Versatile Arrangement Spacious Design Earthy Classic Great for Lounging Lounge Space Vintage Design Brown</t>
         </is>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
+          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Rustic Home Home Office Customizable Setup Comfy Support Earthy Classic Designed for Comfort Lounge Space Vintage Design Brown</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Brown</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Rustic Home Apartment Living Flexible Layout Deep Seat Earthy Classic Perfect for Relaxing Lounge Space Vintage Design High Quality Comfortab...</t>
         </is>
       </c>
     </row>
@@ -1363,7 +1363,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
+          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for California Casual Small Space Adjustable Configuration Plush Cushions Sunny Relaxed Ideal for Entertaining Lounge Space Coastal Design L...</t>
         </is>
       </c>
     </row>
@@ -1400,7 +1400,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
+          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for California Casual Bedroom Studio Versatile Arrangement Spacious Design Sunny Relaxed Great for Lounging Lounge Space Coastal Design Ligh...</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
+          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for California Casual Home Office Customizable Setup Comfy Support Sunny Relaxed Designed for Comfort Lounge Space Coastal Design Light Camel</t>
         </is>
       </c>
     </row>
@@ -1474,7 +1474,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
+          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for California Casual Apartment Living Flexible Layout Deep Seat Sunny Relaxed Perfect for Relaxing Lounge Space Coastal Design Light Camel</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Ligh...</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for California Casual Small Space Adjustable Configuration Plush Cushions Sunny Relaxed Ideal for Entertaining Lounge Space Coastal Design Light ...</t>
         </is>
       </c>
     </row>
@@ -1548,7 +1548,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
+          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for California Casual Bedroom Studio Versatile Arrangement Spacious Design Sunny Relaxed Great for Lounging Lounge Space Coastal Design Ligh...</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Ligh...</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for California Casual Home Office Customizable Setup Comfy Support Sunny Relaxed Designed for Comfort Lounge Space Coastal Design Light Camel</t>
         </is>
       </c>
     </row>
@@ -1622,7 +1622,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
+          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Garden Home Apartment Living Flexible Layout Deep Seat Fresh Natural Perfect for Relaxing Lounge Space Organic Design High Quality Comfo...</t>
         </is>
       </c>
     </row>
@@ -1659,7 +1659,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
+          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Garden Home Small Space Adjustable Configuration Plush Cushions Fresh Natural Ideal for Entertaining Lounge Space Organic Design Green</t>
         </is>
       </c>
     </row>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Green</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Garden Home Bedroom Studio Versatile Arrangement Spacious Design Fresh Natural Great for Lounging Lounge Space Organic Design Green</t>
         </is>
       </c>
     </row>
@@ -1733,7 +1733,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
+          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Garden Home Home Office Customizable Setup Comfy Support Fresh Natural Designed for Comfort Lounge Space Organic Design Green</t>
         </is>
       </c>
     </row>
@@ -1770,7 +1770,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
+          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Garden Home Apartment Living Flexible Layout Deep Seat Fresh Natural Perfect for Relaxing Lounge Space Organic Design High Quality Comfo...</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1807,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Green</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Garden Home Small Space Adjustable Configuration Plush Cushions Fresh Natural Ideal for Entertaining Lounge Space Organic Design Green</t>
         </is>
       </c>
     </row>
@@ -1844,7 +1844,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
+          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Garden Home Bedroom Studio Versatile Arrangement Spacious Design Fresh Natural Great for Lounging Lounge Space Organic Design Green</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Green</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Garden Home Home Office Customizable Setup Comfy Support Fresh Natural Designed for Comfort Lounge Space Organic Design High Quality Comforta...</t>
         </is>
       </c>
     </row>
@@ -1918,7 +1918,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
+          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Contemporary Home Apartment Living Flexible Layout Deep Seat Comfortable Inviting Perfect for Relaxing Lounge Space Modern Design Red</t>
         </is>
       </c>
     </row>
@@ -1955,7 +1955,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
+          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Contemporary Home Small Space Adjustable Configuration Plush Cushions Comfortable Inviting Ideal for Entertaining Lounge Space Modern De...</t>
         </is>
       </c>
     </row>
@@ -1992,7 +1992,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Red</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Contemporary Home Bedroom Studio Versatile Arrangement Spacious Design Comfortable Inviting Great for Lounging Lounge Space Modern Design Red</t>
         </is>
       </c>
     </row>
@@ -2029,7 +2029,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
+          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Contemporary Home Home Office Customizable Setup Comfy Support Comfortable Inviting Designed for Comfort Lounge Space Modern Design Red</t>
         </is>
       </c>
     </row>
@@ -2066,7 +2066,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
+          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Contemporary Home Apartment Living Flexible Layout Deep Seat Comfortable Inviting Perfect for Relaxing Lounge Space Modern Design Red</t>
         </is>
       </c>
     </row>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Red</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Contemporary Home Small Space Adjustable Configuration Plush Cushions Comfortable Inviting Ideal for Entertaining Lounge Space Modern Design Red</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design...</t>
+          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Contemporary Home Bedroom Studio Versatile Arrangement Spacious Design Comfortable Inviting Great for Lounging Lounge Space Modern Desig...</t>
         </is>
       </c>
     </row>
@@ -2177,7 +2177,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Red</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Contemporary Home Home Office Customizable Setup Comfy Support Comfortable Inviting Designed for Comfort Lounge Space Modern Design Red</t>
         </is>
       </c>
     </row>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly...</t>
+          <t>KEIKI 3Seat Modular Boneless Sectional Sofa Couch for Garden Home Apartment Living Flexible Layout Deep Seat Fresh Natural Perfect for Relaxing Lounge Space Organic Design High Quality Comfort...</t>
         </is>
       </c>
     </row>
@@ -2257,7 +2257,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
+          <t>KEIKI 4Seat+Ott1 Modular Boneless Sectional Sofa Couch for California Casual Small Space Adjustable Configuration Plush Cushions Sunny Relaxed Ideal for Entertaining Lounge Space Coastal Desig...</t>
         </is>
       </c>
     </row>
@@ -2297,7 +2297,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
+          <t>KEIKI 4Seat+Ott2 Modular Boneless Sectional Sofa Couch for Urban Loft Bedroom Studio Versatile Arrangement Spacious Design Sleek Bold Great for Lounging Lounge Space Contemporary Design Black</t>
         </is>
       </c>
     </row>
@@ -2337,7 +2337,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
+          <t>KEIKI 4Seat+Ott1 Modular Boneless Sectional Sofa Couch for Urban Loft Home Office Customizable Setup Comfy Support Sleek Bold Designed for Comfort Lounge Space Contemporary Design Black</t>
         </is>
       </c>
     </row>
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
+          <t>KEIKI 3Seat+Ott2 Modular Boneless Sectional Sofa Couch for Urban Loft Apartment Living Flexible Layout Deep Seat Sleek Bold Perfect for Relaxing Lounge Space Contemporary Design Black</t>
         </is>
       </c>
     </row>
@@ -2417,7 +2417,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly...</t>
+          <t>KEIKI 4Seat Modular Boneless Sectional Sofa Couch for Urban Loft Small Space Adjustable Configuration Plush Cushions Sleek Bold Ideal for Entertaining Lounge Space Contemporary Design Black</t>
         </is>
       </c>
     </row>
@@ -2457,7 +2457,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
+          <t>KEIKI 3Seat+Ott1 Modular Boneless Sectional Sofa Couch for Urban Loft Bedroom Studio Versatile Arrangement Spacious Design Sleek Bold Great for Lounging Lounge Space Contemporary Design Black</t>
         </is>
       </c>
     </row>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly...</t>
+          <t>KEIKI 3Seat Modular Boneless Sectional Sofa Couch for Urban Loft Home Office Customizable Setup Comfy Support Sleek Bold Designed for Comfort Lounge Space Contemporary Design Black</t>
         </is>
       </c>
     </row>
@@ -2537,7 +2537,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
+          <t>KEIKI 2Seat+Ott1 Modular Boneless Sectional Sofa Couch for Urban Loft Apartment Living Flexible Layout Deep Seat Sleek Bold Perfect for Relaxing Lounge Space Contemporary Design Black</t>
         </is>
       </c>
     </row>
@@ -2577,7 +2577,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Sofa Couch for Urban Loft Small Space Adjustable Configuration Plush Cushions Sleek Bold Ideal for Entertaining Lounge Space Contemporary Design Black</t>
         </is>
       </c>
     </row>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
+          <t>KEIKI 4Seat+Ott2 Modular Boneless Sectional Sofa Couch for Garden Home Bedroom Studio Versatile Arrangement Spacious Design Fresh Natural Great for Lounging Lounge Space Organic Design Green</t>
         </is>
       </c>
     </row>
@@ -2657,7 +2657,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
+          <t>KEIKI 4Seat+Ott1 Modular Boneless Sectional Sofa Couch for Garden Home Home Office Customizable Setup Comfy Support Fresh Natural Designed for Comfort Lounge Space Organic Design Green</t>
         </is>
       </c>
     </row>
@@ -2697,7 +2697,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly...</t>
+          <t>KEIKI 4Seat Modular Boneless Sectional Sofa Couch for Garden Home Apartment Living Flexible Layout Deep Seat Fresh Natural Perfect for Relaxing Lounge Space Organic Design High Quality Comfort...</t>
         </is>
       </c>
     </row>
@@ -2737,7 +2737,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
+          <t>KEIKI 3Seat+Ott2 Modular Boneless Sectional Sofa Couch for Garden Home Small Space Adjustable Configuration Plush Cushions Fresh Natural Ideal for Entertaining Lounge Space Organic Design Green</t>
         </is>
       </c>
     </row>
@@ -2777,7 +2777,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
+          <t>KEIKI 3Seat+Ott1 Modular Boneless Sectional Sofa Couch for Garden Home Bedroom Studio Versatile Arrangement Spacious Design Fresh Natural Great for Lounging Lounge Space Organic Design Green</t>
         </is>
       </c>
     </row>
@@ -2817,7 +2817,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
+          <t>KEIKI 2Seat+Ott1 Modular Boneless Sectional Sofa Couch for Garden Home Home Office Customizable Setup Comfy Support Fresh Natural Designed for Comfort Lounge Space Organic Design Green</t>
         </is>
       </c>
     </row>
@@ -2857,7 +2857,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Sofa Couch for Garden Home Apartment Living Flexible Layout Deep Seat Fresh Natural Perfect for Relaxing Lounge Space Organic Design High Quality Comfort...</t>
         </is>
       </c>
     </row>
@@ -2897,7 +2897,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
+          <t>KEIKI 4Seat+Ott2 Modular Boneless Sectional Sofa Couch for Contemporary Home Small Space Adjustable Configuration Plush Cushions Comfortable Inviting Ideal for Entertaining Lounge Space Modern...</t>
         </is>
       </c>
     </row>
@@ -2937,7 +2937,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
+          <t>KEIKI 4Seat+Ott1 Modular Boneless Sectional Sofa Couch for Contemporary Home Bedroom Studio Versatile Arrangement Spacious Design Comfortable Inviting Great for Lounging Lounge Space Modern De...</t>
         </is>
       </c>
     </row>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly...</t>
+          <t>KEIKI 4Seat Modular Boneless Sectional Sofa Couch for Contemporary Home Home Office Customizable Setup Comfy Support Comfortable Inviting Designed for Comfort Lounge Space Modern Design Cream</t>
         </is>
       </c>
     </row>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
+          <t>KEIKI 3Seat+Ott2 Modular Boneless Sectional Sofa Couch for Contemporary Home Apartment Living Flexible Layout Deep Seat Comfortable Inviting Perfect for Relaxing Lounge Space Modern Design Cream</t>
         </is>
       </c>
     </row>
@@ -3057,7 +3057,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
+          <t>KEIKI 3Seat+Ott1 Modular Boneless Sectional Sofa Couch for Contemporary Home Small Space Adjustable Configuration Plush Cushions Comfortable Inviting Ideal for Entertaining Lounge Space Modern...</t>
         </is>
       </c>
     </row>
@@ -3097,7 +3097,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly...</t>
+          <t>KEIKI 3Seat Modular Boneless Sectional Sofa Couch for Contemporary Home Bedroom Studio Versatile Arrangement Spacious Design Comfortable Inviting Great for Lounging Lounge Space Modern Design ...</t>
         </is>
       </c>
     </row>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
+          <t>KEIKI 2Seat+Ott1 Modular Boneless Sectional Sofa Couch for Contemporary Home Home Office Customizable Setup Comfy Support Comfortable Inviting Designed for Comfort Lounge Space Modern Design C...</t>
         </is>
       </c>
     </row>
@@ -3177,7 +3177,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Sofa Couch for Contemporary Home Apartment Living Flexible Layout Deep Seat Comfortable Inviting Perfect for Relaxing Lounge Space Modern Design Cream</t>
         </is>
       </c>
     </row>
@@ -3217,7 +3217,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
+          <t>KEIKI 4Seat+Ott2 Modular Boneless Sectional Sofa Couch for California Casual Small Space Adjustable Configuration Plush Cushions Sunny Relaxed Ideal for Entertaining Lounge Space Coastal Desig...</t>
         </is>
       </c>
     </row>
@@ -3257,7 +3257,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly...</t>
+          <t>KEIKI 4Seat Modular Boneless Sectional Sofa Couch for California Casual Bedroom Studio Versatile Arrangement Spacious Design Sunny Relaxed Great for Lounging Lounge Space Coastal Design Light ...</t>
         </is>
       </c>
     </row>
@@ -3297,7 +3297,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
+          <t>KEIKI 3Seat+Ott2 Modular Boneless Sectional Sofa Couch for California Casual Home Office Customizable Setup Comfy Support Sunny Relaxed Designed for Comfort Lounge Space Coastal Design Light C...</t>
         </is>
       </c>
     </row>
@@ -3337,7 +3337,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
+          <t>KEIKI 3Seat+Ott1 Modular Boneless Sectional Sofa Couch for California Casual Apartment Living Flexible Layout Deep Seat Sunny Relaxed Perfect for Relaxing Lounge Space Coastal Design Light Camel</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly...</t>
+          <t>KEIKI 3Seat Modular Boneless Sectional Sofa Couch for California Casual Small Space Adjustable Configuration Plush Cushions Sunny Relaxed Ideal for Entertaining Lounge Space Coastal Design Lig...</t>
         </is>
       </c>
     </row>
@@ -3417,7 +3417,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Ass...</t>
+          <t>KEIKI 2Seat+Ott1 Modular Boneless Sectional Sofa Couch for California Casual Bedroom Studio Versatile Arrangement Spacious Design Sunny Relaxed Great for Lounging Lounge Space Coastal Design L...</t>
         </is>
       </c>
     </row>
@@ -3457,7 +3457,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Sectional Sofa Couch for Living Room Apartment Small Space Flexible Layout Deep Seat Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Sofa Couch for California Casual Home Office Customizable Setup Comfy Support Sunny Relaxed Designed for Comfort Lounge Space Coastal Design Light Camel</t>
         </is>
       </c>
     </row>
@@ -3495,7 +3495,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 77.2" Modular Boneless Sectional Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy ...</t>
+          <t>KEIKI Full Chaise 77.2" Modular Boneless Sectional Sofa Couch with Chaise for Urban Loft Apartment Living Flexible Layout Deep Seat Sleek Bold Perfect for Relaxing Lounge Space Contemporary De...</t>
         </is>
       </c>
     </row>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 135" Modular Boneless Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern D...</t>
+          <t>KEIKI Full Chaise 135" Modular Boneless Sectional Sofa Couch for Urban Loft Small Space Adjustable Configuration Plush Cushions Sleek Bold Ideal for Entertaining Lounge Space Contemporary Desi...</t>
         </is>
       </c>
     </row>
@@ -3571,7 +3571,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy A...</t>
+          <t>KEIKI Left Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Urban Loft Bedroom Studio Versatile Arrangement Spacious Design Sleek Bold Great for Lounging Lounge Space Contempo...</t>
         </is>
       </c>
     </row>
@@ -3609,7 +3609,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy ...</t>
+          <t>KEIKI Right Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Urban Loft Home Office Customizable Setup Comfy Support Sleek Bold Designed for Comfort Lounge Space Contemporary ...</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3647,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 77.2" Modular Boneless Sectional Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy ...</t>
+          <t>KEIKI Full Chaise 77.2" Modular Boneless Sectional Sofa Couch with Chaise for Garden Home Apartment Living Flexible Layout Deep Seat Fresh Natural Perfect for Relaxing Lounge Space Organic Des...</t>
         </is>
       </c>
     </row>
@@ -3685,7 +3685,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 135" Modular Boneless Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern D...</t>
+          <t>KEIKI Full Chaise 135" Modular Boneless Sectional Sofa Couch for Garden Home Small Space Adjustable Configuration Plush Cushions Fresh Natural Ideal for Entertaining Lounge Space Organic Desig...</t>
         </is>
       </c>
     </row>
@@ -3723,7 +3723,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy A...</t>
+          <t>KEIKI Left Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Garden Home Bedroom Studio Versatile Arrangement Spacious Design Fresh Natural Great for Lounging Lounge Space Orga...</t>
         </is>
       </c>
     </row>
@@ -3761,7 +3761,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy ...</t>
+          <t>KEIKI Right Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Garden Home Home Office Customizable Setup Comfy Support Fresh Natural Designed for Comfort Lounge Space Organic D...</t>
         </is>
       </c>
     </row>
@@ -3799,7 +3799,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 77.2" Modular Boneless Sectional Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy ...</t>
+          <t>KEIKI Full Chaise 77.2" Modular Boneless Sectional Sofa Couch with Chaise for Contemporary Home Apartment Living Flexible Layout Deep Seat Comfortable Inviting Perfect for Relaxing Lounge Spac...</t>
         </is>
       </c>
     </row>
@@ -3837,7 +3837,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 135" Modular Boneless Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern D...</t>
+          <t>KEIKI Full Chaise 135" Modular Boneless Sectional Sofa Couch for Contemporary Home Small Space Adjustable Configuration Plush Cushions Comfortable Inviting Ideal for Entertaining Lounge Space ...</t>
         </is>
       </c>
     </row>
@@ -3875,7 +3875,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy A...</t>
+          <t>KEIKI Left Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Contemporary Home Bedroom Studio Versatile Arrangement Spacious Design Comfortable Inviting Great for Lounging Loun...</t>
         </is>
       </c>
     </row>
@@ -3913,7 +3913,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy ...</t>
+          <t>KEIKI Right Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Contemporary Home Home Office Customizable Setup Comfy Support Comfortable Inviting Designed for Comfort Lounge Sp...</t>
         </is>
       </c>
     </row>
@@ -3951,7 +3951,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 77.2" Modular Boneless Sectional Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy ...</t>
+          <t>KEIKI Full Chaise 77.2" Modular Boneless Sectional Sofa Couch with Chaise for Modern Home Apartment Living Flexible Layout Deep Seat Clean Bright Perfect for Relaxing Lounge Space Minimalist D...</t>
         </is>
       </c>
     </row>
@@ -3989,7 +3989,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 135" Modular Boneless Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Comfy Lounge Seating Perfect for Relaxing Easy Assembly Modern D...</t>
+          <t>KEIKI Full Chaise 135" Modular Boneless Sectional Sofa Couch for Modern Home Small Space Adjustable Configuration Plush Cushions Clean Bright Ideal for Entertaining Lounge Space Minimalist Des...</t>
         </is>
       </c>
     </row>
@@ -4027,7 +4027,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy A...</t>
+          <t>KEIKI Left Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Modern Home Bedroom Studio Versatile Arrangement Spacious Design Clean Bright Great for Lounging Lounge Space Minim...</t>
         </is>
       </c>
     </row>
@@ -4065,7 +4065,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy ...</t>
+          <t>KEIKI Right Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Modern Home Home Office Customizable Setup Comfy Support Clean Bright Designed for Comfort Lounge Space Minimalist...</t>
         </is>
       </c>
     </row>
@@ -4099,7 +4099,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>KEIKI Sofa Couch for Living Room Bedroom Apartment Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design High Density Foam Cushions Resilience ...</t>
+          <t>KEIKI Sofa Couch for Urban Loft Apartment Living Flexible Layout Deep Seat Sleek Bold Perfect for Relaxing Lounge Space Contemporary Design High Quality Comfortable Supportive Elegant Black</t>
         </is>
       </c>
     </row>
@@ -4133,7 +4133,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>KEIKI Sofa Couch for Living Room Bedroom Apartment Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design High Density Foam Cushions Resilience ...</t>
+          <t>KEIKI Sofa Couch for City Apartment Small Space Adjustable Configuration Plush Cushions Neutral Calm Ideal for Entertaining Lounge Space Modern Design High Quality Comfortable Supportive Elega...</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>KEIKI Sofa Couch for Living Room Bedroom Apartment Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design High Density Foam Cushions Resilience ...</t>
+          <t>KEIKI Sofa Couch for Cozy Cottage Bedroom Studio Versatile Arrangement Spacious Design Warm Inviting Great for Lounging Lounge Space Traditional Design High Quality Comfortable Supportive Eleg...</t>
         </is>
       </c>
     </row>
@@ -4204,7 +4204,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Sectional Sofa Couch Memory Foam for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern...</t>
+          <t>KEIKI Left Chaise Modular Sectional Sofa Couch Memory Foam for Contemporary Home Home Office Customizable Setup Comfy Support Comfortable Inviting Designed for Comfort Lounge Space Modern Desi...</t>
         </is>
       </c>
     </row>
@@ -4241,7 +4241,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Sectional Sofa Couch Memory Foam for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern...</t>
+          <t>KEIKI Left Chaise Modular Sectional Sofa Couch Memory Foam for Garden Home Apartment Living Flexible Layout Deep Seat Fresh Natural Perfect for Relaxing Lounge Space Organic Design Green</t>
         </is>
       </c>
     </row>
@@ -4278,7 +4278,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Sectional Sofa Couch Memory Foam for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern...</t>
+          <t>KEIKI Left Chaise Modular Sectional Sofa Couch Memory Foam for Modern Home Small Space Adjustable Configuration Plush Cushions Clean Bright Ideal for Entertaining Lounge Space Minimalist Desig...</t>
         </is>
       </c>
     </row>
@@ -4315,7 +4315,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Sectional Sofa Couch Memory Foam for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern...</t>
+          <t>KEIKI Left Chaise Modular Sectional Sofa Couch Memory Foam for Urban Loft Bedroom Studio Versatile Arrangement Spacious Design Sleek Bold Great for Lounging Lounge Space Contemporary Design Black</t>
         </is>
       </c>
     </row>
@@ -4352,7 +4352,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Sectional Sofa Couch Memory Foam for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
+          <t>KEIKI Right Chaise Modular Sectional Sofa Couch Memory Foam for Contemporary Home Home Office Customizable Setup Comfy Support Comfortable Inviting Designed for Comfort Lounge Space Modern Des...</t>
         </is>
       </c>
     </row>
@@ -4389,7 +4389,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Sectional Sofa Couch Memory Foam for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
+          <t>KEIKI Right Chaise Modular Sectional Sofa Couch Memory Foam for Garden Home Apartment Living Flexible Layout Deep Seat Fresh Natural Perfect for Relaxing Lounge Space Organic Design Green</t>
         </is>
       </c>
     </row>
@@ -4426,7 +4426,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Sectional Sofa Couch Memory Foam for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
+          <t>KEIKI Right Chaise Modular Sectional Sofa Couch Memory Foam for Modern Home Small Space Adjustable Configuration Plush Cushions Clean Bright Ideal for Entertaining Lounge Space Minimalist Desi...</t>
         </is>
       </c>
     </row>
@@ -4463,7 +4463,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Sectional Sofa Couch Memory Foam for Living Room Home Office Flexible Layout Deep Seat Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
+          <t>KEIKI Right Chaise Modular Sectional Sofa Couch Memory Foam for Urban Loft Bedroom Studio Versatile Arrangement Spacious Design Sleek Bold Great for Lounging Lounge Space Contemporary Design B...</t>
         </is>
       </c>
     </row>
@@ -4500,7 +4500,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Turtle Velvet Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Mo...</t>
+          <t>KEIKI Left Chaise Modular Turtle Velvet Sofa Couch with Chaise for Garden Home Home Office Customizable Setup Fresh Natural Designed for Comfort Lounge Space Organic Design High Quality Comfor...</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4537,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Turtle Velvet Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly M...</t>
+          <t>KEIKI Right Chaise Modular Turtle Velvet Sofa Couch with Chaise for Garden Home Apartment Living Flexible Layout Fresh Natural Perfect for Relaxing Lounge Space Organic Design Green</t>
         </is>
       </c>
     </row>
@@ -4574,7 +4574,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Turtle Velvet Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Mo...</t>
+          <t>KEIKI Left Chaise Modular Turtle Velvet Sofa Couch with Chaise for Modern Home Small Space Adjustable Configuration Clean Bright Ideal for Entertaining Lounge Space Minimalist Design White</t>
         </is>
       </c>
     </row>
@@ -4611,7 +4611,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Turtle Velvet Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly M...</t>
+          <t>KEIKI Right Chaise Modular Turtle Velvet Sofa Couch with Chaise for Modern Home Bedroom Studio Versatile Arrangement Clean Bright Great for Lounging Lounge Space Minimalist Design White</t>
         </is>
       </c>
     </row>
@@ -4648,7 +4648,7 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Turtle Velvet Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Mo...</t>
+          <t>KEIKI Left Chaise Modular Turtle Velvet Sofa Couch with Chaise for Urban Loft Home Office Customizable Setup Sleek Bold Designed for Comfort Lounge Space Contemporary Design High Quality Comfo...</t>
         </is>
       </c>
     </row>
@@ -4685,7 +4685,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Turtle Velvet Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly M...</t>
+          <t>KEIKI Right Chaise Modular Turtle Velvet Sofa Couch with Chaise for Urban Loft Apartment Living Flexible Layout Sleek Bold Perfect for Relaxing Lounge Space Contemporary Design Black</t>
         </is>
       </c>
     </row>
@@ -4722,7 +4722,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Turtle Velvet Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Mo...</t>
+          <t>KEIKI Left Chaise Modular Turtle Velvet Sofa Couch with Chaise for Feminine Retreat Small Space Adjustable Configuration Romantic Dreamy Ideal for Entertaining Lounge Space Glam Design Pink</t>
         </is>
       </c>
     </row>
@@ -4759,7 +4759,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Turtle Velvet Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly M...</t>
+          <t>KEIKI Right Chaise Modular Turtle Velvet Sofa Couch with Chaise for Feminine Retreat Bedroom Studio Versatile Arrangement Romantic Dreamy Great for Lounging Lounge Space Glam Design Pink</t>
         </is>
       </c>
     </row>
@@ -4815,7 +4815,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat Modular Boneless Sectional Loveseat Sofa Couch for Living Room Bedroom Apartment Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern ...</t>
+          <t>KEIKI Loveseat Modular Boneless Sectional Loveseat Sofa Couch for Contemporary Home Home Office Customizable Setup Comfortable Inviting Designed for Comfort Lounge Space Modern Design Light Grey</t>
         </is>
       </c>
     </row>
@@ -4871,7 +4871,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat Modular Boneless Sectional Loveseat Sofa Couch for Living Room Bedroom Apartment Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern ...</t>
+          <t>KEIKI Loveseat Modular Boneless Sectional Loveseat Sofa Couch for Contemporary Home Apartment Living Flexible Layout Comfortable Inviting Perfect for Relaxing Lounge Space Modern Design Dark Grey</t>
         </is>
       </c>
     </row>
@@ -4927,7 +4927,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat Modular Boneless Sectional Loveseat Sofa Couch for Living Room Bedroom Apartment Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern ...</t>
+          <t>KEIKI Loveseat Modular Boneless Sectional Loveseat Sofa Couch for Creative Studio Small Space Adjustable Configuration Energetic Vibrant Ideal for Entertaining Lounge Space Eclectic Design Orange</t>
         </is>
       </c>
     </row>
@@ -4983,7 +4983,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat Modular Boneless Sectional Loveseat Sofa Couch for Living Room Bedroom Apartment Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern ...</t>
+          <t>KEIKI Loveseat Modular Boneless Sectional Loveseat Sofa Couch for Modern Home Bedroom Studio Versatile Arrangement Clean Bright Great for Lounging Lounge Space Minimalist Design White</t>
         </is>
       </c>
     </row>
@@ -5027,7 +5027,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>KEIKI 2 seat Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Dark ...</t>
+          <t>KEIKI 2 seat Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Home Office Customizable Setup Comfortable Inviting Designed for Comfort Lounge Space Modern Design Dark Grey</t>
         </is>
       </c>
     </row>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>KEIKI 2 seat Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Light...</t>
+          <t>KEIKI 2 seat Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Apartment Living Flexible Layout Comfortable Inviting Perfect for Relaxing Lounge Space Modern Design Light Grey</t>
         </is>
       </c>
     </row>
@@ -5115,7 +5115,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>KEIKI 2 seat Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design White</t>
+          <t>KEIKI 2 seat Modular Sofa Couch with Chaise Memory Foam for Modern Home Small Space Adjustable Configuration Clean Bright Ideal for Entertaining Lounge Space Minimalist Design White</t>
         </is>
       </c>
     </row>
@@ -5159,7 +5159,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>KEIKI 2 seat Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Orange</t>
+          <t>KEIKI 2 seat Modular Sofa Couch with Chaise Memory Foam for Creative Studio Bedroom Studio Versatile Arrangement Energetic Vibrant Great for Lounging Lounge Space Eclectic Design Orange</t>
         </is>
       </c>
     </row>
@@ -5203,7 +5203,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>KEIKI 1 seater and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Mod...</t>
+          <t>KEIKI 1 seater and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Home Office Customizable Setup Comfortable Inviting Designed for Comfort Lounge Space Modern Desig...</t>
         </is>
       </c>
     </row>
@@ -5247,7 +5247,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>KEIKI 1 seater and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Mod...</t>
+          <t>KEIKI 1 seater and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Apartment Living Flexible Layout Comfortable Inviting Perfect for Relaxing Lounge Space Modern Des...</t>
         </is>
       </c>
     </row>
@@ -5291,7 +5291,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>KEIKI 1 seater and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Mod...</t>
+          <t>KEIKI 1 seater and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Modern Home Small Space Adjustable Configuration Clean Bright Ideal for Entertaining Lounge Space Minimalist Design ...</t>
         </is>
       </c>
     </row>
@@ -5335,7 +5335,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>KEIKI 1 seater and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Mod...</t>
+          <t>KEIKI 1 seater and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Creative Studio Bedroom Studio Versatile Arrangement Energetic Vibrant Great for Lounging Lounge Space Eclectic Desi...</t>
         </is>
       </c>
     </row>
@@ -5379,7 +5379,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 2 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
+          <t>KEIKI 4 seat and 2 Ottoman Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Home Office Customizable Setup Comfortable Inviting Designed for Comfort Lounge Space Modern Design ...</t>
         </is>
       </c>
     </row>
@@ -5423,7 +5423,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 2 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
+          <t>KEIKI 4 seat and 2 Ottoman Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Apartment Living Flexible Layout Comfortable Inviting Perfect for Relaxing Lounge Space Modern Desig...</t>
         </is>
       </c>
     </row>
@@ -5467,7 +5467,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 2 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
+          <t>KEIKI 4 seat and 2 Ottoman Modular Sofa Couch with Chaise Memory Foam for Modern Home Small Space Adjustable Configuration Clean Bright Ideal for Entertaining Lounge Space Minimalist Design White</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 2 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
+          <t>KEIKI 4 seat and 2 Ottoman Modular Sofa Couch with Chaise Memory Foam for Creative Studio Bedroom Studio Versatile Arrangement Energetic Vibrant Great for Lounging Lounge Space Eclectic Design...</t>
         </is>
       </c>
     </row>
@@ -5555,7 +5555,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
+          <t>KEIKI 4 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Home Office Customizable Setup Comfortable Inviting Designed for Comfort Lounge Space Modern Design ...</t>
         </is>
       </c>
     </row>
@@ -5599,7 +5599,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
+          <t>KEIKI 4 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Apartment Living Flexible Layout Comfortable Inviting Perfect for Relaxing Lounge Space Modern Desig...</t>
         </is>
       </c>
     </row>
@@ -5643,7 +5643,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
+          <t>KEIKI 4 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Modern Home Small Space Adjustable Configuration Clean Bright Ideal for Entertaining Lounge Space Minimalist Design White</t>
         </is>
       </c>
     </row>
@@ -5687,7 +5687,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
+          <t>KEIKI 4 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Creative Studio Bedroom Studio Versatile Arrangement Energetic Vibrant Great for Lounging Lounge Space Eclectic Design...</t>
         </is>
       </c>
     </row>
@@ -5731,7 +5731,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Dark ...</t>
+          <t>KEIKI 4 seat Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Home Office Customizable Setup Comfortable Inviting Designed for Comfort Lounge Space Modern Design Dark Grey</t>
         </is>
       </c>
     </row>
@@ -5775,7 +5775,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Light...</t>
+          <t>KEIKI 4 seat Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Apartment Living Flexible Layout Comfortable Inviting Perfect for Relaxing Lounge Space Modern Design Light Grey</t>
         </is>
       </c>
     </row>
@@ -5819,7 +5819,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design White</t>
+          <t>KEIKI 4 seat Modular Sofa Couch with Chaise Memory Foam for Modern Home Small Space Adjustable Configuration Clean Bright Ideal for Entertaining Lounge Space Minimalist Design White</t>
         </is>
       </c>
     </row>
@@ -5863,7 +5863,7 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Orange</t>
+          <t>KEIKI 4 seat Modular Sofa Couch with Chaise Memory Foam for Creative Studio Bedroom Studio Versatile Arrangement Energetic Vibrant Great for Lounging Lounge Space Eclectic Design Orange</t>
         </is>
       </c>
     </row>
@@ -5907,7 +5907,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Mod...</t>
+          <t>KEIKI Loveseat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Home Office Customizable Setup Comfortable Inviting Designed for Comfort Lounge Space Modern Desig...</t>
         </is>
       </c>
     </row>
@@ -5951,7 +5951,7 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Mod...</t>
+          <t>KEIKI Loveseat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Apartment Living Flexible Layout Comfortable Inviting Perfect for Relaxing Lounge Space Modern Des...</t>
         </is>
       </c>
     </row>
@@ -5995,7 +5995,7 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Mod...</t>
+          <t>KEIKI Loveseat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Modern Home Small Space Adjustable Configuration Clean Bright Ideal for Entertaining Lounge Space Minimalist Design ...</t>
         </is>
       </c>
     </row>
@@ -6039,7 +6039,7 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Mod...</t>
+          <t>KEIKI Loveseat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Creative Studio Bedroom Studio Versatile Arrangement Energetic Vibrant Great for Lounging Lounge Space Eclectic Desi...</t>
         </is>
       </c>
     </row>
@@ -6083,7 +6083,7 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
+          <t>KEIKI 3 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Home Office Customizable Setup Comfortable Inviting Designed for Comfort Lounge Space Modern Design ...</t>
         </is>
       </c>
     </row>
@@ -6127,7 +6127,7 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
+          <t>KEIKI 3 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Apartment Living Flexible Layout Comfortable Inviting Perfect for Relaxing Lounge Space Modern Desig...</t>
         </is>
       </c>
     </row>
@@ -6171,7 +6171,7 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
+          <t>KEIKI 3 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Modern Home Small Space Adjustable Configuration Clean Bright Ideal for Entertaining Lounge Space Minimalist Design White</t>
         </is>
       </c>
     </row>
@@ -6215,7 +6215,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Moder...</t>
+          <t>KEIKI 3 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Creative Studio Bedroom Studio Versatile Arrangement Energetic Vibrant Great for Lounging Lounge Space Eclectic Design...</t>
         </is>
       </c>
     </row>
@@ -6259,7 +6259,7 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Dark ...</t>
+          <t>KEIKI 3 seat Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Home Office Customizable Setup Comfortable Inviting Designed for Comfort Lounge Space Modern Design Dark Grey</t>
         </is>
       </c>
     </row>
@@ -6303,7 +6303,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Light...</t>
+          <t>KEIKI 3 seat Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Apartment Living Flexible Layout Comfortable Inviting Perfect for Relaxing Lounge Space Modern Design Light Grey</t>
         </is>
       </c>
     </row>
@@ -6347,7 +6347,7 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design White</t>
+          <t>KEIKI 3 seat Modular Sofa Couch with Chaise Memory Foam for Modern Home Small Space Adjustable Configuration Clean Bright Ideal for Entertaining Lounge Space Minimalist Design White</t>
         </is>
       </c>
     </row>
@@ -6391,7 +6391,7 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat Modular Sofa Couch with Chaise Memory Foam for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly Modern Design Orange</t>
+          <t>KEIKI 3 seat Modular Sofa Couch with Chaise Memory Foam for Creative Studio Bedroom Studio Versatile Arrangement Energetic Vibrant Great for Lounging Lounge Space Eclectic Design Orange</t>
         </is>
       </c>
     </row>
@@ -6431,7 +6431,7 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Sectional Corduroy Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly ...</t>
+          <t>KEIKI Modular Boneless Sectional Corduroy Sofa Couch with Chaise for Contemporary Home Home Office Customizable Setup Comfy Support Comfortable Inviting Designed for Comfort Lounge Space Moder...</t>
         </is>
       </c>
     </row>
@@ -6471,7 +6471,7 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Sectional Corduroy Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly ...</t>
+          <t>KEIKI Modular Boneless Sectional Corduroy Sofa Couch with Chaise for Contemporary Home Apartment Living Flexible Layout Deep Seat Comfortable Inviting Perfect for Relaxing Lounge Space Modern ...</t>
         </is>
       </c>
     </row>
@@ -6511,7 +6511,7 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Sectional Corduroy Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly ...</t>
+          <t>KEIKI Modular Boneless Sectional Corduroy Sofa Couch with Chaise for City Apartment Small Space Adjustable Configuration Plush Cushions Neutral Calm Ideal for Entertaining Lounge Space Modern ...</t>
         </is>
       </c>
     </row>
@@ -6551,7 +6551,7 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Sectional Corduroy Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly ...</t>
+          <t>KEIKI Modular Boneless Sectional Corduroy Sofa Couch with Chaise for Urban Loft Bedroom Studio Versatile Arrangement Spacious Design Sleek Bold Great for Lounging Lounge Space Contemporary Des...</t>
         </is>
       </c>
     </row>
@@ -6591,7 +6591,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Sectional Corduroy Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly ...</t>
+          <t>KEIKI Modular Boneless Sectional Corduroy Sofa Couch with Chaise for Urban Loft Home Office Customizable Setup Comfy Support Sleek Bold Designed for Comfort Lounge Space Contemporary Design Black</t>
         </is>
       </c>
     </row>
@@ -6631,7 +6631,7 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Sectional Corduroy Sofa Couch with Chaise for Living Room Apartment Small Space Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Easy Assembly ...</t>
+          <t>KEIKI Modular Boneless Sectional Corduroy Sofa Couch with Chaise for City Apartment Apartment Living Flexible Layout Deep Seat Neutral Calm Perfect for Relaxing Lounge Space Modern Design Grey</t>
         </is>
       </c>
     </row>
@@ -6676,7 +6676,7 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>KEIKI 4 Seat Modular Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Oversized Easy Assembly Modern Design Black</t>
+          <t>KEIKI 4 Seat Modular Sectional Sofa Couch for Urban Loft Small Space Adjustable Configuration Plush Cushions Sleek Bold Ideal for Entertaining Lounge Space Contemporary Design Black</t>
         </is>
       </c>
     </row>
@@ -6721,7 +6721,7 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>KEIKI 3 Seat Modular Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Oversized Easy Assembly Modern Design Black</t>
+          <t>KEIKI 3 Seat Modular Sectional Sofa Couch for Urban Loft Bedroom Studio Versatile Arrangement Spacious Design Sleek Bold Great for Lounging Lounge Space Contemporary Design High Quality Comfor...</t>
         </is>
       </c>
     </row>
@@ -6766,7 +6766,7 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>KEIKI 2 Seat Modular Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Oversized Easy Assembly Modern Design Black</t>
+          <t>KEIKI 2 Seat Modular Sectional Sofa Couch for Urban Loft Home Office Customizable Setup Comfy Support Sleek Bold Designed for Comfort Lounge Space Contemporary Design High Quality Comfortable ...</t>
         </is>
       </c>
     </row>
@@ -6811,7 +6811,7 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>KEIKI 4 Seat Modular Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Oversized Easy Assembly Modern Design Creamy White</t>
+          <t>KEIKI 4 Seat Modular Sectional Sofa Couch for Contemporary Home Apartment Living Flexible Layout Deep Seat Comfortable Inviting Perfect for Relaxing Lounge Space Modern Design Creamy White</t>
         </is>
       </c>
     </row>
@@ -6856,7 +6856,7 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>KEIKI 3 Seat Modular Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Oversized Easy Assembly Modern Design Creamy White</t>
+          <t>KEIKI 3 Seat Modular Sectional Sofa Couch for Contemporary Home Small Space Adjustable Configuration Plush Cushions Comfortable Inviting Ideal for Entertaining Lounge Space Modern Design Cream...</t>
         </is>
       </c>
     </row>
@@ -6901,7 +6901,7 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>KEIKI 2 Seat Modular Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Oversized Easy Assembly Modern Design Creamy White</t>
+          <t>KEIKI 2 Seat Modular Sectional Sofa Couch for Contemporary Home Bedroom Studio Versatile Arrangement Spacious Design Comfortable Inviting Great for Lounging Lounge Space Modern Design Creamy W...</t>
         </is>
       </c>
     </row>
@@ -6946,7 +6946,7 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>KEIKI 4 Seat Modular Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Oversized Easy Assembly Modern Design Grey</t>
+          <t>KEIKI 4 Seat Modular Sectional Sofa Couch for City Apartment Home Office Customizable Setup Comfy Support Neutral Calm Designed for Comfort Lounge Space Modern Design High Quality Comfortable ...</t>
         </is>
       </c>
     </row>
@@ -6991,7 +6991,7 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>KEIKI 3 Seat Modular Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Oversized Easy Assembly Modern Design Grey</t>
+          <t>KEIKI 3 Seat Modular Sectional Sofa Couch for City Apartment Apartment Living Flexible Layout Deep Seat Neutral Calm Perfect for Relaxing Lounge Space Modern Design High Quality Comfortable Su...</t>
         </is>
       </c>
     </row>
@@ -7036,7 +7036,7 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>KEIKI 2 Seat Modular Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Oversized Easy Assembly Modern Design Grey</t>
+          <t>KEIKI 2 Seat Modular Sectional Sofa Couch for City Apartment Small Space Adjustable Configuration Plush Cushions Neutral Calm Ideal for Entertaining Lounge Space Modern Design Grey</t>
         </is>
       </c>
     </row>
@@ -7081,7 +7081,7 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>KEIKI 1 Seat Modular Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Oversized Easy Assembly Modern Design Grey</t>
+          <t>KEIKI 1 Seat Modular Sectional Sofa Couch for City Apartment Bedroom Studio Versatile Arrangement Spacious Design Neutral Calm Great for Lounging Lounge Space Modern Design High Quality Comfor...</t>
         </is>
       </c>
     </row>
@@ -7126,7 +7126,7 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>KEIKI 1 Seat Modular Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Oversized Easy Assembly Modern Design Creamy White</t>
+          <t>KEIKI 1 Seat Modular Sectional Sofa Couch for Contemporary Home Home Office Customizable Setup Comfy Support Comfortable Inviting Designed for Comfort Lounge Space Modern Design Creamy White</t>
         </is>
       </c>
     </row>
@@ -7171,7 +7171,7 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>KEIKI 1 Seat Modular Sectional Sofa Couch for Living Room Home Office Flexible Layout Soft Plush Comfortable Lounge Seating Perfect for Relaxing Oversized Easy Assembly Modern Design Black</t>
+          <t>KEIKI 1 Seat Modular Sectional Sofa Couch for Urban Loft Apartment Living Flexible Layout Deep Seat Sleek Bold Perfect for Relaxing Lounge Space Contemporary Design High Quality Comfortable Su...</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
final: precise matching of fabric+style+size+color to audience/scene, 180-195 chars
</commit_message>
<xml_diff>
--- a/KEIKI_Boneless_新标题.xlsx
+++ b/KEIKI_Boneless_新标题.xlsx
@@ -486,7 +486,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for California Casual Apartment Living Flexible Layout Deep Seat Sunny Relaxed Perfect for Relaxing Lounge Space Coastal Design Light Camel</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for California Casual Family Living Room Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Perfect for Sunny Relaxed...</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Garden Home Small Space Adjustable Configuration Fresh Natural Ideal for Entertaining Lounge Space Organic Design High Quality Comfortable Supportive...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Garden Oasis Compact Studio Comfort Seekers Plant Parents Adaptable Homeowners Ultra Soft Plush Ideal for Ultra Soft Plush Lounging Co...</t>
         </is>
       </c>
     </row>
@@ -554,7 +554,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Modern Home Bedroom Studio Versatile Arrangement Clean Bright Great for Lounging Lounge Space Minimalist Design High Quality Comfortable Supportive E...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Bright Modern Home Compact Studio Comfort Seekers Minimalists Adaptable Homeowners Ultra Soft Plush Great for Intimate Cozy Corner Con...</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Urban Loft Home Office Customizable Setup Sleek Bold Designed for Comfort Lounge Space Contemporary Design High Quality Comfortable Supportive Elegan...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Industrial Loft Compact Studio Comfort Seekers Urban Professionals Adaptable Homeowners Ultra Soft Plush Designed for Flexible Configu...</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Feminine Retreat Apartment Living Flexible Layout Romantic Dreamy Perfect for Relaxing Lounge Space Glam Design High Quality Comfortable Supportive E...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Feminine Retreat Compact Studio Comfort Seekers Glam Seekers Adaptable Homeowners Ultra Soft Plush Perfect for Romantic Soft Relaxatio...</t>
         </is>
       </c>
     </row>
@@ -656,7 +656,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Contemporary Home Small Space Adjustable Configuration Comfortable Inviting Ideal for Entertaining Lounge Space Modern Design Black Green</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Modern Home Compact Studio Comfort Seekers Homeowners Adaptable Homeowners Ultra Soft Plush Ideal for Ultra Soft Plush Lounging Contem...</t>
         </is>
       </c>
     </row>
@@ -690,7 +690,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Contemporary Home Bedroom Studio Versatile Arrangement Comfortable Inviting Great for Lounging Lounge Space Modern Series High Quality Comfortable Su...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Modern Home Compact Studio Comfort Seekers Homeowners Adaptable Homeowners Ultra Soft Plush Great for Intimate Cozy Corner Contemporar...</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Contemporary Home Home Office Customizable Setup Comfortable Inviting Designed for Comfort Lounge Space Modern Series High Quality Comfortable Suppor...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Modern Home Compact Studio Comfort Seekers Homeowners Adaptable Homeowners Ultra Soft Plush Designed for Flexible Configuration Contem...</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Contemporary Home Apartment Living Flexible Layout Comfortable Inviting Perfect for Relaxing Lounge Space Modern Series High Quality Comfortable Supp...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Modern Home Compact Studio Comfort Seekers Homeowners Adaptable Homeowners Ultra Soft Plush Perfect for Comfortable Relaxation Contemp...</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Contemporary Home Small Space Adjustable Configuration Comfortable Inviting Ideal for Entertaining Lounge Space Modern Series High Quality Comfortabl...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Modern Home Compact Studio Comfort Seekers Homeowners Adaptable Homeowners Ultra Soft Plush Ideal for Ultra Soft Plush Lounging Contem...</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Contemporary Home Bedroom Studio Versatile Arrangement Comfortable Inviting Great for Lounging Lounge Space Modern Series High Quality Co Style 0 Su...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Modern Home Compact Studio Comfort Seekers Homeowners Adaptable Homeowners Ultra Soft Plush Great for Intimate Cozy Corner Contemporar...</t>
         </is>
       </c>
     </row>
@@ -860,7 +860,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Contemporary Home Home Office Customizable Setup Comfortable Inviting Designed for Comfort Lounge Space Modern Series High Quality Comfor Style 1 Sup...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Modern Home Compact Studio Comfort Seekers Homeowners Adaptable Homeowners Ultra Soft Plush Designed for Flexible Configuration Contem...</t>
         </is>
       </c>
     </row>
@@ -894,7 +894,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Contemporary Home Apartment Living Flexible Layout Comfortable Inviting Perfect for Relaxing Lounge Space Modern Series High Quality Comf Style 2 Sup...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Modern Home Compact Studio Comfort Seekers Homeowners Adaptable Homeowners Ultra Soft Plush Perfect for Comfortable Relaxation Contemp...</t>
         </is>
       </c>
     </row>
@@ -928,7 +928,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Contemporary Home Small Space Adjustable Configuration Comfortable Inviting Ideal for Entertaining Lounge Space Modern Design High Quality Comfortabl...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Modern Home Compact Studio Comfort Seekers Homeowners Adaptable Homeowners Ultra Soft Plush Ideal for Ultra Soft Plush Lounging Contem...</t>
         </is>
       </c>
     </row>
@@ -962,7 +962,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Contemporary Home Bedroom Studio Versatile Arrangement Comfortable Inviting Great for Lounging Lounge Space Modern Design High Quality Comfortable Su...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Modern Home Compact Studio Comfort Seekers Homeowners Adaptable Homeowners Ultra Soft Plush Great for Intimate Cozy Corner Contemporar...</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Contemporary Home Home Office Customizable Setup Comfortable Inviting Designed for Comfort Lounge Space Modern Design High Quality Comfortable Suppor...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Modern Home Compact Studio Comfort Seekers Homeowners Adaptable Homeowners Ultra Soft Plush Designed for Flexible Configuration Contem...</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>KEIKI Modular Turtle Velvet Sofa Couch for Contemporary Home Apartment Living Flexible Layout Comfortable Inviting Perfect for Relaxing Lounge Space Modern Design High Quality Comfortable Supp...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Modern Home Compact Studio Comfort Seekers Homeowners Adaptable Homeowners Ultra Soft Plush Perfect for Comfortable Relaxation Contemp...</t>
         </is>
       </c>
     </row>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Rustic Home Small Space Adjustable Configuration Plush Cushions Earthy Classic Ideal for Entertaining Lounge Space Vintage Design Brown</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Rustic Home Small Apartment Style Conscious Nature Lovers Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft Lounging G...</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1104,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Rustic Home Bedroom Studio Versatile Arrangement Spacious Design Earthy Classic Great for Lounging Lounge Space Vintage Design Brown</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Rustic Home Family Living Room Style Conscious Nature Lovers Adaptable Relaxation Seekers Luxuriously Soft Great for Comfortable Gathering Sp...</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Rustic Home Home Office Customizable Setup Comfy Support Earthy Classic Designed for Comfort Lounge Space Vintage Design Brown</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Rustic Home Family Living Room Style Conscious Nature Lovers Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-in Comf...</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Rustic Home Apartment Living Flexible Layout Deep Seat Earthy Classic Perfect for Relaxing Lounge Space Vintage Design High Quality Comfortab...</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Rustic Home Family Living Room Style Conscious Nature Lovers Adaptable Relaxation Seekers Luxuriously Soft Perfect for Grounded Natural Relax...</t>
         </is>
       </c>
     </row>
@@ -1215,7 +1215,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Rustic Home Small Space Adjustable Configuration Plush Cushions Earthy Classic Ideal for Entertaining Lounge Space Vintage Design Brown</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Rustic Home Small Apartment Style Conscious Nature Lovers Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft Lounging G...</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1252,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Rustic Home Bedroom Studio Versatile Arrangement Spacious Design Earthy Classic Great for Lounging Lounge Space Vintage Design Brown</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Rustic Home Small Apartment Style Conscious Nature Lovers Adaptable Relaxation Seekers Luxuriously Soft Great for Functional Relaxation Spot ...</t>
         </is>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Rustic Home Home Office Customizable Setup Comfy Support Earthy Classic Designed for Comfort Lounge Space Vintage Design Brown</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Rustic Home Compact Studio Style Conscious Nature Lovers Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-in...</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Rustic Home Apartment Living Flexible Layout Deep Seat Earthy Classic Perfect for Relaxing Lounge Space Vintage Design High Quality Comfortab...</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Rustic Home Compact Studio Style Conscious Nature Lovers Adaptable Relaxation Seekers Luxuriously Soft Perfect for Grounded Natural ...</t>
         </is>
       </c>
     </row>
@@ -1363,7 +1363,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for California Casual Small Space Adjustable Configuration Plush Cushions Sunny Relaxed Ideal for Entertaining Lounge Space Coastal Design L...</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for California Casual Family Living Room Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Sof...</t>
         </is>
       </c>
     </row>
@@ -1400,7 +1400,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for California Casual Bedroom Studio Versatile Arrangement Spacious Design Sunny Relaxed Great for Lounging Lounge Space Coastal Design Ligh...</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for California Casual Family Living Room Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Great for Comfortable Gat...</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for California Casual Home Office Customizable Setup Comfy Support Sunny Relaxed Designed for Comfort Lounge Space Coastal Design Light Camel</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for California Casual Small Apartment Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-i...</t>
         </is>
       </c>
     </row>
@@ -1474,7 +1474,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for California Casual Apartment Living Flexible Layout Deep Seat Sunny Relaxed Perfect for Relaxing Lounge Space Coastal Design Light Camel</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for California Casual Small Apartment Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Perfect for Sunny Relaxed Re...</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for California Casual Small Space Adjustable Configuration Plush Cushions Sunny Relaxed Ideal for Entertaining Lounge Space Coastal Design Light ...</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for California Casual Small Apartment Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft L...</t>
         </is>
       </c>
     </row>
@@ -1548,7 +1548,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for California Casual Bedroom Studio Versatile Arrangement Spacious Design Sunny Relaxed Great for Lounging Lounge Space Coastal Design Ligh...</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for California Casual Compact Studio Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Great for Intimate C...</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for California Casual Home Office Customizable Setup Comfy Support Sunny Relaxed Designed for Comfort Lounge Space Coastal Design Light Camel</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for California Casual Compact Studio Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexibl...</t>
         </is>
       </c>
     </row>
@@ -1622,7 +1622,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Garden Home Apartment Living Flexible Layout Deep Seat Fresh Natural Perfect for Relaxing Lounge Space Organic Design High Quality Comfo...</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Garden Oasis Family Living Room Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Perfect for Fresh Natural Relaxat...</t>
         </is>
       </c>
     </row>
@@ -1659,7 +1659,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Garden Home Small Space Adjustable Configuration Plush Cushions Fresh Natural Ideal for Entertaining Lounge Space Organic Design Green</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Garden Oasis Family Living Room Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft Loungi...</t>
         </is>
       </c>
     </row>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Garden Home Bedroom Studio Versatile Arrangement Spacious Design Fresh Natural Great for Lounging Lounge Space Organic Design Green</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Garden Oasis Family Living Room Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Great for Comfortable Gathering S...</t>
         </is>
       </c>
     </row>
@@ -1733,7 +1733,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Garden Home Home Office Customizable Setup Comfy Support Fresh Natural Designed for Comfort Lounge Space Organic Design Green</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Garden Oasis Small Apartment Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-in Comfor...</t>
         </is>
       </c>
     </row>
@@ -1770,7 +1770,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Garden Home Apartment Living Flexible Layout Deep Seat Fresh Natural Perfect for Relaxing Lounge Space Organic Design High Quality Comfo...</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Garden Oasis Small Apartment Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Perfect for Fresh Natural Relaxation...</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1807,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Garden Home Small Space Adjustable Configuration Plush Cushions Fresh Natural Ideal for Entertaining Lounge Space Organic Design Green</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Garden Oasis Small Apartment Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft Lounging ...</t>
         </is>
       </c>
     </row>
@@ -1844,7 +1844,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Garden Home Bedroom Studio Versatile Arrangement Spacious Design Fresh Natural Great for Lounging Lounge Space Organic Design Green</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Garden Oasis Compact Studio Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Great for Intimate Cozy Corn...</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Garden Home Home Office Customizable Setup Comfy Support Fresh Natural Designed for Comfort Lounge Space Organic Design High Quality Comforta...</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Garden Oasis Compact Studio Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-i...</t>
         </is>
       </c>
     </row>
@@ -1918,7 +1918,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Velvet Sofa Couch for Contemporary Home Apartment Living Flexible Layout Deep Seat Comfortable Inviting Perfect for Relaxing Lounge Space Modern Design Red</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Modern Home Family Living Room Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Perfect for Comfortable Relaxation Gl...</t>
         </is>
       </c>
     </row>
@@ -1955,7 +1955,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Velvet Sofa Couch for Contemporary Home Small Space Adjustable Configuration Plush Cushions Comfortable Inviting Ideal for Entertaining Lounge Space Modern De...</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Modern Home Family Living Room Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft Lounging G...</t>
         </is>
       </c>
     </row>
@@ -1992,7 +1992,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Contemporary Home Bedroom Studio Versatile Arrangement Spacious Design Comfortable Inviting Great for Lounging Lounge Space Modern Design Red</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Modern Home Family Living Room Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Great for Comfortable Gathering Space...</t>
         </is>
       </c>
     </row>
@@ -2029,7 +2029,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Velvet Sofa Couch for Contemporary Home Home Office Customizable Setup Comfy Support Comfortable Inviting Designed for Comfort Lounge Space Modern Design Red</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Modern Home Small Apartment Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-in Comfort Gl...</t>
         </is>
       </c>
     </row>
@@ -2066,7 +2066,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Velvet Sofa Couch for Contemporary Home Apartment Living Flexible Layout Deep Seat Comfortable Inviting Perfect for Relaxing Lounge Space Modern Design Red</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Modern Home Small Apartment Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Perfect for Comfortable Relaxation Glam ...</t>
         </is>
       </c>
     </row>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Contemporary Home Small Space Adjustable Configuration Plush Cushions Comfortable Inviting Ideal for Entertaining Lounge Space Modern Design Red</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Modern Home Small Apartment Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft Lounging Glam...</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Velvet Sofa Couch for Contemporary Home Bedroom Studio Versatile Arrangement Spacious Design Comfortable Inviting Great for Lounging Lounge Space Modern Desig...</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Modern Home Compact Studio Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Great for Intimate Cozy Corner G...</t>
         </is>
       </c>
     </row>
@@ -2177,7 +2177,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Contemporary Home Home Office Customizable Setup Comfy Support Comfortable Inviting Designed for Comfort Lounge Space Modern Design Red</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Modern Home Compact Studio Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-in Co...</t>
         </is>
       </c>
     </row>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Sectional Sofa Couch for Garden Home Apartment Living Flexible Layout Deep Seat Fresh Natural Perfect for Relaxing Lounge Space Organic Design High Quality Comfort...</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Garden Oasis Small Apartment Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Perfect for Fresh Natural Relaxation...</t>
         </is>
       </c>
     </row>
@@ -2257,7 +2257,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Sectional Sofa Couch for California Casual Small Space Adjustable Configuration Plush Cushions Sunny Relaxed Ideal for Entertaining Lounge Space Coastal Desig...</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for California Casual Family Living Room Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Sof...</t>
         </is>
       </c>
     </row>
@@ -2297,7 +2297,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Sectional Sofa Couch for Urban Loft Bedroom Studio Versatile Arrangement Spacious Design Sleek Bold Great for Lounging Lounge Space Contemporary Design Black</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Industrial Loft Family Living Room Style Conscious Urban Professionals Adaptable Relaxation Seekers Luxuriously Soft Great for Comfortable Ga...</t>
         </is>
       </c>
     </row>
@@ -2337,7 +2337,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Sectional Sofa Couch for Urban Loft Home Office Customizable Setup Comfy Support Sleek Bold Designed for Comfort Lounge Space Contemporary Design Black</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Industrial Loft Family Living Room Style Conscious Urban Professionals Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Si...</t>
         </is>
       </c>
     </row>
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Sectional Sofa Couch for Urban Loft Apartment Living Flexible Layout Deep Seat Sleek Bold Perfect for Relaxing Lounge Space Contemporary Design Black</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Industrial Loft Small Apartment Style Conscious Urban Professionals Adaptable Relaxation Seekers Luxuriously Soft Perfect for Bold Sophistica...</t>
         </is>
       </c>
     </row>
@@ -2417,7 +2417,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Sectional Sofa Couch for Urban Loft Small Space Adjustable Configuration Plush Cushions Sleek Bold Ideal for Entertaining Lounge Space Contemporary Design Black</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Industrial Loft Family Living Room Style Conscious Urban Professionals Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously So...</t>
         </is>
       </c>
     </row>
@@ -2457,7 +2457,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Sectional Sofa Couch for Urban Loft Bedroom Studio Versatile Arrangement Spacious Design Sleek Bold Great for Lounging Lounge Space Contemporary Design Black</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Industrial Loft Small Apartment Style Conscious Urban Professionals Adaptable Relaxation Seekers Luxuriously Soft Great for Functional Relaxa...</t>
         </is>
       </c>
     </row>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Sectional Sofa Couch for Urban Loft Home Office Customizable Setup Comfy Support Sleek Bold Designed for Comfort Lounge Space Contemporary Design Black</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Industrial Loft Small Apartment Style Conscious Urban Professionals Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-...</t>
         </is>
       </c>
     </row>
@@ -2537,7 +2537,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Sectional Sofa Couch for Urban Loft Apartment Living Flexible Layout Deep Seat Sleek Bold Perfect for Relaxing Lounge Space Contemporary Design Black</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Industrial Loft Compact Studio Style Conscious Urban Professionals Adaptable Relaxation Seekers Luxuriously Soft Perfect for Bold So...</t>
         </is>
       </c>
     </row>
@@ -2577,7 +2577,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Sectional Sofa Couch for Urban Loft Small Space Adjustable Configuration Plush Cushions Sleek Bold Ideal for Entertaining Lounge Space Contemporary Design Black</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Industrial Loft Compact Studio Style Conscious Urban Professionals Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxurious...</t>
         </is>
       </c>
     </row>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Sectional Sofa Couch for Garden Home Bedroom Studio Versatile Arrangement Spacious Design Fresh Natural Great for Lounging Lounge Space Organic Design Green</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Garden Oasis Family Living Room Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Great for Comfortable Gathering S...</t>
         </is>
       </c>
     </row>
@@ -2657,7 +2657,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Sectional Sofa Couch for Garden Home Home Office Customizable Setup Comfy Support Fresh Natural Designed for Comfort Lounge Space Organic Design Green</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Garden Oasis Family Living Room Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-in Com...</t>
         </is>
       </c>
     </row>
@@ -2697,7 +2697,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Sectional Sofa Couch for Garden Home Apartment Living Flexible Layout Deep Seat Fresh Natural Perfect for Relaxing Lounge Space Organic Design High Quality Comfort...</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Garden Oasis Family Living Room Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Perfect for Fresh Natural Relaxat...</t>
         </is>
       </c>
     </row>
@@ -2737,7 +2737,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Sectional Sofa Couch for Garden Home Small Space Adjustable Configuration Plush Cushions Fresh Natural Ideal for Entertaining Lounge Space Organic Design Green</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Garden Oasis Small Apartment Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft Lounging ...</t>
         </is>
       </c>
     </row>
@@ -2777,7 +2777,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Sectional Sofa Couch for Garden Home Bedroom Studio Versatile Arrangement Spacious Design Fresh Natural Great for Lounging Lounge Space Organic Design Green</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Garden Oasis Small Apartment Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Great for Functional Relaxation Spot...</t>
         </is>
       </c>
     </row>
@@ -2817,7 +2817,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Sectional Sofa Couch for Garden Home Home Office Customizable Setup Comfy Support Fresh Natural Designed for Comfort Lounge Space Organic Design Green</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Garden Oasis Compact Studio Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-i...</t>
         </is>
       </c>
     </row>
@@ -2857,7 +2857,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Sectional Sofa Couch for Garden Home Apartment Living Flexible Layout Deep Seat Fresh Natural Perfect for Relaxing Lounge Space Organic Design High Quality Comfort...</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Garden Oasis Compact Studio Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Perfect for Fresh Natural Re...</t>
         </is>
       </c>
     </row>
@@ -2897,7 +2897,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Sectional Sofa Couch for Contemporary Home Small Space Adjustable Configuration Plush Cushions Comfortable Inviting Ideal for Entertaining Lounge Space Modern...</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Modern Home Family Living Room Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft Lounging G...</t>
         </is>
       </c>
     </row>
@@ -2937,7 +2937,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott1 Modular Boneless Sectional Sofa Couch for Contemporary Home Bedroom Studio Versatile Arrangement Spacious Design Comfortable Inviting Great for Lounging Lounge Space Modern De...</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Modern Home Family Living Room Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Great for Comfortable Gathering Space...</t>
         </is>
       </c>
     </row>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Sectional Sofa Couch for Contemporary Home Home Office Customizable Setup Comfy Support Comfortable Inviting Designed for Comfort Lounge Space Modern Design Cream</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Modern Home Family Living Room Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-in Comfort...</t>
         </is>
       </c>
     </row>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Sectional Sofa Couch for Contemporary Home Apartment Living Flexible Layout Deep Seat Comfortable Inviting Perfect for Relaxing Lounge Space Modern Design Cream</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Modern Home Small Apartment Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Perfect for Comfortable Relaxation Glam ...</t>
         </is>
       </c>
     </row>
@@ -3057,7 +3057,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Sectional Sofa Couch for Contemporary Home Small Space Adjustable Configuration Plush Cushions Comfortable Inviting Ideal for Entertaining Lounge Space Modern...</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Modern Home Small Apartment Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft Lounging Glam...</t>
         </is>
       </c>
     </row>
@@ -3097,7 +3097,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Sectional Sofa Couch for Contemporary Home Bedroom Studio Versatile Arrangement Spacious Design Comfortable Inviting Great for Lounging Lounge Space Modern Design ...</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Modern Home Small Apartment Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Great for Functional Relaxation Spot Gla...</t>
         </is>
       </c>
     </row>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Sectional Sofa Couch for Contemporary Home Home Office Customizable Setup Comfy Support Comfortable Inviting Designed for Comfort Lounge Space Modern Design C...</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Modern Home Compact Studio Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-in Co...</t>
         </is>
       </c>
     </row>
@@ -3177,7 +3177,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Sectional Sofa Couch for Contemporary Home Apartment Living Flexible Layout Deep Seat Comfortable Inviting Perfect for Relaxing Lounge Space Modern Design Cream</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Modern Home Compact Studio Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Perfect for Comfortable Relaxati...</t>
         </is>
       </c>
     </row>
@@ -3217,7 +3217,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat+Ott2 Modular Boneless Sectional Sofa Couch for California Casual Small Space Adjustable Configuration Plush Cushions Sunny Relaxed Ideal for Entertaining Lounge Space Coastal Desig...</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for California Casual Family Living Room Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Sof...</t>
         </is>
       </c>
     </row>
@@ -3257,7 +3257,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Sectional Sofa Couch for California Casual Bedroom Studio Versatile Arrangement Spacious Design Sunny Relaxed Great for Lounging Lounge Space Coastal Design Light ...</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for California Casual Family Living Room Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Great for Comfortable Gat...</t>
         </is>
       </c>
     </row>
@@ -3297,7 +3297,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott2 Modular Boneless Sectional Sofa Couch for California Casual Home Office Customizable Setup Comfy Support Sunny Relaxed Designed for Comfort Lounge Space Coastal Design Light C...</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for California Casual Small Apartment Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-i...</t>
         </is>
       </c>
     </row>
@@ -3337,7 +3337,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat+Ott1 Modular Boneless Sectional Sofa Couch for California Casual Apartment Living Flexible Layout Deep Seat Sunny Relaxed Perfect for Relaxing Lounge Space Coastal Design Light Camel</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for California Casual Small Apartment Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Perfect for Sunny Relaxed Re...</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Sectional Sofa Couch for California Casual Small Space Adjustable Configuration Plush Cushions Sunny Relaxed Ideal for Entertaining Lounge Space Coastal Design Lig...</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for California Casual Small Apartment Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft L...</t>
         </is>
       </c>
     </row>
@@ -3417,7 +3417,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat+Ott1 Modular Boneless Sectional Sofa Couch for California Casual Bedroom Studio Versatile Arrangement Spacious Design Sunny Relaxed Great for Lounging Lounge Space Coastal Design L...</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for California Casual Compact Studio Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Great for Intimate C...</t>
         </is>
       </c>
     </row>
@@ -3457,7 +3457,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Sectional Sofa Couch for California Casual Home Office Customizable Setup Comfy Support Sunny Relaxed Designed for Comfort Lounge Space Coastal Design Light Camel</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for California Casual Compact Studio Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexibl...</t>
         </is>
       </c>
     </row>
@@ -3495,7 +3495,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 77.2" Modular Boneless Sectional Sofa Couch with Chaise for Urban Loft Apartment Living Flexible Layout Deep Seat Sleek Bold Perfect for Relaxing Lounge Space Contemporary De...</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch with Chaise for Industrial Loft Compact Studio Style Conscious Urban Professionals Adaptable Relaxation Seekers Luxuriously Soft Perfect...</t>
         </is>
       </c>
     </row>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 135" Modular Boneless Sectional Sofa Couch for Urban Loft Small Space Adjustable Configuration Plush Cushions Sleek Bold Ideal for Entertaining Lounge Space Contemporary Desi...</t>
+          <t>KEIKI 5Seat Modular Boneless Velvet Sofa Couch for Industrial Loft Open Concept Living Style Conscious Urban Professionals Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously S...</t>
         </is>
       </c>
     </row>
@@ -3571,7 +3571,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Urban Loft Bedroom Studio Versatile Arrangement Spacious Design Sleek Bold Great for Lounging Lounge Space Contempo...</t>
+          <t>KEIKI 6Seat Modular Boneless Velvet Sofa Couch with Chaise for Industrial Loft Great Room Style Conscious Urban Professionals Adaptable Relaxation Seekers Luxuriously Soft Great for Maximum Se...</t>
         </is>
       </c>
     </row>
@@ -3609,7 +3609,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Urban Loft Home Office Customizable Setup Comfy Support Sleek Bold Designed for Comfort Lounge Space Contemporary ...</t>
+          <t>KEIKI 6Seat Modular Boneless Velvet Sofa Couch with Chaise for Industrial Loft Great Room Style Conscious Urban Professionals Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexibl...</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3647,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 77.2" Modular Boneless Sectional Sofa Couch with Chaise for Garden Home Apartment Living Flexible Layout Deep Seat Fresh Natural Perfect for Relaxing Lounge Space Organic Des...</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch with Chaise for Garden Oasis Compact Studio Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Perfect for Fres...</t>
         </is>
       </c>
     </row>
@@ -3685,7 +3685,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 135" Modular Boneless Sectional Sofa Couch for Garden Home Small Space Adjustable Configuration Plush Cushions Fresh Natural Ideal for Entertaining Lounge Space Organic Desig...</t>
+          <t>KEIKI 5Seat Modular Boneless Velvet Sofa Couch for Garden Oasis Open Concept Living Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft Loung...</t>
         </is>
       </c>
     </row>
@@ -3723,7 +3723,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Garden Home Bedroom Studio Versatile Arrangement Spacious Design Fresh Natural Great for Lounging Lounge Space Orga...</t>
+          <t>KEIKI 6Seat Modular Boneless Velvet Sofa Couch with Chaise for Garden Oasis Great Room Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Great for Maximum Seating Cap...</t>
         </is>
       </c>
     </row>
@@ -3761,7 +3761,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Garden Home Home Office Customizable Setup Comfy Support Fresh Natural Designed for Comfort Lounge Space Organic D...</t>
+          <t>KEIKI 6Seat Modular Boneless Velvet Sofa Couch with Chaise for Garden Oasis Great Room Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-in...</t>
         </is>
       </c>
     </row>
@@ -3799,7 +3799,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 77.2" Modular Boneless Sectional Sofa Couch with Chaise for Contemporary Home Apartment Living Flexible Layout Deep Seat Comfortable Inviting Perfect for Relaxing Lounge Spac...</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch with Chaise for Modern Home Compact Studio Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Perfect for Comforta...</t>
         </is>
       </c>
     </row>
@@ -3837,7 +3837,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 135" Modular Boneless Sectional Sofa Couch for Contemporary Home Small Space Adjustable Configuration Plush Cushions Comfortable Inviting Ideal for Entertaining Lounge Space ...</t>
+          <t>KEIKI 5Seat Modular Boneless Velvet Sofa Couch for Modern Home Open Concept Living Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft Lounging ...</t>
         </is>
       </c>
     </row>
@@ -3875,7 +3875,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Contemporary Home Bedroom Studio Versatile Arrangement Spacious Design Comfortable Inviting Great for Lounging Loun...</t>
+          <t>KEIKI 6Seat Modular Boneless Velvet Sofa Couch with Chaise for Modern Home Great Room Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Great for Maximum Seating Capacit...</t>
         </is>
       </c>
     </row>
@@ -3913,7 +3913,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Contemporary Home Home Office Customizable Setup Comfy Support Comfortable Inviting Designed for Comfort Lounge Sp...</t>
+          <t>KEIKI 6Seat Modular Boneless Velvet Sofa Couch with Chaise for Modern Home Great Room Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-in Com...</t>
         </is>
       </c>
     </row>
@@ -3951,7 +3951,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 77.2" Modular Boneless Sectional Sofa Couch with Chaise for Modern Home Apartment Living Flexible Layout Deep Seat Clean Bright Perfect for Relaxing Lounge Space Minimalist D...</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch with Chaise for Bright Modern Home Compact Studio Style Conscious Minimalists Adaptable Relaxation Seekers Luxuriously Soft Perfect for ...</t>
         </is>
       </c>
     </row>
@@ -3989,7 +3989,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>KEIKI Full Chaise 135" Modular Boneless Sectional Sofa Couch for Modern Home Small Space Adjustable Configuration Plush Cushions Clean Bright Ideal for Entertaining Lounge Space Minimalist Des...</t>
+          <t>KEIKI 5Seat Modular Boneless Velvet Sofa Couch for Bright Modern Home Open Concept Living Style Conscious Minimalists Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft L...</t>
         </is>
       </c>
     </row>
@@ -4027,7 +4027,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Modern Home Bedroom Studio Versatile Arrangement Spacious Design Clean Bright Great for Lounging Lounge Space Minim...</t>
+          <t>KEIKI 6Seat Modular Boneless Velvet Sofa Couch with Chaise for Bright Modern Home Great Room Style Conscious Minimalists Adaptable Relaxation Seekers Luxuriously Soft Great for Maximum Seating...</t>
         </is>
       </c>
     </row>
@@ -4065,7 +4065,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise 106" Modular Boneless Sectional Sofa Couch with Chaise for Modern Home Home Office Customizable Setup Comfy Support Clean Bright Designed for Comfort Lounge Space Minimalist...</t>
+          <t>KEIKI 6Seat Modular Boneless Velvet Sofa Couch with Chaise for Bright Modern Home Great Room Style Conscious Minimalists Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sin...</t>
         </is>
       </c>
     </row>
@@ -4099,7 +4099,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>KEIKI Sofa Couch for Urban Loft Apartment Living Flexible Layout Deep Seat Sleek Bold Perfect for Relaxing Lounge Space Contemporary Design High Quality Comfortable Supportive Elegant Black</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch for Industrial Loft Compact Studio Style Conscious Urban Professionals Practical Buyers Luxuriously Soft Perfect for Bold Sophisticated Relaxatio...</t>
         </is>
       </c>
     </row>
@@ -4133,7 +4133,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>KEIKI Sofa Couch for City Apartment Small Space Adjustable Configuration Plush Cushions Neutral Calm Ideal for Entertaining Lounge Space Modern Design High Quality Comfortable Supportive Elega...</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch for Modern Home Compact Studio Style Conscious Homeowners Practical Buyers Luxuriously Soft Ideal for Luxuriously Soft Lounging Glam Modern Gray</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>KEIKI Sofa Couch for Cozy Cottage Bedroom Studio Versatile Arrangement Spacious Design Warm Inviting Great for Lounging Lounge Space Traditional Design High Quality Comfortable Supportive Eleg...</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch for Cozy Cottage Compact Studio Style Conscious Traditional Families Practical Buyers Luxuriously Soft Great for Intimate Cozy Corner Glam Modern...</t>
         </is>
       </c>
     </row>
@@ -4204,7 +4204,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Sectional Sofa Couch Memory Foam for Contemporary Home Home Office Customizable Setup Comfy Support Comfortable Inviting Designed for Comfort Lounge Space Modern Desi...</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch Memory Foam for Modern Home Compact Studio Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Designed for Flexible Configuration G...</t>
         </is>
       </c>
     </row>
@@ -4241,7 +4241,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Sectional Sofa Couch Memory Foam for Garden Home Apartment Living Flexible Layout Deep Seat Fresh Natural Perfect for Relaxing Lounge Space Organic Design Green</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch Memory Foam for Garden Oasis Compact Studio Style Conscious Plant Parents Adaptable Homeowners Luxuriously Soft Perfect for Fresh Natural Relaxat...</t>
         </is>
       </c>
     </row>
@@ -4278,7 +4278,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Sectional Sofa Couch Memory Foam for Modern Home Small Space Adjustable Configuration Plush Cushions Clean Bright Ideal for Entertaining Lounge Space Minimalist Desig...</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch Memory Foam for Bright Modern Home Compact Studio Style Conscious Minimalists Adaptable Homeowners Luxuriously Soft Ideal for Luxuriously Soft Lo...</t>
         </is>
       </c>
     </row>
@@ -4315,7 +4315,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Sectional Sofa Couch Memory Foam for Urban Loft Bedroom Studio Versatile Arrangement Spacious Design Sleek Bold Great for Lounging Lounge Space Contemporary Design Black</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch Memory Foam for Industrial Loft Compact Studio Style Conscious Urban Professionals Adaptable Homeowners Luxuriously Soft Great for Intimate Cozy ...</t>
         </is>
       </c>
     </row>
@@ -4352,7 +4352,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Sectional Sofa Couch Memory Foam for Contemporary Home Home Office Customizable Setup Comfy Support Comfortable Inviting Designed for Comfort Lounge Space Modern Des...</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch Memory Foam for Modern Home Compact Studio Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Designed for Flexible Configuration G...</t>
         </is>
       </c>
     </row>
@@ -4389,7 +4389,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Sectional Sofa Couch Memory Foam for Garden Home Apartment Living Flexible Layout Deep Seat Fresh Natural Perfect for Relaxing Lounge Space Organic Design Green</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch Memory Foam for Garden Oasis Compact Studio Style Conscious Plant Parents Adaptable Homeowners Luxuriously Soft Perfect for Fresh Natural Relaxat...</t>
         </is>
       </c>
     </row>
@@ -4426,7 +4426,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Sectional Sofa Couch Memory Foam for Modern Home Small Space Adjustable Configuration Plush Cushions Clean Bright Ideal for Entertaining Lounge Space Minimalist Desi...</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch Memory Foam for Bright Modern Home Compact Studio Style Conscious Minimalists Adaptable Homeowners Luxuriously Soft Ideal for Luxuriously Soft Lo...</t>
         </is>
       </c>
     </row>
@@ -4463,7 +4463,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Sectional Sofa Couch Memory Foam for Urban Loft Bedroom Studio Versatile Arrangement Spacious Design Sleek Bold Great for Lounging Lounge Space Contemporary Design B...</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch Memory Foam for Industrial Loft Compact Studio Style Conscious Urban Professionals Adaptable Homeowners Luxuriously Soft Great for Intimate Cozy ...</t>
         </is>
       </c>
     </row>
@@ -4500,7 +4500,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Turtle Velvet Sofa Couch with Chaise for Garden Home Home Office Customizable Setup Fresh Natural Designed for Comfort Lounge Space Organic Design High Quality Comfor...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch with Chaise for Garden Oasis Compact Studio Comfort Seekers Plant Parents Adaptable Homeowners Ultra Soft Plush Designed for Flexible Conf...</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4537,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Turtle Velvet Sofa Couch with Chaise for Garden Home Apartment Living Flexible Layout Fresh Natural Perfect for Relaxing Lounge Space Organic Design Green</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch with Chaise for Garden Oasis Compact Studio Comfort Seekers Plant Parents Adaptable Homeowners Ultra Soft Plush Perfect for Fresh Natural ...</t>
         </is>
       </c>
     </row>
@@ -4574,7 +4574,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Turtle Velvet Sofa Couch with Chaise for Modern Home Small Space Adjustable Configuration Clean Bright Ideal for Entertaining Lounge Space Minimalist Design White</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch with Chaise for Bright Modern Home Compact Studio Comfort Seekers Minimalists Adaptable Homeowners Ultra Soft Plush Ideal for Ultra Soft P...</t>
         </is>
       </c>
     </row>
@@ -4611,7 +4611,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Turtle Velvet Sofa Couch with Chaise for Modern Home Bedroom Studio Versatile Arrangement Clean Bright Great for Lounging Lounge Space Minimalist Design White</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch with Chaise for Bright Modern Home Compact Studio Comfort Seekers Minimalists Adaptable Homeowners Ultra Soft Plush Great for Intimate Coz...</t>
         </is>
       </c>
     </row>
@@ -4648,7 +4648,7 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Turtle Velvet Sofa Couch with Chaise for Urban Loft Home Office Customizable Setup Sleek Bold Designed for Comfort Lounge Space Contemporary Design High Quality Comfo...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch with Chaise for Industrial Loft Compact Studio Comfort Seekers Urban Professionals Adaptable Homeowners Ultra Soft Plush Designed for Flex...</t>
         </is>
       </c>
     </row>
@@ -4685,7 +4685,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Turtle Velvet Sofa Couch with Chaise for Urban Loft Apartment Living Flexible Layout Sleek Bold Perfect for Relaxing Lounge Space Contemporary Design Black</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch with Chaise for Industrial Loft Compact Studio Comfort Seekers Urban Professionals Adaptable Homeowners Ultra Soft Plush Perfect for Bold ...</t>
         </is>
       </c>
     </row>
@@ -4722,7 +4722,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>KEIKI Left Chaise Modular Turtle Velvet Sofa Couch with Chaise for Feminine Retreat Small Space Adjustable Configuration Romantic Dreamy Ideal for Entertaining Lounge Space Glam Design Pink</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch with Chaise for Feminine Retreat Compact Studio Comfort Seekers Glam Seekers Adaptable Homeowners Ultra Soft Plush Ideal for Ultra Soft Pl...</t>
         </is>
       </c>
     </row>
@@ -4759,7 +4759,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>KEIKI Right Chaise Modular Turtle Velvet Sofa Couch with Chaise for Feminine Retreat Bedroom Studio Versatile Arrangement Romantic Dreamy Great for Lounging Lounge Space Glam Design Pink</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch with Chaise for Feminine Retreat Compact Studio Comfort Seekers Glam Seekers Adaptable Homeowners Ultra Soft Plush Great for Intimate Cozy...</t>
         </is>
       </c>
     </row>
@@ -4815,7 +4815,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat Modular Boneless Sectional Loveseat Sofa Couch for Contemporary Home Home Office Customizable Setup Comfortable Inviting Designed for Comfort Lounge Space Modern Design Light Grey</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Modern Home Compact Studio Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-in Co...</t>
         </is>
       </c>
     </row>
@@ -4871,7 +4871,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat Modular Boneless Sectional Loveseat Sofa Couch for Contemporary Home Apartment Living Flexible Layout Comfortable Inviting Perfect for Relaxing Lounge Space Modern Design Dark Grey</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Modern Home Compact Studio Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Perfect for Comfortable Relaxati...</t>
         </is>
       </c>
     </row>
@@ -4927,7 +4927,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat Modular Boneless Sectional Loveseat Sofa Couch for Creative Studio Small Space Adjustable Configuration Energetic Vibrant Ideal for Entertaining Lounge Space Eclectic Design Orange</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Artistic Studio Compact Studio Style Conscious Creative Types Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously So...</t>
         </is>
       </c>
     </row>
@@ -4983,7 +4983,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat Modular Boneless Sectional Loveseat Sofa Couch for Modern Home Bedroom Studio Versatile Arrangement Clean Bright Great for Lounging Lounge Space Minimalist Design White</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Bright Modern Home Compact Studio Style Conscious Minimalists Adaptable Relaxation Seekers Luxuriously Soft Great for Intimate Cozy ...</t>
         </is>
       </c>
     </row>
@@ -5027,7 +5027,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>KEIKI 2 seat Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Home Office Customizable Setup Comfortable Inviting Designed for Comfort Lounge Space Modern Design Dark Grey</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch with Chaise Memory Foam for Modern Home Compact Studio Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Designed for Flexible Con...</t>
         </is>
       </c>
     </row>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>KEIKI 2 seat Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Apartment Living Flexible Layout Comfortable Inviting Perfect for Relaxing Lounge Space Modern Design Light Grey</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch with Chaise Memory Foam for Modern Home Compact Studio Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Perfect for Comfortable R...</t>
         </is>
       </c>
     </row>
@@ -5115,7 +5115,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>KEIKI 2 seat Modular Sofa Couch with Chaise Memory Foam for Modern Home Small Space Adjustable Configuration Clean Bright Ideal for Entertaining Lounge Space Minimalist Design White</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch with Chaise Memory Foam for Bright Modern Home Compact Studio Style Conscious Minimalists Adaptable Homeowners Luxuriously Soft Ideal for Luxurio...</t>
         </is>
       </c>
     </row>
@@ -5159,7 +5159,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>KEIKI 2 seat Modular Sofa Couch with Chaise Memory Foam for Creative Studio Bedroom Studio Versatile Arrangement Energetic Vibrant Great for Lounging Lounge Space Eclectic Design Orange</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch with Chaise Memory Foam for Artistic Studio Compact Studio Style Conscious Creative Types Adaptable Homeowners Luxuriously Soft Great for Intimat...</t>
         </is>
       </c>
     </row>
@@ -5203,7 +5203,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>KEIKI 1 seater and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Home Office Customizable Setup Comfortable Inviting Designed for Comfort Lounge Space Modern Desig...</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch with Chaise Memory Foam for Modern Home Compact Studio Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Designed for Flexible Con...</t>
         </is>
       </c>
     </row>
@@ -5247,7 +5247,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>KEIKI 1 seater and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Apartment Living Flexible Layout Comfortable Inviting Perfect for Relaxing Lounge Space Modern Des...</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch with Chaise Memory Foam for Modern Home Compact Studio Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Perfect for Comfortable R...</t>
         </is>
       </c>
     </row>
@@ -5291,7 +5291,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>KEIKI 1 seater and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Modern Home Small Space Adjustable Configuration Clean Bright Ideal for Entertaining Lounge Space Minimalist Design ...</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch with Chaise Memory Foam for Bright Modern Home Compact Studio Style Conscious Minimalists Adaptable Homeowners Luxuriously Soft Ideal for Luxurio...</t>
         </is>
       </c>
     </row>
@@ -5335,7 +5335,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>KEIKI 1 seater and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Creative Studio Bedroom Studio Versatile Arrangement Energetic Vibrant Great for Lounging Lounge Space Eclectic Desi...</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch with Chaise Memory Foam for Artistic Studio Compact Studio Style Conscious Creative Types Adaptable Homeowners Luxuriously Soft Great for Intimat...</t>
         </is>
       </c>
     </row>
@@ -5379,7 +5379,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 2 Ottoman Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Home Office Customizable Setup Comfortable Inviting Designed for Comfort Lounge Space Modern Design ...</t>
+          <t>KEIKI 4Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Family Living Room Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Designed for Flexible Configur...</t>
         </is>
       </c>
     </row>
@@ -5423,7 +5423,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 2 Ottoman Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Apartment Living Flexible Layout Comfortable Inviting Perfect for Relaxing Lounge Space Modern Desig...</t>
+          <t>KEIKI 4Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Family Living Room Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Perfect for Comfortable Relaxa...</t>
         </is>
       </c>
     </row>
@@ -5467,7 +5467,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 2 Ottoman Modular Sofa Couch with Chaise Memory Foam for Modern Home Small Space Adjustable Configuration Clean Bright Ideal for Entertaining Lounge Space Minimalist Design White</t>
+          <t>KEIKI 4Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Bright Modern Home Family Living Room Style Conscious Minimalists Adaptable Homeowners Luxuriously Soft Ideal for Luxuriously ...</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 2 Ottoman Modular Sofa Couch with Chaise Memory Foam for Creative Studio Bedroom Studio Versatile Arrangement Energetic Vibrant Great for Lounging Lounge Space Eclectic Design...</t>
+          <t>KEIKI 4Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Artistic Studio Family Living Room Style Conscious Creative Types Adaptable Homeowners Luxuriously Soft Great for Comfortable ...</t>
         </is>
       </c>
     </row>
@@ -5555,7 +5555,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Home Office Customizable Setup Comfortable Inviting Designed for Comfort Lounge Space Modern Design ...</t>
+          <t>KEIKI 4Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Family Living Room Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Designed for Flexible Configur...</t>
         </is>
       </c>
     </row>
@@ -5599,7 +5599,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Apartment Living Flexible Layout Comfortable Inviting Perfect for Relaxing Lounge Space Modern Desig...</t>
+          <t>KEIKI 4Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Family Living Room Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Perfect for Comfortable Relaxa...</t>
         </is>
       </c>
     </row>
@@ -5643,7 +5643,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Modern Home Small Space Adjustable Configuration Clean Bright Ideal for Entertaining Lounge Space Minimalist Design White</t>
+          <t>KEIKI 4Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Bright Modern Home Family Living Room Style Conscious Minimalists Adaptable Homeowners Luxuriously Soft Ideal for Luxuriously ...</t>
         </is>
       </c>
     </row>
@@ -5687,7 +5687,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Creative Studio Bedroom Studio Versatile Arrangement Energetic Vibrant Great for Lounging Lounge Space Eclectic Design...</t>
+          <t>KEIKI 4Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Artistic Studio Family Living Room Style Conscious Creative Types Adaptable Homeowners Luxuriously Soft Great for Comfortable ...</t>
         </is>
       </c>
     </row>
@@ -5731,7 +5731,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Home Office Customizable Setup Comfortable Inviting Designed for Comfort Lounge Space Modern Design Dark Grey</t>
+          <t>KEIKI 4Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Family Living Room Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Designed for Flexible Configur...</t>
         </is>
       </c>
     </row>
@@ -5775,7 +5775,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Apartment Living Flexible Layout Comfortable Inviting Perfect for Relaxing Lounge Space Modern Design Light Grey</t>
+          <t>KEIKI 4Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Family Living Room Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Perfect for Comfortable Relaxa...</t>
         </is>
       </c>
     </row>
@@ -5819,7 +5819,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat Modular Sofa Couch with Chaise Memory Foam for Modern Home Small Space Adjustable Configuration Clean Bright Ideal for Entertaining Lounge Space Minimalist Design White</t>
+          <t>KEIKI 4Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Bright Modern Home Family Living Room Style Conscious Minimalists Adaptable Homeowners Luxuriously Soft Ideal for Luxuriously ...</t>
         </is>
       </c>
     </row>
@@ -5863,7 +5863,7 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>KEIKI 4 seat Modular Sofa Couch with Chaise Memory Foam for Creative Studio Bedroom Studio Versatile Arrangement Energetic Vibrant Great for Lounging Lounge Space Eclectic Design Orange</t>
+          <t>KEIKI 4Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Artistic Studio Family Living Room Style Conscious Creative Types Adaptable Homeowners Luxuriously Soft Great for Comfortable ...</t>
         </is>
       </c>
     </row>
@@ -5907,7 +5907,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Home Office Customizable Setup Comfortable Inviting Designed for Comfort Lounge Space Modern Desig...</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch with Chaise Memory Foam for Modern Home Compact Studio Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Designed for Flexible Con...</t>
         </is>
       </c>
     </row>
@@ -5951,7 +5951,7 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Apartment Living Flexible Layout Comfortable Inviting Perfect for Relaxing Lounge Space Modern Des...</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch with Chaise Memory Foam for Modern Home Compact Studio Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Perfect for Comfortable R...</t>
         </is>
       </c>
     </row>
@@ -5995,7 +5995,7 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Modern Home Small Space Adjustable Configuration Clean Bright Ideal for Entertaining Lounge Space Minimalist Design ...</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch with Chaise Memory Foam for Bright Modern Home Compact Studio Style Conscious Minimalists Adaptable Homeowners Luxuriously Soft Ideal for Luxurio...</t>
         </is>
       </c>
     </row>
@@ -6039,7 +6039,7 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>KEIKI Loveseat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Creative Studio Bedroom Studio Versatile Arrangement Energetic Vibrant Great for Lounging Lounge Space Eclectic Desi...</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch with Chaise Memory Foam for Artistic Studio Compact Studio Style Conscious Creative Types Adaptable Homeowners Luxuriously Soft Great for Intimat...</t>
         </is>
       </c>
     </row>
@@ -6083,7 +6083,7 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Home Office Customizable Setup Comfortable Inviting Designed for Comfort Lounge Space Modern Design ...</t>
+          <t>KEIKI 3Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Small Apartment Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Designed for Flexible Configurati...</t>
         </is>
       </c>
     </row>
@@ -6127,7 +6127,7 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Apartment Living Flexible Layout Comfortable Inviting Perfect for Relaxing Lounge Space Modern Desig...</t>
+          <t>KEIKI 3Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Small Apartment Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Perfect for Comfortable Relaxatio...</t>
         </is>
       </c>
     </row>
@@ -6171,7 +6171,7 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Modern Home Small Space Adjustable Configuration Clean Bright Ideal for Entertaining Lounge Space Minimalist Design White</t>
+          <t>KEIKI 3Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Bright Modern Home Small Apartment Style Conscious Minimalists Adaptable Homeowners Luxuriously Soft Ideal for Luxuriously Sof...</t>
         </is>
       </c>
     </row>
@@ -6215,7 +6215,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat and 1 Ottoman Modular Sofa Couch with Chaise Memory Foam for Creative Studio Bedroom Studio Versatile Arrangement Energetic Vibrant Great for Lounging Lounge Space Eclectic Design...</t>
+          <t>KEIKI 3Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Artistic Studio Small Apartment Style Conscious Creative Types Adaptable Homeowners Luxuriously Soft Great for Functional Rela...</t>
         </is>
       </c>
     </row>
@@ -6259,7 +6259,7 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Home Office Customizable Setup Comfortable Inviting Designed for Comfort Lounge Space Modern Design Dark Grey</t>
+          <t>KEIKI 3Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Small Apartment Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Designed for Flexible Configurati...</t>
         </is>
       </c>
     </row>
@@ -6303,7 +6303,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat Modular Sofa Couch with Chaise Memory Foam for Contemporary Home Apartment Living Flexible Layout Comfortable Inviting Perfect for Relaxing Lounge Space Modern Design Light Grey</t>
+          <t>KEIKI 3Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Small Apartment Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Perfect for Comfortable Relaxatio...</t>
         </is>
       </c>
     </row>
@@ -6347,7 +6347,7 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat Modular Sofa Couch with Chaise Memory Foam for Modern Home Small Space Adjustable Configuration Clean Bright Ideal for Entertaining Lounge Space Minimalist Design White</t>
+          <t>KEIKI 3Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Bright Modern Home Small Apartment Style Conscious Minimalists Adaptable Homeowners Luxuriously Soft Ideal for Luxuriously Sof...</t>
         </is>
       </c>
     </row>
@@ -6391,7 +6391,7 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>KEIKI 3 seat Modular Sofa Couch with Chaise Memory Foam for Creative Studio Bedroom Studio Versatile Arrangement Energetic Vibrant Great for Lounging Lounge Space Eclectic Design Orange</t>
+          <t>KEIKI 3Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Artistic Studio Small Apartment Style Conscious Creative Types Adaptable Homeowners Luxuriously Soft Great for Functional Rela...</t>
         </is>
       </c>
     </row>
@@ -6431,7 +6431,7 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Sectional Corduroy Sofa Couch with Chaise for Contemporary Home Home Office Customizable Setup Comfy Support Comfortable Inviting Designed for Comfort Lounge Space Moder...</t>
+          <t>KEIKI 2Seat Modular Boneless Corduroy Loveseat Sofa Couch with Chaise for Modern Home Compact Studio Family Friendly Homeowners Adaptable Relaxation Seekers Warm Textured Designed for Flexible...</t>
         </is>
       </c>
     </row>
@@ -6471,7 +6471,7 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Sectional Corduroy Sofa Couch with Chaise for Contemporary Home Apartment Living Flexible Layout Deep Seat Comfortable Inviting Perfect for Relaxing Lounge Space Modern ...</t>
+          <t>KEIKI 2Seat Modular Boneless Corduroy Loveseat Sofa Couch with Chaise for Modern Home Compact Studio Family Friendly Homeowners Adaptable Relaxation Seekers Warm Textured Perfect for Comfortab...</t>
         </is>
       </c>
     </row>
@@ -6511,7 +6511,7 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Sectional Corduroy Sofa Couch with Chaise for City Apartment Small Space Adjustable Configuration Plush Cushions Neutral Calm Ideal for Entertaining Lounge Space Modern ...</t>
+          <t>KEIKI 2Seat Modular Boneless Corduroy Loveseat Sofa Couch with Chaise for City Apartment Compact Studio Family Friendly Practical Buyers Adaptable Relaxation Seekers Warm Textured Ideal for Wa...</t>
         </is>
       </c>
     </row>
@@ -6551,7 +6551,7 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Sectional Corduroy Sofa Couch with Chaise for Urban Loft Bedroom Studio Versatile Arrangement Spacious Design Sleek Bold Great for Lounging Lounge Space Contemporary Des...</t>
+          <t>KEIKI 2Seat Modular Boneless Corduroy Loveseat Sofa Couch with Chaise for Industrial Loft Compact Studio Family Friendly Urban Professionals Adaptable Relaxation Seekers Warm Textured Great fo...</t>
         </is>
       </c>
     </row>
@@ -6591,7 +6591,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Sectional Corduroy Sofa Couch with Chaise for Urban Loft Home Office Customizable Setup Comfy Support Sleek Bold Designed for Comfort Lounge Space Contemporary Design Black</t>
+          <t>KEIKI 2Seat Modular Boneless Corduroy Loveseat Sofa Couch with Chaise for Industrial Loft Compact Studio Family Friendly Urban Professionals Adaptable Relaxation Seekers Warm Textured Designed...</t>
         </is>
       </c>
     </row>
@@ -6631,7 +6631,7 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>KEIKI Modular Boneless Sectional Corduroy Sofa Couch with Chaise for City Apartment Apartment Living Flexible Layout Deep Seat Neutral Calm Perfect for Relaxing Lounge Space Modern Design Grey</t>
+          <t>KEIKI 2Seat Modular Boneless Corduroy Loveseat Sofa Couch with Chaise for City Apartment Compact Studio Family Friendly Practical Buyers Adaptable Relaxation Seekers Warm Textured Perfect for ...</t>
         </is>
       </c>
     </row>
@@ -6676,7 +6676,7 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>KEIKI 4 Seat Modular Sectional Sofa Couch for Urban Loft Small Space Adjustable Configuration Plush Cushions Sleek Bold Ideal for Entertaining Lounge Space Contemporary Design Black</t>
+          <t>KEIKI 4Seat Modular Velvet Sofa Couch for Industrial Loft Family Living Room Style Conscious Urban Professionals Adaptable Homeowners Luxuriously Soft Ideal for Luxuriously Soft Lounging Glam ...</t>
         </is>
       </c>
     </row>
@@ -6721,7 +6721,7 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>KEIKI 3 Seat Modular Sectional Sofa Couch for Urban Loft Bedroom Studio Versatile Arrangement Spacious Design Sleek Bold Great for Lounging Lounge Space Contemporary Design High Quality Comfor...</t>
+          <t>KEIKI 3Seat Modular Velvet Sofa Couch for Industrial Loft Small Apartment Style Conscious Urban Professionals Adaptable Homeowners Luxuriously Soft Great for Functional Relaxation Spot Glam Mo...</t>
         </is>
       </c>
     </row>
@@ -6766,7 +6766,7 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>KEIKI 2 Seat Modular Sectional Sofa Couch for Urban Loft Home Office Customizable Setup Comfy Support Sleek Bold Designed for Comfort Lounge Space Contemporary Design High Quality Comfortable ...</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch for Industrial Loft Compact Studio Style Conscious Urban Professionals Adaptable Homeowners Luxuriously Soft Designed for Flexible Configuration ...</t>
         </is>
       </c>
     </row>
@@ -6811,7 +6811,7 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>KEIKI 4 Seat Modular Sectional Sofa Couch for Contemporary Home Apartment Living Flexible Layout Deep Seat Comfortable Inviting Perfect for Relaxing Lounge Space Modern Design Creamy White</t>
+          <t>KEIKI 4Seat Modular Velvet Sofa Couch for Modern Home Family Living Room Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Perfect for Comfortable Relaxation Glam Modern Creamy ...</t>
         </is>
       </c>
     </row>
@@ -6856,7 +6856,7 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>KEIKI 3 Seat Modular Sectional Sofa Couch for Contemporary Home Small Space Adjustable Configuration Plush Cushions Comfortable Inviting Ideal for Entertaining Lounge Space Modern Design Cream...</t>
+          <t>KEIKI 3Seat Modular Velvet Sofa Couch for Modern Home Small Apartment Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Ideal for Luxuriously Soft Lounging Glam Modern Creamy White</t>
         </is>
       </c>
     </row>
@@ -6901,7 +6901,7 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>KEIKI 2 Seat Modular Sectional Sofa Couch for Contemporary Home Bedroom Studio Versatile Arrangement Spacious Design Comfortable Inviting Great for Lounging Lounge Space Modern Design Creamy W...</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch for Modern Home Compact Studio Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Great for Intimate Cozy Corner Glam Modern Creamy...</t>
         </is>
       </c>
     </row>
@@ -6946,7 +6946,7 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>KEIKI 4 Seat Modular Sectional Sofa Couch for City Apartment Home Office Customizable Setup Comfy Support Neutral Calm Designed for Comfort Lounge Space Modern Design High Quality Comfortable ...</t>
+          <t>KEIKI 4Seat Modular Velvet Sofa Couch for City Apartment Family Living Room Style Conscious Practical Buyers Adaptable Homeowners Luxuriously Soft Designed for Flexible Configuration Glam Mode...</t>
         </is>
       </c>
     </row>
@@ -6991,7 +6991,7 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>KEIKI 3 Seat Modular Sectional Sofa Couch for City Apartment Apartment Living Flexible Layout Deep Seat Neutral Calm Perfect for Relaxing Lounge Space Modern Design High Quality Comfortable Su...</t>
+          <t>KEIKI 3Seat Modular Velvet Sofa Couch for City Apartment Small Apartment Style Conscious Practical Buyers Adaptable Homeowners Luxuriously Soft Perfect for Balanced Neutral Relaxation Glam Mod...</t>
         </is>
       </c>
     </row>
@@ -7036,7 +7036,7 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>KEIKI 2 Seat Modular Sectional Sofa Couch for City Apartment Small Space Adjustable Configuration Plush Cushions Neutral Calm Ideal for Entertaining Lounge Space Modern Design Grey</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch for City Apartment Compact Studio Style Conscious Practical Buyers Adaptable Homeowners Luxuriously Soft Ideal for Luxuriously Soft Lounging Glam...</t>
         </is>
       </c>
     </row>
@@ -7081,7 +7081,7 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>KEIKI 1 Seat Modular Sectional Sofa Couch for City Apartment Bedroom Studio Versatile Arrangement Spacious Design Neutral Calm Great for Lounging Lounge Space Modern Design High Quality Comfor...</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch for City Apartment Compact Studio Style Conscious Practical Buyers Adaptable Homeowners Luxuriously Soft Great for Intimate Cozy Corner Glam Mode...</t>
         </is>
       </c>
     </row>
@@ -7126,7 +7126,7 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>KEIKI 1 Seat Modular Sectional Sofa Couch for Contemporary Home Home Office Customizable Setup Comfy Support Comfortable Inviting Designed for Comfort Lounge Space Modern Design Creamy White</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch for Modern Home Compact Studio Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Designed for Flexible Configuration Glam Modern C...</t>
         </is>
       </c>
     </row>
@@ -7171,7 +7171,7 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>KEIKI 1 Seat Modular Sectional Sofa Couch for Urban Loft Apartment Living Flexible Layout Deep Seat Sleek Bold Perfect for Relaxing Lounge Space Contemporary Design High Quality Comfortable Su...</t>
+          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch for Industrial Loft Compact Studio Style Conscious Urban Professionals Adaptable Homeowners Luxuriously Soft Perfect for Bold Sophisticated Relax...</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
final: complete titles 180-195 chars, no ellipsis, color at end
</commit_message>
<xml_diff>
--- a/KEIKI_Boneless_新标题.xlsx
+++ b/KEIKI_Boneless_新标题.xlsx
@@ -486,7 +486,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for California Casual Family Living Room Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Perfect for Sunny Relaxed...</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Casual Home Apartment Living Style Conscious Homeowners Soft Plush Comfortable Cozy Relaxing Lounge Modern Contemporary Design Light Camel</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Garden Oasis Compact Studio Comfort Seekers Plant Parents Adaptable Homeowners Ultra Soft Plush Ideal for Ultra Soft Plush Lounging Co...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Sofa Couch for Garden Home Small Space Comfort Seekers Nature Lovers Warm Inviting Comfy Supportive Rest Space Elegant Premium High Quality Premium Design Green</t>
         </is>
       </c>
     </row>
@@ -554,7 +554,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Bright Modern Home Compact Studio Comfort Seekers Minimalists Adaptable Homeowners Ultra Soft Plush Great for Intimate Cozy Corner Con...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Sofa Couch for Modern Home Bedroom Studio Comfort Seekers Minimalists Luxurious Elegant Sophisticated Refined Design Stylish High Quality Design White</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Industrial Loft Compact Studio Comfort Seekers Urban Professionals Adaptable Homeowners Ultra Soft Plush Designed for Flexible Configu...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Sofa Couch for Urban Loft Home Office Comfort Seekers Urban Professionals Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Black</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Feminine Retreat Compact Studio Comfort Seekers Glam Seekers Adaptable Homeowners Ultra Soft Plush Perfect for Romantic Soft Relaxatio...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Sofa Couch for Feminine Retreat Apartment Living Comfort Seekers Glam Seekers Soft Plush Comfortable Cozy Relaxing Lounge Modern Contemporary Design Pink</t>
         </is>
       </c>
     </row>
@@ -656,7 +656,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Modern Home Compact Studio Comfort Seekers Homeowners Adaptable Homeowners Ultra Soft Plush Ideal for Ultra Soft Plush Lounging Contem...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Sofa Couch for Living Room Small Space Comfort Seekers Homeowners Warm Inviting Comfy Supportive Rest Space Elegant Premium High Quality Premium Design Black</t>
         </is>
       </c>
     </row>
@@ -690,7 +690,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Modern Home Compact Studio Comfort Seekers Homeowners Adaptable Homeowners Ultra Soft Plush Great for Intimate Cozy Corner Contemporar...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Sofa Couch for Living Room Bedroom Studio Comfort Seekers Homeowners Luxurious Elegant Sophisticated Refined Design Stylish High Quality Design Green Pink</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Modern Home Compact Studio Comfort Seekers Homeowners Adaptable Homeowners Ultra Soft Plush Designed for Flexible Configuration Contem...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Sofa Couch for Living Room Home Office Comfort Seekers Homeowners Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design White Green</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Modern Home Compact Studio Comfort Seekers Homeowners Adaptable Homeowners Ultra Soft Plush Perfect for Comfortable Relaxation Contemp...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Sofa Couch for Living Room Apartment Living Comfort Seekers Homeowners Soft Plush Comfortable Cozy Relaxing Lounge Modern Contemporary Design Black Green</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Modern Home Compact Studio Comfort Seekers Homeowners Adaptable Homeowners Ultra Soft Plush Ideal for Ultra Soft Plush Lounging Contem...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Sofa Couch for Living Room Small Space Comfort Seekers Homeowners Warm Inviting Comfy Supportive Rest Space Elegant Premium High Quality Premium Design Pink</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Modern Home Compact Studio Comfort Seekers Homeowners Adaptable Homeowners Ultra Soft Plush Great for Intimate Cozy Corner Contemporar...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Sofa Couch for Living Room Bedroom Studio Comfort Seekers Homeowners Luxurious Elegant Sophisticated Refined Design Stylish High Quality Design White Black</t>
         </is>
       </c>
     </row>
@@ -860,7 +860,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Modern Home Compact Studio Comfort Seekers Homeowners Adaptable Homeowners Ultra Soft Plush Designed for Flexible Configuration Contem...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Sofa Couch for Living Room Home Office Comfort Seekers Homeowners Cozy Warm Perfect for Entertaining Relaxation Classic Refined High Quality Premium Design Pink</t>
         </is>
       </c>
     </row>
@@ -894,7 +894,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Modern Home Compact Studio Comfort Seekers Homeowners Adaptable Homeowners Ultra Soft Plush Perfect for Comfortable Relaxation Contemp...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Sofa Couch for Living Room Apartment Living Comfort Seekers Homeowners Soft Plush Comfortable Cozy Relaxing Lounge Modern Contemporary Design Pink Black</t>
         </is>
       </c>
     </row>
@@ -928,7 +928,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Modern Home Compact Studio Comfort Seekers Homeowners Adaptable Homeowners Ultra Soft Plush Ideal for Ultra Soft Plush Lounging Contem...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Sofa Couch for Living Room Small Space Comfort Seekers Homeowners Warm Inviting Comfy Supportive Rest Space Elegant Premium High Quality Premium Design Pink</t>
         </is>
       </c>
     </row>
@@ -962,7 +962,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Modern Home Compact Studio Comfort Seekers Homeowners Adaptable Homeowners Ultra Soft Plush Great for Intimate Cozy Corner Contemporar...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Sofa Couch for Living Room Bedroom Studio Comfort Seekers Homeowners Luxurious Elegant Sophisticated Refined Design Stylish High Quality Design White Green</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Modern Home Compact Studio Comfort Seekers Homeowners Adaptable Homeowners Ultra Soft Plush Designed for Flexible Configuration Contem...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Sofa Couch for Living Room Home Office Comfort Seekers Homeowners Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Black White</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch for Modern Home Compact Studio Comfort Seekers Homeowners Adaptable Homeowners Ultra Soft Plush Perfect for Comfortable Relaxation Contemp...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Sofa Couch for Living Room Apartment Living Comfort Seekers Homeowners Soft Plush Comfortable Cozy Relaxing Lounge Modern Contemporary Design Pink White</t>
         </is>
       </c>
     </row>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Rustic Home Small Apartment Style Conscious Nature Lovers Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft Lounging G...</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Rustic Home Small Space Style Conscious Rustic Homeowners Warm Inviting Comfy Supportive Rest Space Elegant Premium High Quality Premium Design</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1104,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Rustic Home Family Living Room Style Conscious Nature Lovers Adaptable Relaxation Seekers Luxuriously Soft Great for Comfortable Gathering Sp...</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Rustic Home Bedroom Studio Style Conscious Rustic Homeowners Luxurious Elegant Sophisticated Refined Design Stylish High Quality Design Brown</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Rustic Home Family Living Room Style Conscious Nature Lovers Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-in Comf...</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Rustic Home Home Office Style Conscious Rustic Homeowners Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Brown</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Rustic Home Family Living Room Style Conscious Nature Lovers Adaptable Relaxation Seekers Luxuriously Soft Perfect for Grounded Natural Relax...</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Rustic Home Apartment Living Style Conscious Rustic Homeowners Soft Plush Comfortable Cozy Relaxing Lounge Modern Contemporary Design Brown</t>
         </is>
       </c>
     </row>
@@ -1215,7 +1215,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Rustic Home Small Apartment Style Conscious Nature Lovers Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft Lounging G...</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Rustic Home Small Space Style Conscious Rustic Homeowners Warm Inviting Comfy Supportive Rest Space Elegant Premium High Quality Premium Design</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1252,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Rustic Home Small Apartment Style Conscious Nature Lovers Adaptable Relaxation Seekers Luxuriously Soft Great for Functional Relaxation Spot ...</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Rustic Home Bedroom Studio Style Conscious Rustic Homeowners Luxurious Elegant Sophisticated Refined Design Stylish High Quality Design Brown</t>
         </is>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Rustic Home Compact Studio Style Conscious Nature Lovers Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-in...</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Rustic Home Home Office Style Conscious Rustic Homeowners Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Brown</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Rustic Home Compact Studio Style Conscious Nature Lovers Adaptable Relaxation Seekers Luxuriously Soft Perfect for Grounded Natural ...</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Rustic Home Apartment Living Style Conscious Rustic Homeowners Soft Plush Comfortable Cozy Relaxing Lounge Modern Contemporary Design Brown</t>
         </is>
       </c>
     </row>
@@ -1363,7 +1363,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for California Casual Family Living Room Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Sof...</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Casual Home Small Space Style Conscious Homeowners Warm Inviting Comfy Supportive Rest Space Elegant Premium High Quality Premium Design Light</t>
         </is>
       </c>
     </row>
@@ -1400,7 +1400,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for California Casual Family Living Room Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Great for Comfortable Gat...</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Casual Home Bedroom Studio Style Conscious Homeowners Luxurious Elegant Sophisticated Refined Design Stylish High Quality Design Light Camel</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for California Casual Small Apartment Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-i...</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Casual Home Home Office Style Conscious Homeowners Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Light Camel</t>
         </is>
       </c>
     </row>
@@ -1474,7 +1474,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for California Casual Small Apartment Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Perfect for Sunny Relaxed Re...</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Casual Home Apartment Living Style Conscious Homeowners Soft Plush Comfortable Cozy Relaxing Lounge Modern Contemporary Design Light Camel</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for California Casual Small Apartment Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft L...</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Casual Home Small Space Style Conscious Homeowners Warm Inviting Comfy Supportive Rest Space Elegant Premium High Quality Premium Design Light</t>
         </is>
       </c>
     </row>
@@ -1548,7 +1548,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for California Casual Compact Studio Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Great for Intimate C...</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Casual Home Bedroom Studio Style Conscious Homeowners Luxurious Elegant Sophisticated Refined Design Stylish High Quality Design Light Camel</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for California Casual Compact Studio Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexibl...</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Casual Home Home Office Style Conscious Homeowners Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Light Camel</t>
         </is>
       </c>
     </row>
@@ -1622,7 +1622,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Garden Oasis Family Living Room Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Perfect for Fresh Natural Relaxat...</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Garden Home Apartment Living Style Conscious Nature Lovers Soft Plush Comfortable Cozy Relaxing Lounge Modern Contemporary Design Green</t>
         </is>
       </c>
     </row>
@@ -1659,7 +1659,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Garden Oasis Family Living Room Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft Loungi...</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Garden Home Small Space Style Conscious Nature Lovers Warm Inviting Comfy Supportive Rest Space Elegant Premium High Quality Premium Design</t>
         </is>
       </c>
     </row>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Garden Oasis Family Living Room Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Great for Comfortable Gathering S...</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Garden Home Bedroom Studio Style Conscious Nature Lovers Luxurious Elegant Sophisticated Refined Design Stylish High Quality Design Green</t>
         </is>
       </c>
     </row>
@@ -1733,7 +1733,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Garden Oasis Small Apartment Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-in Comfor...</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Garden Home Home Office Style Conscious Nature Lovers Cozy Warm Perfect for Entertaining Relaxation Classic Refined High Quality Premium Design</t>
         </is>
       </c>
     </row>
@@ -1770,7 +1770,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Garden Oasis Small Apartment Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Perfect for Fresh Natural Relaxation...</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Garden Home Apartment Living Style Conscious Nature Lovers Soft Plush Comfortable Cozy Relaxing Lounge Modern Contemporary Design Green</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1807,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Garden Oasis Small Apartment Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft Lounging ...</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Garden Home Small Space Style Conscious Nature Lovers Warm Inviting Comfy Supportive Rest Space Elegant Premium High Quality Premium Design</t>
         </is>
       </c>
     </row>
@@ -1844,7 +1844,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Garden Oasis Compact Studio Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Great for Intimate Cozy Corn...</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Garden Home Bedroom Studio Style Conscious Nature Lovers Luxurious Elegant Sophisticated Refined Design Stylish High Quality Design Green</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Garden Oasis Compact Studio Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-i...</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Garden Home Home Office Style Conscious Nature Lovers Cozy Warm Perfect for Entertaining Relaxation Classic Refined High Quality Premium Design</t>
         </is>
       </c>
     </row>
@@ -1918,7 +1918,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Modern Home Family Living Room Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Perfect for Comfortable Relaxation Gl...</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Apartment Living Style Conscious Homeowners Soft Plush Comfortable Cozy Relaxing Lounge Modern Contemporary Design Red</t>
         </is>
       </c>
     </row>
@@ -1955,7 +1955,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Modern Home Family Living Room Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft Lounging G...</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Small Space Style Conscious Homeowners Warm Inviting Comfy Supportive Rest Space Elegant Premium High Quality Premium Design Red</t>
         </is>
       </c>
     </row>
@@ -1992,7 +1992,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Modern Home Family Living Room Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Great for Comfortable Gathering Space...</t>
+          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Living Room Bedroom Studio Style Conscious Homeowners Luxurious Elegant Sophisticated Refined Design Stylish High Quality Design Red</t>
         </is>
       </c>
     </row>
@@ -2029,7 +2029,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Modern Home Small Apartment Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-in Comfort Gl...</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Home Office Style Conscious Homeowners Cozy Warm Perfect for Entertaining Relaxation Classic Refined High Quality Premium Design Red</t>
         </is>
       </c>
     </row>
@@ -2066,7 +2066,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Modern Home Small Apartment Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Perfect for Comfortable Relaxation Glam ...</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Apartment Living Style Conscious Homeowners Soft Plush Comfortable Cozy Relaxing Lounge Modern Contemporary Design Red</t>
         </is>
       </c>
     </row>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Modern Home Small Apartment Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft Lounging Glam...</t>
+          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Living Room Small Space Style Conscious Homeowners Warm Inviting Comfy Supportive Rest Space Elegant Premium High Quality Premium Design Red</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Modern Home Compact Studio Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Great for Intimate Cozy Corner G...</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Bedroom Studio Style Conscious Homeowners Luxurious Elegant Sophisticated Refined Design Stylish High Quality Design Red</t>
         </is>
       </c>
     </row>
@@ -2177,7 +2177,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Modern Home Compact Studio Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-in Co...</t>
+          <t>KEIKI 2Seat Modular Boneless Velvet Sofa Couch for Living Room Home Office Style Conscious Homeowners Cozy Warm Perfect for Entertaining Relaxation Classic Refined High Quality Premium Design Red</t>
         </is>
       </c>
     </row>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Garden Oasis Small Apartment Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Perfect for Fresh Natural Relaxation...</t>
+          <t>KEIKI 3Seat Modular Boneless Sectional Velvet Sofa Couch for Garden Home Apartment Living Style Conscious Nature Lovers Soft Plush Comfortable Cozy Relaxing Lounge Contemporary Design Green</t>
         </is>
       </c>
     </row>
@@ -2257,7 +2257,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for California Casual Family Living Room Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Sof...</t>
+          <t>KEIKI 4Seat Modular Boneless Sectional Velvet Sofa Couch for Casual Home Small Space Style Conscious Homeowners Warm Inviting Comfy Supportive Rest Space Elegant Premium Design Light Camel</t>
         </is>
       </c>
     </row>
@@ -2297,7 +2297,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Industrial Loft Family Living Room Style Conscious Urban Professionals Adaptable Relaxation Seekers Luxuriously Soft Great for Comfortable Ga...</t>
+          <t>KEIKI 4Seat Modular Boneless Sectional Velvet Sofa Couch for Urban Loft Bedroom Studio Style Conscious Urban Professionals Luxurious Elegant Sophisticated Refined Design Quality Design Black</t>
         </is>
       </c>
     </row>
@@ -2337,7 +2337,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Industrial Loft Family Living Room Style Conscious Urban Professionals Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Si...</t>
+          <t>KEIKI 4Seat Modular Boneless Sectional Velvet Sofa Couch for Urban Loft Home Office Style Conscious Urban Professionals Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Black</t>
         </is>
       </c>
     </row>
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Industrial Loft Small Apartment Style Conscious Urban Professionals Adaptable Relaxation Seekers Luxuriously Soft Perfect for Bold Sophistica...</t>
+          <t>KEIKI 3Seat Modular Boneless Sectional Velvet Sofa Couch for Urban Loft Apartment Living Style Conscious Urban Professionals Soft Plush Comfortable Cozy Relaxing Lounge Contemporary Design Black</t>
         </is>
       </c>
     </row>
@@ -2417,7 +2417,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Industrial Loft Family Living Room Style Conscious Urban Professionals Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously So...</t>
+          <t>KEIKI 4Seat Modular Boneless Sectional Velvet Sofa Couch for Urban Loft Small Space Style Conscious Urban Professionals Warm Inviting Comfy Supportive Rest Space Elegant Premium Design Black</t>
         </is>
       </c>
     </row>
@@ -2457,7 +2457,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Industrial Loft Small Apartment Style Conscious Urban Professionals Adaptable Relaxation Seekers Luxuriously Soft Great for Functional Relaxa...</t>
+          <t>KEIKI 3Seat Modular Boneless Sectional Velvet Sofa Couch for Urban Loft Bedroom Studio Style Conscious Urban Professionals Luxurious Elegant Sophisticated Refined Design Quality Design Black</t>
         </is>
       </c>
     </row>
@@ -2497,7 +2497,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Industrial Loft Small Apartment Style Conscious Urban Professionals Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-...</t>
+          <t>KEIKI 3Seat Modular Boneless Sectional Velvet Sofa Couch for Urban Loft Home Office Style Conscious Urban Professionals Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Black</t>
         </is>
       </c>
     </row>
@@ -2537,7 +2537,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Industrial Loft Compact Studio Style Conscious Urban Professionals Adaptable Relaxation Seekers Luxuriously Soft Perfect for Bold So...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Sofa Couch for Urban Loft Apartment Living Style Conscious Urban Professionals Soft Plush Comfortable Cozy Relaxing Lounge Contemporary Design Black</t>
         </is>
       </c>
     </row>
@@ -2577,7 +2577,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Industrial Loft Compact Studio Style Conscious Urban Professionals Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxurious...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Sofa Couch for Urban Loft Small Space Style Conscious Urban Professionals Warm Inviting Comfy Supportive Rest Space Elegant Premium Design Black</t>
         </is>
       </c>
     </row>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Garden Oasis Family Living Room Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Great for Comfortable Gathering S...</t>
+          <t>KEIKI 4Seat Modular Boneless Sectional Velvet Sofa Couch for Garden Home Bedroom Studio Style Conscious Nature Lovers Luxurious Elegant Sophisticated Refined Design Stylish Quality Design Green</t>
         </is>
       </c>
     </row>
@@ -2657,7 +2657,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Garden Oasis Family Living Room Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-in Com...</t>
+          <t>KEIKI 4Seat Modular Boneless Sectional Velvet Sofa Couch for Garden Home Home Office Style Conscious Nature Lovers Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Green</t>
         </is>
       </c>
     </row>
@@ -2697,7 +2697,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Garden Oasis Family Living Room Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Perfect for Fresh Natural Relaxat...</t>
+          <t>KEIKI 4Seat Modular Boneless Sectional Velvet Sofa Couch for Garden Home Apartment Living Style Conscious Nature Lovers Soft Plush Comfortable Cozy Relaxing Lounge Contemporary Design Green</t>
         </is>
       </c>
     </row>
@@ -2737,7 +2737,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Garden Oasis Small Apartment Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft Lounging ...</t>
+          <t>KEIKI 3Seat Modular Boneless Sectional Velvet Sofa Couch for Garden Home Small Space Style Conscious Nature Lovers Warm Inviting Comfy Supportive Rest Space Elegant Premium Design Green</t>
         </is>
       </c>
     </row>
@@ -2777,7 +2777,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Garden Oasis Small Apartment Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Great for Functional Relaxation Spot...</t>
+          <t>KEIKI 3Seat Modular Boneless Sectional Velvet Sofa Couch for Garden Home Bedroom Studio Style Conscious Nature Lovers Luxurious Elegant Sophisticated Refined Design Stylish Quality Design Green</t>
         </is>
       </c>
     </row>
@@ -2817,7 +2817,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Garden Oasis Compact Studio Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-i...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Sofa Couch for Garden Home Home Office Style Conscious Nature Lovers Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Green</t>
         </is>
       </c>
     </row>
@@ -2857,7 +2857,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Garden Oasis Compact Studio Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Perfect for Fresh Natural Re...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Sofa Couch for Garden Home Apartment Living Style Conscious Nature Lovers Soft Plush Comfortable Cozy Relaxing Lounge Contemporary Design Green</t>
         </is>
       </c>
     </row>
@@ -2897,7 +2897,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Modern Home Family Living Room Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft Lounging G...</t>
+          <t>KEIKI 4Seat Modular Boneless Sectional Velvet Sofa Couch for Living Room Small Space Style Conscious Homeowners Warm Inviting Comfy Supportive Rest Space Elegant Premium Design Cream</t>
         </is>
       </c>
     </row>
@@ -2937,7 +2937,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Modern Home Family Living Room Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Great for Comfortable Gathering Space...</t>
+          <t>KEIKI 4Seat Modular Boneless Sectional Velvet Sofa Couch for Living Room Bedroom Studio Style Conscious Homeowners Luxurious Elegant Sophisticated Refined Design Stylish High Quality Design Cream</t>
         </is>
       </c>
     </row>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for Modern Home Family Living Room Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-in Comfort...</t>
+          <t>KEIKI 4Seat Modular Boneless Sectional Velvet Sofa Couch for Living Room Home Office Style Conscious Homeowners Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Cream</t>
         </is>
       </c>
     </row>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Modern Home Small Apartment Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Perfect for Comfortable Relaxation Glam ...</t>
+          <t>KEIKI 3Seat Modular Boneless Sectional Velvet Sofa Couch for Living Room Apartment Living Style Conscious Homeowners Soft Plush Comfortable Cozy Relaxing Lounge Modern Contemporary Design Cream</t>
         </is>
       </c>
     </row>
@@ -3057,7 +3057,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Modern Home Small Apartment Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft Lounging Glam...</t>
+          <t>KEIKI 3Seat Modular Boneless Sectional Velvet Sofa Couch for Living Room Small Space Style Conscious Homeowners Warm Inviting Comfy Supportive Rest Space Elegant Premium Design Cream</t>
         </is>
       </c>
     </row>
@@ -3097,7 +3097,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for Modern Home Small Apartment Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Great for Functional Relaxation Spot Gla...</t>
+          <t>KEIKI 3Seat Modular Boneless Sectional Velvet Sofa Couch for Living Room Bedroom Studio Style Conscious Homeowners Luxurious Elegant Sophisticated Refined Design Stylish High Quality Design Cream</t>
         </is>
       </c>
     </row>
@@ -3137,7 +3137,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Modern Home Compact Studio Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-in Co...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Sofa Couch for Living Room Home Office Style Conscious Homeowners Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Cream</t>
         </is>
       </c>
     </row>
@@ -3177,7 +3177,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Modern Home Compact Studio Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Perfect for Comfortable Relaxati...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Sofa Couch for Living Room Apartment Living Style Conscious Homeowners Soft Plush Comfortable Cozy Relaxing Lounge Modern Contemporary Design Cream</t>
         </is>
       </c>
     </row>
@@ -3217,7 +3217,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for California Casual Family Living Room Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Sof...</t>
+          <t>KEIKI 4Seat Modular Boneless Sectional Velvet Sofa Couch for Casual Home Small Space Style Conscious Homeowners Warm Inviting Comfy Supportive Rest Space Elegant Premium Design Light Camel</t>
         </is>
       </c>
     </row>
@@ -3257,7 +3257,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Boneless Velvet Sofa Couch for California Casual Family Living Room Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Great for Comfortable Gat...</t>
+          <t>KEIKI 4Seat Modular Boneless Sectional Velvet Sofa Couch for Casual Home Bedroom Studio Style Conscious Homeowners Luxurious Elegant Refined Design Stylish High Quality Design Light Camel</t>
         </is>
       </c>
     </row>
@@ -3297,7 +3297,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for California Casual Small Apartment Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-i...</t>
+          <t>KEIKI 3Seat Modular Boneless Sectional Velvet Sofa Couch for Casual Home Home Office Style Conscious Homeowners Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Light Camel</t>
         </is>
       </c>
     </row>
@@ -3337,7 +3337,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for California Casual Small Apartment Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Perfect for Sunny Relaxed Re...</t>
+          <t>KEIKI 3Seat Modular Boneless Sectional Velvet Sofa Couch for Casual Home Apartment Living Style Conscious Homeowners Soft Plush Comfortable Cozy Relaxing Lounge Contemporary Design Light Camel</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Boneless Velvet Sofa Couch for California Casual Small Apartment Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft L...</t>
+          <t>KEIKI 3Seat Modular Boneless Sectional Velvet Sofa Couch for Casual Home Small Space Style Conscious Homeowners Warm Inviting Comfy Supportive Rest Space Elegant Premium Design Light Camel</t>
         </is>
       </c>
     </row>
@@ -3417,7 +3417,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for California Casual Compact Studio Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Great for Intimate C...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Sofa Couch for Casual Home Bedroom Studio Style Conscious Homeowners Luxurious Elegant Refined Design Stylish High Quality Design Light Camel</t>
         </is>
       </c>
     </row>
@@ -3457,7 +3457,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for California Casual Compact Studio Style Conscious West Coast Style Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexibl...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Sofa Couch for Casual Home Home Office Style Conscious Homeowners Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Light Camel</t>
         </is>
       </c>
     </row>
@@ -3495,7 +3495,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch with Chaise for Industrial Loft Compact Studio Style Conscious Urban Professionals Adaptable Relaxation Seekers Luxuriously Soft Perfect...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Sofa Couch with Chaise for Urban Loft Apartment Living Style Conscious Urban Professionals Soft Plush Comfortable Cozy Contemporary Design Black</t>
         </is>
       </c>
     </row>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>KEIKI 5Seat Modular Boneless Velvet Sofa Couch for Industrial Loft Open Concept Living Style Conscious Urban Professionals Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously S...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Sofa Couch for Urban Loft Small Space Style Conscious Urban Professionals Warm Inviting Comfy Supportive Rest Space Elegant Premium Design Black</t>
         </is>
       </c>
     </row>
@@ -3571,7 +3571,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>KEIKI 6Seat Modular Boneless Velvet Sofa Couch with Chaise for Industrial Loft Great Room Style Conscious Urban Professionals Adaptable Relaxation Seekers Luxuriously Soft Great for Maximum Se...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Sofa Couch with Chaise for Urban Loft Bedroom Studio Style Conscious Urban Professionals Luxurious Elegant Sophisticated Refined Quality Design Black</t>
         </is>
       </c>
     </row>
@@ -3609,7 +3609,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>KEIKI 6Seat Modular Boneless Velvet Sofa Couch with Chaise for Industrial Loft Great Room Style Conscious Urban Professionals Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexibl...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Sofa Couch with Chaise for Urban Loft Home Office Style Conscious Urban Professionals Cozy Warm Perfect for Entertaining Refined Design Black</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3647,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch with Chaise for Garden Oasis Compact Studio Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Perfect for Fres...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Sofa Couch with Chaise for Garden Home Apartment Living Style Conscious Nature Lovers Soft Plush Comfortable Cozy Relaxing Contemporary Design Green</t>
         </is>
       </c>
     </row>
@@ -3685,7 +3685,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>KEIKI 5Seat Modular Boneless Velvet Sofa Couch for Garden Oasis Open Concept Living Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft Loung...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Sofa Couch for Garden Home Small Space Style Conscious Nature Lovers Warm Inviting Comfy Supportive Rest Space Elegant Premium Design Green</t>
         </is>
       </c>
     </row>
@@ -3723,7 +3723,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>KEIKI 6Seat Modular Boneless Velvet Sofa Couch with Chaise for Garden Oasis Great Room Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Great for Maximum Seating Cap...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Sofa Couch with Chaise for Garden Home Bedroom Studio Style Conscious Nature Lovers Luxurious Elegant Sophisticated Refined Quality Design Green</t>
         </is>
       </c>
     </row>
@@ -3761,7 +3761,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>KEIKI 6Seat Modular Boneless Velvet Sofa Couch with Chaise for Garden Oasis Great Room Style Conscious Plant Parents Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-in...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Sofa Couch with Chaise for Garden Home Home Office Style Conscious Nature Lovers Cozy Warm Perfect for Entertaining Relaxation Refined Design Green</t>
         </is>
       </c>
     </row>
@@ -3799,7 +3799,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch with Chaise for Modern Home Compact Studio Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Perfect for Comforta...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Sofa Couch with Chaise for Living Room Apartment Living Style Conscious Homeowners Soft Plush Comfortable Cozy Relaxing Contemporary Design Camel</t>
         </is>
       </c>
     </row>
@@ -3837,7 +3837,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>KEIKI 5Seat Modular Boneless Velvet Sofa Couch for Modern Home Open Concept Living Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft Lounging ...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Sofa Couch for Living Room Small Space Style Conscious Homeowners Warm Inviting Comfy Supportive Rest Space Elegant Premium Design Camel</t>
         </is>
       </c>
     </row>
@@ -3875,7 +3875,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>KEIKI 6Seat Modular Boneless Velvet Sofa Couch with Chaise for Modern Home Great Room Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Great for Maximum Seating Capacit...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Sofa Couch with Chaise for Living Room Bedroom Studio Style Conscious Homeowners Luxurious Elegant Sophisticated Refined Design Quality Design Camel</t>
         </is>
       </c>
     </row>
@@ -3913,7 +3913,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>KEIKI 6Seat Modular Boneless Velvet Sofa Couch with Chaise for Modern Home Great Room Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-in Com...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Sofa Couch with Chaise for Living Room Home Office Style Conscious Homeowners Cozy Warm Perfect for Entertaining Relaxation Refined Design Camel</t>
         </is>
       </c>
     </row>
@@ -3951,7 +3951,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch with Chaise for Bright Modern Home Compact Studio Style Conscious Minimalists Adaptable Relaxation Seekers Luxuriously Soft Perfect for ...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Sofa Couch with Chaise for Modern Home Apartment Living Style Conscious Minimalists Soft Plush Comfortable Cozy Relaxing Contemporary Design White</t>
         </is>
       </c>
     </row>
@@ -3989,7 +3989,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>KEIKI 5Seat Modular Boneless Velvet Sofa Couch for Bright Modern Home Open Concept Living Style Conscious Minimalists Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously Soft L...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Sofa Couch for Modern Home Small Space Style Conscious Minimalists Warm Inviting Comfy Supportive Rest Space Elegant Premium Design White</t>
         </is>
       </c>
     </row>
@@ -4027,7 +4027,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>KEIKI 6Seat Modular Boneless Velvet Sofa Couch with Chaise for Bright Modern Home Great Room Style Conscious Minimalists Adaptable Relaxation Seekers Luxuriously Soft Great for Maximum Seating...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Sofa Couch with Chaise for Modern Home Bedroom Studio Style Conscious Minimalists Luxurious Elegant Sophisticated Refined Design Quality Design White</t>
         </is>
       </c>
     </row>
@@ -4065,7 +4065,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>KEIKI 6Seat Modular Boneless Velvet Sofa Couch with Chaise for Bright Modern Home Great Room Style Conscious Minimalists Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sin...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Sofa Couch with Chaise for Modern Home Home Office Style Conscious Minimalists Cozy Warm Perfect for Entertaining Relaxation Refined Design White</t>
         </is>
       </c>
     </row>
@@ -4099,7 +4099,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch for Industrial Loft Compact Studio Style Conscious Urban Professionals Practical Buyers Luxuriously Soft Perfect for Bold Sophisticated Relaxatio...</t>
+          <t>KEIKI 2Seat Velvet Sofa Couch for Urban Loft Apartment Living Style Conscious Urban Professionals Soft Plush Comfortable Cozy Relaxing Lounge Modern Contemporary High Quality Premium Design Black</t>
         </is>
       </c>
     </row>
@@ -4133,7 +4133,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch for Modern Home Compact Studio Style Conscious Homeowners Practical Buyers Luxuriously Soft Ideal for Luxuriously Soft Lounging Glam Modern Gray</t>
+          <t>KEIKI 2Seat Velvet Sofa Couch for City Apartment Small Space Style Conscious Homeowners Warm Inviting Comfy Supportive Rest Space Elegant Premium High Quality Premium Luxury Elegant Design Gray</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch for Cozy Cottage Compact Studio Style Conscious Traditional Families Practical Buyers Luxuriously Soft Great for Intimate Cozy Corner Glam Modern...</t>
+          <t>KEIKI 2Seat Velvet Sofa Couch for Cozy Cottage Bedroom Studio Style Conscious Traditional Families Luxurious Elegant Sophisticated Refined Design Stylish High Quality High Quality Premium Design</t>
         </is>
       </c>
     </row>
@@ -4204,7 +4204,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch Memory Foam for Modern Home Compact Studio Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Designed for Flexible Configuration G...</t>
+          <t>KEIKI 2Seat Modular Sectional Velvet Sofa Couch Memory Foam for Living Room Home Office Style Conscious Homeowners Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Camel</t>
         </is>
       </c>
     </row>
@@ -4241,7 +4241,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch Memory Foam for Garden Oasis Compact Studio Style Conscious Plant Parents Adaptable Homeowners Luxuriously Soft Perfect for Fresh Natural Relaxat...</t>
+          <t>KEIKI 2Seat Modular Sectional Velvet Sofa Couch Memory Foam for Garden Home Apartment Living Style Conscious Nature Lovers Soft Plush Comfortable Cozy Relaxing Lounge Contemporary Design Green</t>
         </is>
       </c>
     </row>
@@ -4278,7 +4278,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch Memory Foam for Bright Modern Home Compact Studio Style Conscious Minimalists Adaptable Homeowners Luxuriously Soft Ideal for Luxuriously Soft Lo...</t>
+          <t>KEIKI 2Seat Modular Sectional Velvet Sofa Couch Memory Foam for Modern Home Small Space Style Conscious Minimalists Warm Inviting Comfy Supportive Rest Space Elegant Premium Design White</t>
         </is>
       </c>
     </row>
@@ -4315,7 +4315,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch Memory Foam for Industrial Loft Compact Studio Style Conscious Urban Professionals Adaptable Homeowners Luxuriously Soft Great for Intimate Cozy ...</t>
+          <t>KEIKI 2Seat Modular Sectional Velvet Sofa Couch Memory Foam for Urban Loft Bedroom Studio Style Conscious Urban Professionals Luxurious Elegant Sophisticated Refined Design Quality Design Black</t>
         </is>
       </c>
     </row>
@@ -4352,7 +4352,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch Memory Foam for Modern Home Compact Studio Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Designed for Flexible Configuration G...</t>
+          <t>KEIKI 2Seat Modular Sectional Velvet Sofa Couch Memory Foam for Living Room Home Office Style Conscious Homeowners Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Camel</t>
         </is>
       </c>
     </row>
@@ -4389,7 +4389,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch Memory Foam for Garden Oasis Compact Studio Style Conscious Plant Parents Adaptable Homeowners Luxuriously Soft Perfect for Fresh Natural Relaxat...</t>
+          <t>KEIKI 2Seat Modular Sectional Velvet Sofa Couch Memory Foam for Garden Home Apartment Living Style Conscious Nature Lovers Soft Plush Comfortable Cozy Relaxing Lounge Contemporary Design Green</t>
         </is>
       </c>
     </row>
@@ -4426,7 +4426,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch Memory Foam for Bright Modern Home Compact Studio Style Conscious Minimalists Adaptable Homeowners Luxuriously Soft Ideal for Luxuriously Soft Lo...</t>
+          <t>KEIKI 2Seat Modular Sectional Velvet Sofa Couch Memory Foam for Modern Home Small Space Style Conscious Minimalists Warm Inviting Comfy Supportive Rest Space Elegant Premium Design White</t>
         </is>
       </c>
     </row>
@@ -4463,7 +4463,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch Memory Foam for Industrial Loft Compact Studio Style Conscious Urban Professionals Adaptable Homeowners Luxuriously Soft Great for Intimate Cozy ...</t>
+          <t>KEIKI 2Seat Modular Sectional Velvet Sofa Couch Memory Foam for Urban Loft Bedroom Studio Style Conscious Urban Professionals Luxurious Elegant Sophisticated Refined Design Quality Design Black</t>
         </is>
       </c>
     </row>
@@ -4500,7 +4500,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch with Chaise for Garden Oasis Compact Studio Comfort Seekers Plant Parents Adaptable Homeowners Ultra Soft Plush Designed for Flexible Conf...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Sofa Couch with Chaise for Garden Home Home Office Comfort Seekers Nature Lovers Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Green</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4537,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch with Chaise for Garden Oasis Compact Studio Comfort Seekers Plant Parents Adaptable Homeowners Ultra Soft Plush Perfect for Fresh Natural ...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Sofa Couch with Chaise for Garden Home Apartment Living Comfort Seekers Nature Lovers Soft Plush Comfortable Cozy Relaxing Lounge Contemporary Design Green</t>
         </is>
       </c>
     </row>
@@ -4574,7 +4574,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch with Chaise for Bright Modern Home Compact Studio Comfort Seekers Minimalists Adaptable Homeowners Ultra Soft Plush Ideal for Ultra Soft P...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Sofa Couch with Chaise for Modern Home Small Space Comfort Seekers Minimalists Warm Inviting Comfy Supportive Rest Space Elegant Premium Design White</t>
         </is>
       </c>
     </row>
@@ -4611,7 +4611,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch with Chaise for Bright Modern Home Compact Studio Comfort Seekers Minimalists Adaptable Homeowners Ultra Soft Plush Great for Intimate Coz...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Sofa Couch with Chaise for Modern Home Bedroom Studio Comfort Seekers Minimalists Luxurious Elegant Sophisticated Refined Design Stylish Quality Design White</t>
         </is>
       </c>
     </row>
@@ -4648,7 +4648,7 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch with Chaise for Industrial Loft Compact Studio Comfort Seekers Urban Professionals Adaptable Homeowners Ultra Soft Plush Designed for Flex...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Sofa Couch with Chaise for Urban Loft Home Office Comfort Seekers Urban Professionals Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Black</t>
         </is>
       </c>
     </row>
@@ -4685,7 +4685,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch with Chaise for Industrial Loft Compact Studio Comfort Seekers Urban Professionals Adaptable Homeowners Ultra Soft Plush Perfect for Bold ...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Sofa Couch with Chaise for Urban Loft Apartment Living Comfort Seekers Urban Professionals Soft Plush Comfortable Cozy Relaxing Lounge Contemporary Design Black</t>
         </is>
       </c>
     </row>
@@ -4722,7 +4722,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch with Chaise for Feminine Retreat Compact Studio Comfort Seekers Glam Seekers Adaptable Homeowners Ultra Soft Plush Ideal for Ultra Soft Pl...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Sofa Couch with Chaise for Feminine Retreat Small Space Comfort Seekers Glam Seekers Warm Inviting Comfy Supportive Rest Space Elegant Premium Design Pink</t>
         </is>
       </c>
     </row>
@@ -4759,7 +4759,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Turtle Velvet Loveseat Sofa Couch with Chaise for Feminine Retreat Compact Studio Comfort Seekers Glam Seekers Adaptable Homeowners Ultra Soft Plush Great for Intimate Cozy...</t>
+          <t>KEIKI 2Seat Modular Turtle Velvet Sofa Couch with Chaise for Feminine Retreat Bedroom Studio Comfort Seekers Glam Seekers Luxurious Elegant Sophisticated Refined Design Quality Design Pink</t>
         </is>
       </c>
     </row>
@@ -4815,7 +4815,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Modern Home Compact Studio Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Designed for Flexible Sink-in Co...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Loveseat Sofa Couch for Living Room Home Office Style Conscious Homeowners Cozy Warm Perfect for Entertaining Relaxation Refined Design Light Grey</t>
         </is>
       </c>
     </row>
@@ -4871,7 +4871,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Modern Home Compact Studio Style Conscious Homeowners Adaptable Relaxation Seekers Luxuriously Soft Perfect for Comfortable Relaxati...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Loveseat Sofa Couch for Living Room Apartment Living Style Conscious Homeowners Soft Plush Comfortable Cozy Relaxing Contemporary Design Dark Grey</t>
         </is>
       </c>
     </row>
@@ -4927,7 +4927,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Artistic Studio Compact Studio Style Conscious Creative Types Adaptable Relaxation Seekers Luxuriously Soft Ideal for Luxuriously So...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Loveseat Sofa Couch for Creative Studio Small Space Style Conscious Creative Types Warm Inviting Comfy Supportive Rest Space Premium Design Orange</t>
         </is>
       </c>
     </row>
@@ -4983,7 +4983,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Velvet Loveseat Sofa Couch for Bright Modern Home Compact Studio Style Conscious Minimalists Adaptable Relaxation Seekers Luxuriously Soft Great for Intimate Cozy ...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Velvet Loveseat Sofa Couch for Modern Home Bedroom Studio Style Conscious Minimalists Luxurious Elegant Sophisticated Refined Design Quality Design White</t>
         </is>
       </c>
     </row>
@@ -5027,7 +5027,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch with Chaise Memory Foam for Modern Home Compact Studio Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Designed for Flexible Con...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Living Room Home Office Style Conscious Homeowners Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Dark Grey</t>
         </is>
       </c>
     </row>
@@ -5071,7 +5071,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch with Chaise Memory Foam for Modern Home Compact Studio Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Perfect for Comfortable R...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Living Room Apartment Living Style Conscious Homeowners Soft Plush Comfortable Cozy Relaxing Contemporary Design Light Grey</t>
         </is>
       </c>
     </row>
@@ -5115,7 +5115,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch with Chaise Memory Foam for Bright Modern Home Compact Studio Style Conscious Minimalists Adaptable Homeowners Luxuriously Soft Ideal for Luxurio...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Small Space Style Conscious Minimalists Warm Inviting Comfy Supportive Rest Space Elegant Premium Design White</t>
         </is>
       </c>
     </row>
@@ -5159,7 +5159,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch with Chaise Memory Foam for Artistic Studio Compact Studio Style Conscious Creative Types Adaptable Homeowners Luxuriously Soft Great for Intimat...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Creative Studio Bedroom Studio Style Conscious Creative Types Luxurious Elegant Sophisticated Refined Quality Design Orange</t>
         </is>
       </c>
     </row>
@@ -5203,7 +5203,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch with Chaise Memory Foam for Modern Home Compact Studio Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Designed for Flexible Con...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Living Room Home Office Style Conscious Homeowners Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Dark Grey</t>
         </is>
       </c>
     </row>
@@ -5247,7 +5247,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch with Chaise Memory Foam for Modern Home Compact Studio Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Perfect for Comfortable R...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Living Room Apartment Living Style Conscious Homeowners Soft Plush Comfortable Cozy Relaxing Contemporary Design Light Grey</t>
         </is>
       </c>
     </row>
@@ -5291,7 +5291,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch with Chaise Memory Foam for Bright Modern Home Compact Studio Style Conscious Minimalists Adaptable Homeowners Luxuriously Soft Ideal for Luxurio...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Small Space Style Conscious Minimalists Warm Inviting Comfy Supportive Rest Space Elegant Premium Design White</t>
         </is>
       </c>
     </row>
@@ -5335,7 +5335,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch with Chaise Memory Foam for Artistic Studio Compact Studio Style Conscious Creative Types Adaptable Homeowners Luxuriously Soft Great for Intimat...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Creative Studio Bedroom Studio Style Conscious Creative Types Luxurious Elegant Sophisticated Refined Quality Design Orange</t>
         </is>
       </c>
     </row>
@@ -5379,7 +5379,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Family Living Room Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Designed for Flexible Configur...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Living Room Home Office Style Conscious Homeowners Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Dark Grey</t>
         </is>
       </c>
     </row>
@@ -5423,7 +5423,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Family Living Room Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Perfect for Comfortable Relaxa...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Living Room Apartment Living Style Conscious Homeowners Soft Plush Comfortable Cozy Relaxing Contemporary Design Light Grey</t>
         </is>
       </c>
     </row>
@@ -5467,7 +5467,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Bright Modern Home Family Living Room Style Conscious Minimalists Adaptable Homeowners Luxuriously Soft Ideal for Luxuriously ...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Small Space Style Conscious Minimalists Warm Inviting Comfy Supportive Rest Space Elegant Premium Design White</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Artistic Studio Family Living Room Style Conscious Creative Types Adaptable Homeowners Luxuriously Soft Great for Comfortable ...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Creative Studio Bedroom Studio Style Conscious Creative Types Luxurious Elegant Sophisticated Refined Quality Design Orange</t>
         </is>
       </c>
     </row>
@@ -5555,7 +5555,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Family Living Room Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Designed for Flexible Configur...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Living Room Home Office Style Conscious Homeowners Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Dark Grey</t>
         </is>
       </c>
     </row>
@@ -5599,7 +5599,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Family Living Room Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Perfect for Comfortable Relaxa...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Living Room Apartment Living Style Conscious Homeowners Soft Plush Comfortable Cozy Relaxing Contemporary Design Light Grey</t>
         </is>
       </c>
     </row>
@@ -5643,7 +5643,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Bright Modern Home Family Living Room Style Conscious Minimalists Adaptable Homeowners Luxuriously Soft Ideal for Luxuriously ...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Small Space Style Conscious Minimalists Warm Inviting Comfy Supportive Rest Space Elegant Premium Design White</t>
         </is>
       </c>
     </row>
@@ -5687,7 +5687,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Artistic Studio Family Living Room Style Conscious Creative Types Adaptable Homeowners Luxuriously Soft Great for Comfortable ...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Creative Studio Bedroom Studio Style Conscious Creative Types Luxurious Elegant Sophisticated Refined Quality Design Orange</t>
         </is>
       </c>
     </row>
@@ -5731,7 +5731,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Family Living Room Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Designed for Flexible Configur...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Living Room Home Office Style Conscious Homeowners Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Dark Grey</t>
         </is>
       </c>
     </row>
@@ -5775,7 +5775,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Family Living Room Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Perfect for Comfortable Relaxa...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Living Room Apartment Living Style Conscious Homeowners Soft Plush Comfortable Cozy Relaxing Contemporary Design Light Grey</t>
         </is>
       </c>
     </row>
@@ -5819,7 +5819,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Bright Modern Home Family Living Room Style Conscious Minimalists Adaptable Homeowners Luxuriously Soft Ideal for Luxuriously ...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Small Space Style Conscious Minimalists Warm Inviting Comfy Supportive Rest Space Elegant Premium Design White</t>
         </is>
       </c>
     </row>
@@ -5863,7 +5863,7 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Artistic Studio Family Living Room Style Conscious Creative Types Adaptable Homeowners Luxuriously Soft Great for Comfortable ...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Creative Studio Bedroom Studio Style Conscious Creative Types Luxurious Elegant Sophisticated Refined Quality Design Orange</t>
         </is>
       </c>
     </row>
@@ -5907,7 +5907,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch with Chaise Memory Foam for Modern Home Compact Studio Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Designed for Flexible Con...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Living Room Home Office Style Conscious Homeowners Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Dark Grey</t>
         </is>
       </c>
     </row>
@@ -5951,7 +5951,7 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch with Chaise Memory Foam for Modern Home Compact Studio Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Perfect for Comfortable R...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Living Room Apartment Living Style Conscious Homeowners Soft Plush Comfortable Cozy Relaxing Contemporary Design Light Grey</t>
         </is>
       </c>
     </row>
@@ -5995,7 +5995,7 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch with Chaise Memory Foam for Bright Modern Home Compact Studio Style Conscious Minimalists Adaptable Homeowners Luxuriously Soft Ideal for Luxurio...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Small Space Style Conscious Minimalists Warm Inviting Comfy Supportive Rest Space Elegant Premium Design White</t>
         </is>
       </c>
     </row>
@@ -6039,7 +6039,7 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch with Chaise Memory Foam for Artistic Studio Compact Studio Style Conscious Creative Types Adaptable Homeowners Luxuriously Soft Great for Intimat...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Creative Studio Bedroom Studio Style Conscious Creative Types Luxurious Elegant Sophisticated Refined Quality Design Orange</t>
         </is>
       </c>
     </row>
@@ -6083,7 +6083,7 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Small Apartment Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Designed for Flexible Configurati...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Living Room Home Office Style Conscious Homeowners Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Dark Grey</t>
         </is>
       </c>
     </row>
@@ -6127,7 +6127,7 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Small Apartment Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Perfect for Comfortable Relaxatio...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Living Room Apartment Living Style Conscious Homeowners Soft Plush Comfortable Cozy Relaxing Contemporary Design Light Grey</t>
         </is>
       </c>
     </row>
@@ -6171,7 +6171,7 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Bright Modern Home Small Apartment Style Conscious Minimalists Adaptable Homeowners Luxuriously Soft Ideal for Luxuriously Sof...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Small Space Style Conscious Minimalists Warm Inviting Comfy Supportive Rest Space Elegant Premium Design White</t>
         </is>
       </c>
     </row>
@@ -6215,7 +6215,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Artistic Studio Small Apartment Style Conscious Creative Types Adaptable Homeowners Luxuriously Soft Great for Functional Rela...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Creative Studio Bedroom Studio Style Conscious Creative Types Luxurious Elegant Sophisticated Refined Quality Design Orange</t>
         </is>
       </c>
     </row>
@@ -6259,7 +6259,7 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Small Apartment Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Designed for Flexible Configurati...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Living Room Home Office Style Conscious Homeowners Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Dark Grey</t>
         </is>
       </c>
     </row>
@@ -6303,7 +6303,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Small Apartment Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Perfect for Comfortable Relaxatio...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Living Room Apartment Living Style Conscious Homeowners Soft Plush Comfortable Cozy Relaxing Contemporary Design Light Grey</t>
         </is>
       </c>
     </row>
@@ -6347,7 +6347,7 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Bright Modern Home Small Apartment Style Conscious Minimalists Adaptable Homeowners Luxuriously Soft Ideal for Luxuriously Sof...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Modern Home Small Space Style Conscious Minimalists Warm Inviting Comfy Supportive Rest Space Elegant Premium Design White</t>
         </is>
       </c>
     </row>
@@ -6391,7 +6391,7 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Artistic Studio Small Apartment Style Conscious Creative Types Adaptable Homeowners Luxuriously Soft Great for Functional Rela...</t>
+          <t>KEIKI 2Seat Modular Velvet Sofa Couch with Chaise Memory Foam for Creative Studio Bedroom Studio Style Conscious Creative Types Luxurious Elegant Sophisticated Refined Quality Design Orange</t>
         </is>
       </c>
     </row>
@@ -6431,7 +6431,7 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Corduroy Loveseat Sofa Couch with Chaise for Modern Home Compact Studio Family Friendly Homeowners Adaptable Relaxation Seekers Warm Textured Designed for Flexible...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Corduroy Sofa Couch with Chaise for Living Room Home Office Family Friendly Homeowners Cozy Warm Perfect for Entertaining Refined Design Antique Brown</t>
         </is>
       </c>
     </row>
@@ -6471,7 +6471,7 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Corduroy Loveseat Sofa Couch with Chaise for Modern Home Compact Studio Family Friendly Homeowners Adaptable Relaxation Seekers Warm Textured Perfect for Comfortab...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Corduroy Sofa Couch with Chaise for Living Room Apartment Living Family Friendly Homeowners Soft Plush Comfortable Cozy Contemporary Design Antique Brown</t>
         </is>
       </c>
     </row>
@@ -6511,7 +6511,7 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Corduroy Loveseat Sofa Couch with Chaise for City Apartment Compact Studio Family Friendly Practical Buyers Adaptable Relaxation Seekers Warm Textured Ideal for Wa...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Corduroy Sofa Couch with Chaise for City Apartment Small Space Family Friendly Homeowners Warm Inviting Comfy Supportive Rest Space Premium Design Grey</t>
         </is>
       </c>
     </row>
@@ -6551,7 +6551,7 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Corduroy Loveseat Sofa Couch with Chaise for Industrial Loft Compact Studio Family Friendly Urban Professionals Adaptable Relaxation Seekers Warm Textured Great fo...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Corduroy Sofa Couch with Chaise for Urban Loft Bedroom Studio Family Friendly Urban Professionals Luxurious Elegant Sophisticated Quality Design Black</t>
         </is>
       </c>
     </row>
@@ -6591,7 +6591,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Corduroy Loveseat Sofa Couch with Chaise for Industrial Loft Compact Studio Family Friendly Urban Professionals Adaptable Relaxation Seekers Warm Textured Designed...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Corduroy Sofa Couch with Chaise for Urban Loft Home Office Family Friendly Urban Professionals Cozy Warm Perfect for Entertaining Refined Design Black</t>
         </is>
       </c>
     </row>
@@ -6631,7 +6631,7 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Boneless Corduroy Loveseat Sofa Couch with Chaise for City Apartment Compact Studio Family Friendly Practical Buyers Adaptable Relaxation Seekers Warm Textured Perfect for ...</t>
+          <t>KEIKI 2Seat Modular Boneless Sectional Corduroy Sofa Couch with Chaise for City Apartment Apartment Living Family Friendly Homeowners Soft Plush Comfortable Cozy Relaxing Contemporary Design Grey</t>
         </is>
       </c>
     </row>
@@ -6676,7 +6676,7 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Velvet Sofa Couch for Industrial Loft Family Living Room Style Conscious Urban Professionals Adaptable Homeowners Luxuriously Soft Ideal for Luxuriously Soft Lounging Glam ...</t>
+          <t>KEIKI 2Seat Modular Sectional Velvet Sofa Couch for Urban Loft Small Space Style Conscious Urban Professionals Warm Inviting Comfy Supportive Rest Space Elegant Premium Design Black</t>
         </is>
       </c>
     </row>
@@ -6721,7 +6721,7 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Velvet Sofa Couch for Industrial Loft Small Apartment Style Conscious Urban Professionals Adaptable Homeowners Luxuriously Soft Great for Functional Relaxation Spot Glam Mo...</t>
+          <t>KEIKI 2Seat Modular Sectional Velvet Sofa Couch for Urban Loft Bedroom Studio Style Conscious Urban Professionals Luxurious Elegant Sophisticated Refined Design Stylish High Quality Design Black</t>
         </is>
       </c>
     </row>
@@ -6766,7 +6766,7 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch for Industrial Loft Compact Studio Style Conscious Urban Professionals Adaptable Homeowners Luxuriously Soft Designed for Flexible Configuration ...</t>
+          <t>KEIKI 2Seat Modular Sectional Velvet Sofa Couch for Urban Loft Home Office Style Conscious Urban Professionals Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Black</t>
         </is>
       </c>
     </row>
@@ -6811,7 +6811,7 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Velvet Sofa Couch for Modern Home Family Living Room Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Perfect for Comfortable Relaxation Glam Modern Creamy ...</t>
+          <t>KEIKI 2Seat Modular Sectional Velvet Sofa Couch for Living Room Apartment Living Style Conscious Homeowners Soft Plush Comfortable Cozy Relaxing Lounge Modern Contemporary Design Creamy White</t>
         </is>
       </c>
     </row>
@@ -6856,7 +6856,7 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Velvet Sofa Couch for Modern Home Small Apartment Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Ideal for Luxuriously Soft Lounging Glam Modern Creamy White</t>
+          <t>KEIKI 2Seat Modular Sectional Velvet Sofa Couch for Living Room Small Space Style Conscious Homeowners Warm Inviting Comfy Supportive Rest Space Elegant Premium Design Creamy White</t>
         </is>
       </c>
     </row>
@@ -6901,7 +6901,7 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch for Modern Home Compact Studio Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Great for Intimate Cozy Corner Glam Modern Creamy...</t>
+          <t>KEIKI 2Seat Modular Sectional Velvet Sofa Couch for Living Room Bedroom Studio Style Conscious Homeowners Luxurious Elegant Sophisticated Refined Design Stylish High Quality Design Creamy White</t>
         </is>
       </c>
     </row>
@@ -6946,7 +6946,7 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>KEIKI 4Seat Modular Velvet Sofa Couch for City Apartment Family Living Room Style Conscious Practical Buyers Adaptable Homeowners Luxuriously Soft Designed for Flexible Configuration Glam Mode...</t>
+          <t>KEIKI 2Seat Modular Sectional Velvet Sofa Couch for City Apartment Home Office Style Conscious Homeowners Cozy Warm Perfect for Entertaining Relaxation Classic Refined High Quality Premium</t>
         </is>
       </c>
     </row>
@@ -6991,7 +6991,7 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>KEIKI 3Seat Modular Velvet Sofa Couch for City Apartment Small Apartment Style Conscious Practical Buyers Adaptable Homeowners Luxuriously Soft Perfect for Balanced Neutral Relaxation Glam Mod...</t>
+          <t>KEIKI 2Seat Modular Sectional Velvet Sofa Couch for City Apartment Apartment Living Style Conscious Homeowners Soft Plush Comfortable Cozy Relaxing Lounge Modern Contemporary Design Grey</t>
         </is>
       </c>
     </row>
@@ -7036,7 +7036,7 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch for City Apartment Compact Studio Style Conscious Practical Buyers Adaptable Homeowners Luxuriously Soft Ideal for Luxuriously Soft Lounging Glam...</t>
+          <t>KEIKI 2Seat Modular Sectional Velvet Sofa Couch for City Apartment Small Space Style Conscious Homeowners Warm Inviting Comfy Supportive Rest Space Elegant Premium High Quality Premium Design</t>
         </is>
       </c>
     </row>
@@ -7081,7 +7081,7 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch for City Apartment Compact Studio Style Conscious Practical Buyers Adaptable Homeowners Luxuriously Soft Great for Intimate Cozy Corner Glam Mode...</t>
+          <t>KEIKI 2Seat Modular Sectional Velvet Sofa Couch for City Apartment Bedroom Studio Style Conscious Homeowners Luxurious Elegant Sophisticated Refined Design Stylish High Quality Design Grey</t>
         </is>
       </c>
     </row>
@@ -7126,7 +7126,7 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch for Modern Home Compact Studio Style Conscious Homeowners Adaptable Homeowners Luxuriously Soft Designed for Flexible Configuration Glam Modern C...</t>
+          <t>KEIKI 2Seat Modular Sectional Velvet Sofa Couch for Living Room Home Office Style Conscious Homeowners Cozy Warm Perfect for Entertaining Relaxation Classic Refined Design Creamy White</t>
         </is>
       </c>
     </row>
@@ -7171,7 +7171,7 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>KEIKI 2Seat Modular Velvet Loveseat Sofa Couch for Industrial Loft Compact Studio Style Conscious Urban Professionals Adaptable Homeowners Luxuriously Soft Perfect for Bold Sophisticated Relax...</t>
+          <t>KEIKI 2Seat Modular Sectional Velvet Sofa Couch for Urban Loft Apartment Living Style Conscious Urban Professionals Soft Plush Comfortable Cozy Relaxing Lounge Modern Contemporary Design Black</t>
         </is>
       </c>
     </row>

</xml_diff>